<commit_message>
Name every reorganization energy lambda_<surface>_<geometry>
The photocatalyst and quencher tables named their lambdas in two schemes whose
letters read in opposite orders (lambda_S0_to_T1 was the triplet surface,
lambda_S_T the singlet one). Both now use one: lambda_S0_T1 is E_S0 at the T1
geometry minus E_S0 at its own, lambda_T1_S0 the triplet surface, and likewise
lambda_S0_Dplus, lambda_Dplus_S0, lambda_S0_Dminus, lambda_Dminus_S0.

Renamed in the extraction scripts, both DFT tables, the three calculated
workbooks and their column keys, and the benchmark's pair columns. Every value
is unchanged; the benchmark results are regenerated from the current tables.

Drop the photocatalyst manifest.csv and the code that wrote it.
</commit_message>
<xml_diff>
--- a/data/computational_data_processed/photocatalyst_properties_calc.xlsx
+++ b/data/computational_data_processed/photocatalyst_properties_calc.xlsx
@@ -492,8 +492,8 @@
     <col width="2" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="2" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="7" max="7"/>
+    <col width="27" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
     <col width="31" customWidth="1" min="11" max="11"/>
@@ -560,32 +560,32 @@
       </c>
       <c r="G2" s="10" t="inlineStr">
         <is>
-          <t>lambda_S0_to_T1 / kcal mol-1</t>
+          <t>lambda_S0_T1 / kcal mol-1</t>
         </is>
       </c>
       <c r="H2" s="10" t="inlineStr">
         <is>
-          <t>lambda_T1_to_S0 / kcal mol-1</t>
+          <t>lambda_T1_S0 / kcal mol-1</t>
         </is>
       </c>
       <c r="I2" s="10" t="inlineStr">
         <is>
-          <t>lambda_S0_to_ox / kcal mol-1</t>
+          <t>lambda_S0_Dplus / kcal mol-1</t>
         </is>
       </c>
       <c r="J2" s="10" t="inlineStr">
         <is>
-          <t>lambda_ox_to_S0 / kcal mol-1</t>
+          <t>lambda_Dplus_S0 / kcal mol-1</t>
         </is>
       </c>
       <c r="K2" s="10" t="inlineStr">
         <is>
-          <t>lambda_S0_to_red / kcal mol-1</t>
+          <t>lambda_S0_Dminus / kcal mol-1</t>
         </is>
       </c>
       <c r="L2" s="10" t="inlineStr">
         <is>
-          <t>lambda_red_to_S0 / kcal mol-1</t>
+          <t>lambda_Dminus_S0 / kcal mol-1</t>
         </is>
       </c>
       <c r="N2" s="11" t="inlineStr">
@@ -625,22 +625,22 @@
         <v>65.70102948398493</v>
       </c>
       <c r="G3" s="12" t="n">
+        <v>10.27558245293145</v>
+      </c>
+      <c r="H3" s="12" t="n">
         <v>8.251113847131</v>
       </c>
-      <c r="H3" s="12" t="n">
-        <v>10.27558245293145</v>
-      </c>
       <c r="I3" s="12" t="n">
+        <v>2.719382899684559</v>
+      </c>
+      <c r="J3" s="12" t="n">
         <v>2.579593446458603</v>
       </c>
-      <c r="J3" s="12" t="n">
-        <v>2.719382899684559</v>
-      </c>
       <c r="K3" s="12" t="n">
+        <v>6.066670200749988</v>
+      </c>
+      <c r="L3" s="12" t="n">
         <v>6.115006106872588</v>
-      </c>
-      <c r="L3" s="12" t="n">
-        <v>6.066670200749988</v>
       </c>
       <c r="N3" s="12" t="n">
         <v>78.88260727943963</v>
@@ -671,22 +671,22 @@
         <v>64.17789905286688</v>
       </c>
       <c r="G4" s="12" t="n">
+        <v>11.35464264717792</v>
+      </c>
+      <c r="H4" s="12" t="n">
         <v>9.349048755462885</v>
       </c>
-      <c r="H4" s="12" t="n">
-        <v>11.35464264717792</v>
-      </c>
       <c r="I4" s="12" t="n">
+        <v>2.931068175715682</v>
+      </c>
+      <c r="J4" s="12" t="n">
         <v>2.801124465718414</v>
       </c>
-      <c r="J4" s="12" t="n">
-        <v>2.931068175715682</v>
-      </c>
       <c r="K4" s="12" t="n">
+        <v>6.016309364188979</v>
+      </c>
+      <c r="L4" s="12" t="n">
         <v>8.595742985025044</v>
-      </c>
-      <c r="L4" s="12" t="n">
-        <v>6.016309364188979</v>
       </c>
       <c r="N4" s="12" t="n">
         <v>68.86705232991353</v>
@@ -717,22 +717,22 @@
         <v>60.37977711302834</v>
       </c>
       <c r="G5" s="12" t="n">
+        <v>11.81912009778503</v>
+      </c>
+      <c r="H5" s="12" t="n">
         <v>8.481128584206719</v>
       </c>
-      <c r="H5" s="12" t="n">
-        <v>11.81912009778503</v>
-      </c>
       <c r="I5" s="12" t="n">
+        <v>2.863742889509551</v>
+      </c>
+      <c r="J5" s="12" t="n">
         <v>1.822697743843328</v>
       </c>
-      <c r="J5" s="12" t="n">
-        <v>2.863742889509551</v>
-      </c>
       <c r="K5" s="12" t="n">
+        <v>4.599361755362191</v>
+      </c>
+      <c r="L5" s="12" t="n">
         <v>4.320535408871186</v>
-      </c>
-      <c r="L5" s="12" t="n">
-        <v>4.599361755362191</v>
       </c>
       <c r="N5" s="12" t="n">
         <v>61.94475067884279</v>
@@ -763,22 +763,22 @@
         <v>65.61781249707244</v>
       </c>
       <c r="G6" s="12" t="n">
+        <v>13.32092869504703</v>
+      </c>
+      <c r="H6" s="12" t="n">
         <v>8.885442302106865</v>
       </c>
-      <c r="H6" s="12" t="n">
-        <v>13.32092869504703</v>
-      </c>
       <c r="I6" s="12" t="n">
+        <v>1.476863333423498</v>
+      </c>
+      <c r="J6" s="12" t="n">
         <v>1.345780894116102</v>
       </c>
-      <c r="J6" s="12" t="n">
-        <v>1.476863333423498</v>
-      </c>
       <c r="K6" s="12" t="n">
+        <v>4.459122623498202</v>
+      </c>
+      <c r="L6" s="12" t="n">
         <v>4.190890959573786</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>4.459122623498202</v>
       </c>
       <c r="N6" s="12" t="n">
         <v>65.90427545472191</v>
@@ -809,22 +809,22 @@
         <v>45.75110330770049</v>
       </c>
       <c r="G7" s="12" t="n">
+        <v>7.329913250875807</v>
+      </c>
+      <c r="H7" s="12" t="n">
         <v>7.640425739288484</v>
       </c>
-      <c r="H7" s="12" t="n">
-        <v>7.329913250875807</v>
-      </c>
       <c r="I7" s="12" t="n">
+        <v>0.9700102287098725</v>
+      </c>
+      <c r="J7" s="12" t="n">
         <v>1.217932027280818</v>
       </c>
-      <c r="J7" s="12" t="n">
-        <v>0.9700102287098725</v>
-      </c>
       <c r="K7" s="12" t="n">
+        <v>5.82943839833115</v>
+      </c>
+      <c r="L7" s="12" t="n">
         <v>5.784461481258163</v>
-      </c>
-      <c r="L7" s="12" t="n">
-        <v>5.82943839833115</v>
       </c>
       <c r="N7" s="12" t="n">
         <v>78.86315697989353</v>
@@ -855,22 +855,22 @@
         <v>46.98057297731619</v>
       </c>
       <c r="G8" s="12" t="n">
+        <v>7.029133876579498</v>
+      </c>
+      <c r="H8" s="12" t="n">
         <v>7.083066470863391</v>
       </c>
-      <c r="H8" s="12" t="n">
-        <v>7.029133876579498</v>
-      </c>
       <c r="I8" s="12" t="n">
+        <v>0.9323012928471144</v>
+      </c>
+      <c r="J8" s="12" t="n">
         <v>1.031472113423926</v>
       </c>
-      <c r="J8" s="12" t="n">
-        <v>0.9323012928471144</v>
-      </c>
       <c r="K8" s="12" t="n">
+        <v>5.30896556283638</v>
+      </c>
+      <c r="L8" s="12" t="n">
         <v>5.340455803599435</v>
-      </c>
-      <c r="L8" s="12" t="n">
-        <v>5.30896556283638</v>
       </c>
       <c r="N8" s="12" t="n">
         <v>101.2939351971944</v>
@@ -901,22 +901,22 @@
         <v>66.14982962376409</v>
       </c>
       <c r="G9" s="12" t="n">
+        <v>13.76995402293388</v>
+      </c>
+      <c r="H9" s="12" t="n">
         <v>9.099952497328978</v>
       </c>
-      <c r="H9" s="12" t="n">
-        <v>13.76995402293388</v>
-      </c>
       <c r="I9" s="12" t="n">
+        <v>1.456602285984715</v>
+      </c>
+      <c r="J9" s="12" t="n">
         <v>1.395618918193773</v>
       </c>
-      <c r="J9" s="12" t="n">
-        <v>1.456602285984715</v>
-      </c>
       <c r="K9" s="12" t="n">
+        <v>4.253755373423006</v>
+      </c>
+      <c r="L9" s="12" t="n">
         <v>4.065051497415832</v>
-      </c>
-      <c r="L9" s="12" t="n">
-        <v>4.253755373423006</v>
       </c>
       <c r="N9" s="12" t="n">
         <v>64.16731074439966</v>
@@ -947,22 +947,22 @@
         <v>55.94263348569274</v>
       </c>
       <c r="G10" s="12" t="n">
+        <v>8.626784273100959</v>
+      </c>
+      <c r="H10" s="12" t="n">
         <v>9.484973307772082</v>
       </c>
-      <c r="H10" s="12" t="n">
-        <v>8.626784273100959</v>
-      </c>
       <c r="I10" s="12" t="n">
+        <v>2.683798476231521</v>
+      </c>
+      <c r="J10" s="12" t="n">
         <v>2.657746064229599</v>
       </c>
-      <c r="J10" s="12" t="n">
-        <v>2.683798476231521</v>
-      </c>
       <c r="K10" s="12" t="n">
+        <v>6.561976450410632</v>
+      </c>
+      <c r="L10" s="12" t="n">
         <v>7.542257737116455</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>6.561976450410632</v>
       </c>
       <c r="N10" s="12" t="n">
         <v>93.31472892397659</v>
@@ -993,22 +993,22 @@
         <v>67.13698165978478</v>
       </c>
       <c r="G11" s="12" t="n">
+        <v>12.87573434699418</v>
+      </c>
+      <c r="H11" s="12" t="n">
         <v>11.71255566140693</v>
       </c>
-      <c r="H11" s="12" t="n">
-        <v>12.87573434699418</v>
-      </c>
       <c r="I11" s="12" t="n">
+        <v>2.545378533930856</v>
+      </c>
+      <c r="J11" s="12" t="n">
         <v>2.435375699634205</v>
       </c>
-      <c r="J11" s="12" t="n">
-        <v>2.545378533930856</v>
-      </c>
       <c r="K11" s="12" t="n">
+        <v>6.015743179564084</v>
+      </c>
+      <c r="L11" s="12" t="n">
         <v>6.049062549482249</v>
-      </c>
-      <c r="L11" s="12" t="n">
-        <v>6.015743179564084</v>
       </c>
       <c r="N11" s="12" t="n">
         <v>74.28718158644462</v>
@@ -1039,22 +1039,22 @@
         <v>65.8702851631418</v>
       </c>
       <c r="G12" s="12" t="n">
+        <v>13.53391634524303</v>
+      </c>
+      <c r="H12" s="12" t="n">
         <v>13.49597664032086</v>
       </c>
-      <c r="H12" s="12" t="n">
-        <v>13.53391634524303</v>
-      </c>
       <c r="I12" s="12" t="n">
+        <v>2.508810561161085</v>
+      </c>
+      <c r="J12" s="12" t="n">
         <v>2.442336292576434</v>
       </c>
-      <c r="J12" s="12" t="n">
-        <v>2.508810561161085</v>
-      </c>
       <c r="K12" s="12" t="n">
+        <v>6.00640945771851</v>
+      </c>
+      <c r="L12" s="12" t="n">
         <v>6.012674562310913</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>6.00640945771851</v>
       </c>
       <c r="N12" s="12" t="n">
         <v>74.64872727492202</v>
@@ -1085,22 +1085,22 @@
         <v>65.66942408270566</v>
       </c>
       <c r="G13" s="12" t="n">
+        <v>10.34472844680575</v>
+      </c>
+      <c r="H13" s="12" t="n">
         <v>8.752914474025813</v>
       </c>
-      <c r="H13" s="12" t="n">
-        <v>10.34472844680575</v>
-      </c>
       <c r="I13" s="12" t="n">
+        <v>2.600647921697557</v>
+      </c>
+      <c r="J13" s="12" t="n">
         <v>2.4963453565413</v>
       </c>
-      <c r="J13" s="12" t="n">
-        <v>2.600647921697557</v>
-      </c>
       <c r="K13" s="12" t="n">
+        <v>5.974020827613913</v>
+      </c>
+      <c r="L13" s="12" t="n">
         <v>6.038621989942818</v>
-      </c>
-      <c r="L13" s="12" t="n">
-        <v>5.974020827613913</v>
       </c>
       <c r="N13" s="12" t="n">
         <v>79.72717607824583</v>
@@ -1131,22 +1131,22 @@
         <v>65.70741180742932</v>
       </c>
       <c r="G14" s="12" t="n">
+        <v>13.55304835413125</v>
+      </c>
+      <c r="H14" s="12" t="n">
         <v>12.57740499189996</v>
       </c>
-      <c r="H14" s="12" t="n">
-        <v>13.55304835413125</v>
-      </c>
       <c r="I14" s="12" t="n">
+        <v>2.482008693893898</v>
+      </c>
+      <c r="J14" s="12" t="n">
         <v>2.43176420351924</v>
       </c>
-      <c r="J14" s="12" t="n">
-        <v>2.482008693893898</v>
-      </c>
       <c r="K14" s="12" t="n">
+        <v>5.65132604483546</v>
+      </c>
+      <c r="L14" s="12" t="n">
         <v>5.611819489054069</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>5.65132604483546</v>
       </c>
       <c r="N14" s="12" t="n">
         <v>75.03522395951056</v>
@@ -1177,22 +1177,22 @@
         <v>59.38875555604665</v>
       </c>
       <c r="G15" s="12" t="n">
+        <v>11.38909136611622</v>
+      </c>
+      <c r="H15" s="12" t="n">
         <v>9.217988108379465</v>
       </c>
-      <c r="H15" s="12" t="n">
-        <v>11.38909136611622</v>
-      </c>
       <c r="I15" s="12" t="n">
+        <v>2.205507214269044</v>
+      </c>
+      <c r="J15" s="12" t="n">
         <v>2.051430093232368</v>
       </c>
-      <c r="J15" s="12" t="n">
-        <v>2.205507214269044</v>
-      </c>
       <c r="K15" s="12" t="n">
+        <v>5.708035342501153</v>
+      </c>
+      <c r="L15" s="12" t="n">
         <v>5.772609777053156</v>
-      </c>
-      <c r="L15" s="12" t="n">
-        <v>5.708035342501153</v>
       </c>
       <c r="N15" s="12" t="n">
         <v>88.04571359162615</v>
@@ -1223,22 +1223,22 @@
         <v>65.73606767103875</v>
       </c>
       <c r="G16" s="12" t="n">
+        <v>13.46619869627644</v>
+      </c>
+      <c r="H16" s="12" t="n">
         <v>13.0762751285376</v>
       </c>
-      <c r="H16" s="12" t="n">
-        <v>13.46619869627644</v>
-      </c>
       <c r="I16" s="12" t="n">
+        <v>2.530507886461532</v>
+      </c>
+      <c r="J16" s="12" t="n">
         <v>2.406867717645298</v>
       </c>
-      <c r="J16" s="12" t="n">
-        <v>2.530507886461532</v>
-      </c>
       <c r="K16" s="12" t="n">
+        <v>6.880910677440298</v>
+      </c>
+      <c r="L16" s="12" t="n">
         <v>6.997038710981946</v>
-      </c>
-      <c r="L16" s="12" t="n">
-        <v>6.880910677440298</v>
       </c>
       <c r="N16" s="12" t="n">
         <v>73.90577715059779</v>
@@ -1269,22 +1269,22 @@
         <v>64.0383040145167</v>
       </c>
       <c r="G17" s="12" t="n">
+        <v>11.2845364211643</v>
+      </c>
+      <c r="H17" s="12" t="n">
         <v>9.090609075592383</v>
       </c>
-      <c r="H17" s="12" t="n">
-        <v>11.2845364211643</v>
-      </c>
       <c r="I17" s="12" t="n">
+        <v>2.816155411363216</v>
+      </c>
+      <c r="J17" s="12" t="n">
         <v>2.860118844488741</v>
       </c>
-      <c r="J17" s="12" t="n">
-        <v>2.816155411363216</v>
-      </c>
       <c r="K17" s="12" t="n">
+        <v>4.285634093794099</v>
+      </c>
+      <c r="L17" s="12" t="n">
         <v>-5.074183378406207</v>
-      </c>
-      <c r="L17" s="12" t="n">
-        <v>4.285634093794099</v>
       </c>
       <c r="N17" s="12" t="n">
         <v>68.28333024041815</v>
@@ -1315,22 +1315,22 @@
         <v>59.1370210539855</v>
       </c>
       <c r="G18" s="12" t="n">
+        <v>10.90235975619652</v>
+      </c>
+      <c r="H18" s="12" t="n">
         <v>9.298218710358531</v>
       </c>
-      <c r="H18" s="12" t="n">
-        <v>10.90235975619652</v>
-      </c>
       <c r="I18" s="12" t="n">
+        <v>1.785676380497938</v>
+      </c>
+      <c r="J18" s="12" t="n">
         <v>2.234199341235402</v>
       </c>
-      <c r="J18" s="12" t="n">
-        <v>1.785676380497938</v>
-      </c>
       <c r="K18" s="12" t="n">
+        <v>6.28213780192523</v>
+      </c>
+      <c r="L18" s="12" t="n">
         <v>6.153203585999094</v>
-      </c>
-      <c r="L18" s="12" t="n">
-        <v>6.28213780192523</v>
       </c>
       <c r="N18" s="12" t="n">
         <v>88.67943246015832</v>
@@ -1360,14 +1360,14 @@
       <c r="E19" s="12" t="n">
         <v>59.23661201034648</v>
       </c>
-      <c r="G19" s="12" t="n"/>
-      <c r="H19" s="12" t="n">
+      <c r="G19" s="12" t="n">
         <v>13.21362602139954</v>
       </c>
-      <c r="I19" s="12" t="n"/>
-      <c r="J19" s="12" t="n">
+      <c r="H19" s="12" t="n"/>
+      <c r="I19" s="12" t="n">
         <v>1.957221583036022</v>
       </c>
+      <c r="J19" s="12" t="n"/>
       <c r="K19" s="12" t="n"/>
       <c r="L19" s="12" t="n"/>
       <c r="N19" s="12" t="n">
@@ -1399,22 +1399,22 @@
         <v>64.8315352659377</v>
       </c>
       <c r="G20" s="12" t="n">
+        <v>12.70303161119155</v>
+      </c>
+      <c r="H20" s="12" t="n">
         <v>33.66624621193642</v>
       </c>
-      <c r="H20" s="12" t="n">
-        <v>12.70303161119155</v>
-      </c>
       <c r="I20" s="12" t="n">
+        <v>2.57309291690476</v>
+      </c>
+      <c r="J20" s="12" t="n">
         <v>2.445732512291535</v>
       </c>
-      <c r="J20" s="12" t="n">
-        <v>2.57309291690476</v>
-      </c>
       <c r="K20" s="12" t="n">
+        <v>6.007393363162096</v>
+      </c>
+      <c r="L20" s="12" t="n">
         <v>6.075770581889359</v>
-      </c>
-      <c r="L20" s="12" t="n">
-        <v>6.007393363162096</v>
       </c>
       <c r="N20" s="12" t="n">
         <v>73.615117528325</v>
@@ -1445,22 +1445,22 @@
         <v>63.27288167154923</v>
       </c>
       <c r="G21" s="12" t="n">
+        <v>12.88250578863723</v>
+      </c>
+      <c r="H21" s="12" t="n">
         <v>10.57362386348484</v>
       </c>
-      <c r="H21" s="12" t="n">
-        <v>12.88250578863723</v>
-      </c>
       <c r="I21" s="12" t="n">
+        <v>2.65388937934197</v>
+      </c>
+      <c r="J21" s="12" t="n">
         <v>2.660838571659169</v>
       </c>
-      <c r="J21" s="12" t="n">
-        <v>2.65388937934197</v>
-      </c>
       <c r="K21" s="12" t="n">
+        <v>6.03815459399384</v>
+      </c>
+      <c r="L21" s="12" t="n">
         <v>6.082955815541398</v>
-      </c>
-      <c r="L21" s="12" t="n">
-        <v>6.03815459399384</v>
       </c>
       <c r="N21" s="12" t="n">
         <v>76.44849498775712</v>
@@ -1491,22 +1491,22 @@
         <v>59.81068856039619</v>
       </c>
       <c r="G22" s="12" t="n">
+        <v>11.08713154202064</v>
+      </c>
+      <c r="H22" s="12" t="n">
         <v>8.852471066733433</v>
       </c>
-      <c r="H22" s="12" t="n">
-        <v>11.08713154202064</v>
-      </c>
       <c r="I22" s="12" t="n">
+        <v>2.461022994512026</v>
+      </c>
+      <c r="J22" s="12" t="n">
         <v>1.895941221429606</v>
       </c>
-      <c r="J22" s="12" t="n">
-        <v>2.461022994512026</v>
-      </c>
       <c r="K22" s="12" t="n">
+        <v>6.408061033793929</v>
+      </c>
+      <c r="L22" s="12" t="n">
         <v>6.050213606260371</v>
-      </c>
-      <c r="L22" s="12" t="n">
-        <v>6.408061033793929</v>
       </c>
       <c r="N22" s="12" t="n">
         <v>87.42182636278613</v>
@@ -1537,22 +1537,22 @@
         <v>66.11203682412281</v>
       </c>
       <c r="G23" s="12" t="n">
+        <v>8.121909435935089</v>
+      </c>
+      <c r="H23" s="12" t="n">
         <v>8.29544028994597</v>
       </c>
-      <c r="H23" s="12" t="n">
-        <v>8.121909435935089</v>
-      </c>
       <c r="I23" s="12" t="n">
+        <v>2.803934133092058</v>
+      </c>
+      <c r="J23" s="12" t="n">
         <v>3.109771258624045</v>
       </c>
-      <c r="J23" s="12" t="n">
-        <v>2.803934133092058</v>
-      </c>
       <c r="K23" s="12" t="n">
+        <v>6.04003272711709</v>
+      </c>
+      <c r="L23" s="12" t="n">
         <v>6.080498563083318</v>
-      </c>
-      <c r="L23" s="12" t="n">
-        <v>6.04003272711709</v>
       </c>
       <c r="N23" s="12" t="n">
         <v>78.62720513334003</v>
@@ -1583,22 +1583,22 @@
         <v>65.03029109521688</v>
       </c>
       <c r="G24" s="12" t="n">
+        <v>9.084879332389162</v>
+      </c>
+      <c r="H24" s="12" t="n">
         <v>0.8945106292958553</v>
       </c>
-      <c r="H24" s="12" t="n">
-        <v>9.084879332389162</v>
-      </c>
       <c r="I24" s="12" t="n">
+        <v>2.540560117061978</v>
+      </c>
+      <c r="J24" s="12" t="n">
         <v>2.528051805112911</v>
       </c>
-      <c r="J24" s="12" t="n">
-        <v>2.540560117061978</v>
-      </c>
       <c r="K24" s="12" t="n">
+        <v>5.996302561646106</v>
+      </c>
+      <c r="L24" s="12" t="n">
         <v>6.012177087340032</v>
-      </c>
-      <c r="L24" s="12" t="n">
-        <v>5.996302561646106</v>
       </c>
       <c r="N24" s="12" t="n">
         <v>68.39471084960938</v>
@@ -1629,22 +1629,22 @@
         <v>64.62076462366937</v>
       </c>
       <c r="G25" s="12" t="n">
+        <v>8.418931303248074</v>
+      </c>
+      <c r="H25" s="12" t="n">
         <v>8.039895736479545</v>
       </c>
-      <c r="H25" s="12" t="n">
-        <v>8.418931303248074</v>
-      </c>
       <c r="I25" s="12" t="n">
+        <v>2.593971714310483</v>
+      </c>
+      <c r="J25" s="12" t="n">
         <v>2.430102285053141</v>
       </c>
-      <c r="J25" s="12" t="n">
-        <v>2.593971714310483</v>
-      </c>
       <c r="K25" s="12" t="n">
+        <v>6.182711907772715</v>
+      </c>
+      <c r="L25" s="12" t="n">
         <v>6.118250203349784</v>
-      </c>
-      <c r="L25" s="12" t="n">
-        <v>6.182711907772715</v>
       </c>
       <c r="N25" s="12" t="n">
         <v>75.91604772069415</v>
@@ -1675,22 +1675,22 @@
         <v>64.09954293186671</v>
       </c>
       <c r="G26" s="12" t="n">
+        <v>11.5146944102667</v>
+      </c>
+      <c r="H26" s="12" t="n">
         <v>9.772629043412993</v>
       </c>
-      <c r="H26" s="12" t="n">
-        <v>11.5146944102667</v>
-      </c>
       <c r="I26" s="12" t="n">
+        <v>2.779636097849052</v>
+      </c>
+      <c r="J26" s="12" t="n">
         <v>2.830531793569066</v>
       </c>
-      <c r="J26" s="12" t="n">
-        <v>2.779636097849052</v>
-      </c>
       <c r="K26" s="12" t="n">
+        <v>5.110883243669188</v>
+      </c>
+      <c r="L26" s="12" t="n">
         <v>5.057458912602819</v>
-      </c>
-      <c r="L26" s="12" t="n">
-        <v>5.110883243669188</v>
       </c>
       <c r="N26" s="12" t="n">
         <v>69.69585627868229</v>
@@ -1721,22 +1721,22 @@
         <v>73.2274801830293</v>
       </c>
       <c r="G27" s="12" t="n">
+        <v>14.36163396557207</v>
+      </c>
+      <c r="H27" s="12" t="n">
         <v>13.68643387721228</v>
       </c>
-      <c r="H27" s="12" t="n">
-        <v>14.36163396557207</v>
-      </c>
       <c r="I27" s="12" t="n">
+        <v>6.635899196594867</v>
+      </c>
+      <c r="J27" s="12" t="n">
         <v>4.992480401912901</v>
       </c>
-      <c r="J27" s="12" t="n">
-        <v>6.635899196594867</v>
-      </c>
       <c r="K27" s="12" t="n">
+        <v>8.807205305100316</v>
+      </c>
+      <c r="L27" s="12" t="n">
         <v>5.854569338378427</v>
-      </c>
-      <c r="L27" s="12" t="n">
-        <v>8.807205305100316</v>
       </c>
       <c r="N27" s="12" t="n">
         <v>53.51473286129815</v>
@@ -1767,22 +1767,22 @@
         <v>79.94932769353814</v>
       </c>
       <c r="G28" s="12" t="n">
+        <v>35.36355114061585</v>
+      </c>
+      <c r="H28" s="12" t="n">
         <v>24.00107850124972</v>
       </c>
-      <c r="H28" s="12" t="n">
-        <v>35.36355114061585</v>
-      </c>
       <c r="I28" s="12" t="n">
+        <v>2.86117081125284</v>
+      </c>
+      <c r="J28" s="12" t="n">
         <v>2.104280411731666</v>
       </c>
-      <c r="J28" s="12" t="n">
-        <v>2.86117081125284</v>
-      </c>
       <c r="K28" s="12" t="n">
+        <v>5.201027554317148</v>
+      </c>
+      <c r="L28" s="12" t="n">
         <v>4.436353102971825</v>
-      </c>
-      <c r="L28" s="12" t="n">
-        <v>5.201027554317148</v>
       </c>
       <c r="N28" s="12" t="n">
         <v>45.66178232999884</v>
@@ -1813,22 +1813,22 @@
         <v>79.87213161499287</v>
       </c>
       <c r="G29" s="12" t="n">
+        <v>34.95150900429803</v>
+      </c>
+      <c r="H29" s="12" t="n">
         <v>14.49676600322688</v>
       </c>
-      <c r="H29" s="12" t="n">
-        <v>34.95150900429803</v>
-      </c>
       <c r="I29" s="12" t="n">
+        <v>2.97381494482185</v>
+      </c>
+      <c r="J29" s="12" t="n">
         <v>2.023627123703744</v>
       </c>
-      <c r="J29" s="12" t="n">
-        <v>2.97381494482185</v>
-      </c>
       <c r="K29" s="12" t="n">
+        <v>5.17628633518545</v>
+      </c>
+      <c r="L29" s="12" t="n">
         <v>4.417117776204636</v>
-      </c>
-      <c r="L29" s="12" t="n">
-        <v>5.17628633518545</v>
       </c>
       <c r="N29" s="12" t="n">
         <v>47.3887496167302</v>
@@ -2000,7 +2000,7 @@
       </c>
       <c r="B6" s="14" t="inlineStr">
         <is>
-          <t>lambda_S0_to_T1 / kcal mol-1</t>
+          <t>lambda_S0_T1 / kcal mol-1</t>
         </is>
       </c>
       <c r="C6" s="14" t="inlineStr">
@@ -2010,12 +2010,12 @@
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>Relaxation from the S0 geometry to the T1 geometry on the triplet surface, electronic energies x 627.509. lamba_T-S in the delivered file.</t>
+          <t>S0 surface: E_S0 at the T1 geometry minus E_S0 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
       <c r="E6" s="14" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_S0_to_T1 / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_S0_T1 / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="B7" s="14" t="inlineStr">
         <is>
-          <t>lambda_T1_to_S0 / kcal mol-1</t>
+          <t>lambda_T1_S0 / kcal mol-1</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
@@ -2037,12 +2037,12 @@
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>Relaxation from the T1 geometry to the S0 geometry on the singlet surface, electronic energies x 627.509. lambda_S-T in the delivered file.</t>
+          <t>T1 surface: E_T1 at the S0 geometry minus E_T1 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
       <c r="E7" s="14" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_T1_to_S0 / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_T1_S0 / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2054,7 +2054,7 @@
       </c>
       <c r="B8" s="14" t="inlineStr">
         <is>
-          <t>lambda_S0_to_ox / kcal mol-1</t>
+          <t>lambda_S0_Dplus / kcal mol-1</t>
         </is>
       </c>
       <c r="C8" s="14" t="inlineStr">
@@ -2064,12 +2064,12 @@
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Relaxation from the S0 geometry to the ox geometry on the cation surface, electronic energies x 627.509. lambda_D+_S0 in the delivered file.</t>
+          <t>S0 surface: E_S0 at the Dplus geometry minus E_S0 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
       <c r="E8" s="14" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_S0_to_ox / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_S0_Dplus / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2081,7 +2081,7 @@
       </c>
       <c r="B9" s="14" t="inlineStr">
         <is>
-          <t>lambda_ox_to_S0 / kcal mol-1</t>
+          <t>lambda_Dplus_S0 / kcal mol-1</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
@@ -2091,12 +2091,12 @@
       </c>
       <c r="D9" s="15" t="inlineStr">
         <is>
-          <t>Relaxation from the ox geometry to the S0 geometry on the neutral surface, electronic energies x 627.509. lambda_S0_D+ in the delivered file.</t>
+          <t>Dplus surface: E_Dplus at the S0 geometry minus E_Dplus at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
       <c r="E9" s="14" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_ox_to_S0 / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_Dplus_S0 / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2108,7 +2108,7 @@
       </c>
       <c r="B10" s="14" t="inlineStr">
         <is>
-          <t>lambda_S0_to_red / kcal mol-1</t>
+          <t>lambda_S0_Dminus / kcal mol-1</t>
         </is>
       </c>
       <c r="C10" s="14" t="inlineStr">
@@ -2118,12 +2118,12 @@
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>Relaxation from the S0 geometry to the red geometry on the anion surface, electronic energies x 627.509. lambda_D-_S0 in the delivered file.</t>
+          <t>S0 surface: E_S0 at the Dminus geometry minus E_S0 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
       <c r="E10" s="14" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_S0_to_red / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_S0_Dminus / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2135,7 +2135,7 @@
       </c>
       <c r="B11" s="14" t="inlineStr">
         <is>
-          <t>lambda_red_to_S0 / kcal mol-1</t>
+          <t>lambda_Dminus_S0 / kcal mol-1</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
@@ -2145,12 +2145,12 @@
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>Relaxation from the red geometry to the S0 geometry on the neutral surface, electronic energies x 627.509. lambda_S0_D- in the delivered file.</t>
+          <t>Dminus surface: E_Dminus at the S0 geometry minus E_Dminus at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
       <c r="E11" s="14" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_red_to_S0 / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_Dminus_S0 / kcal mol-1</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Drop the strict label and k_q_floor, tidy data/ for publication
The ladder label `quenches` is now the only ground truth: quenches_strict
and quenching_observed are removed, and the benchmark scores one label
(label_regimes.csv is gone). k_q_floor leaves exp_dataset; pairs.py
computes 10/tau0 where the benchmark still needs it.

Docstrings, comments, column descriptions and the data README are cut
down to what is needed to use and re-run the pipeline. emission_spectra.py
and its output are removed, as nothing reads them, along with unused
helpers. Every data output rebuilds unchanged apart from the dropped
columns and the Column key descriptions.
</commit_message>
<xml_diff>
--- a/data/computational_data_processed/photocatalyst_properties_calc.xlsx
+++ b/data/computational_data_processed/photocatalyst_properties_calc.xlsx
@@ -1859,7 +1859,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>Adiabatic, Gibbs-corrected: ((E_T1 + G_T1) - (E_S0 + G_S0)) x 627.503. E_T_calc in the delivered file.</t>
+          <t>Adiabatic, Gibbs-corrected: ((E_T1 + G_T1) - (E_S0 + G_S0)) x 627.503.</t>
         </is>
       </c>
       <c r="E5" s="14" t="inlineStr">
@@ -2226,7 +2226,7 @@
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>PC*/PC-, how strong an oxidant the triplet is: -dG_red_ES / 23.061 - 4.42. E_ox_ES in the delivered file.</t>
+          <t>PC*/PC-, how strong an oxidant the triplet is: -dG_red_ES / 23.061 - 4.42.</t>
         </is>
       </c>
       <c r="E14" s="14" t="inlineStr">
@@ -2253,7 +2253,7 @@
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>PC+/PC*, how strong a reductant the triplet is: dG_ox_ES / 23.061 - 4.42. E_red_ES in the delivered file.</t>
+          <t>PC+/PC*, how strong a reductant the triplet is: dG_ox_ES / 23.061 - 4.42.</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
@@ -2283,7 +2283,7 @@
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>Every value is computed from the</t>
+          <t>Every value is computed from the ORCA outputs. Old PC19 (new 17) lacks four single</t>
         </is>
       </c>
       <c r="B18" s="14" t="n"/>
@@ -2294,7 +2294,7 @@
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>ORCA outputs with the arithmetic of Leon's delivered photocatalyst property file and</t>
+          <t>points, so four of its lambdas are blank. Total energies, Gibbs corrections and</t>
         </is>
       </c>
       <c r="B19" s="14" t="n"/>
@@ -2305,7 +2305,7 @@
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>reproduces it to 5e-8, except E_T for old PC10, PC13, PC25 and PC28 (new 8, 11, 23,</t>
+          <t>frequency checks are in computational_data_raw/photocatalysts/photocatalyst_dft.csv.</t>
         </is>
       </c>
       <c r="B20" s="14" t="n"/>
@@ -2316,7 +2316,7 @@
     <row r="21">
       <c r="A21" s="14" t="inlineStr">
         <is>
-          <t>26), where that file carries values no delivered job reproduces. Old PC19 (new 17)</t>
+          <t>Read with pandas as: pd.read_excel(path, header=1), then drop the 'Unnamed' columns.</t>
         </is>
       </c>
       <c r="B21" s="14" t="n"/>
@@ -2324,39 +2324,6 @@
       <c r="D21" s="15" t="n"/>
       <c r="E21" s="14" t="n"/>
     </row>
-    <row r="22">
-      <c r="A22" s="14" t="inlineStr">
-        <is>
-          <t>lacks four single points, so four of its lambdas are blank. Total energies, Gibbs corrections and frequency checks are</t>
-        </is>
-      </c>
-      <c r="B22" s="14" t="n"/>
-      <c r="C22" s="14" t="n"/>
-      <c r="D22" s="15" t="n"/>
-      <c r="E22" s="14" t="n"/>
-    </row>
-    <row r="23">
-      <c r="A23" s="14" t="inlineStr">
-        <is>
-          <t>in computational_data_raw/photocatalysts/photocatalyst_dft.csv.</t>
-        </is>
-      </c>
-      <c r="B23" s="14" t="n"/>
-      <c r="C23" s="14" t="n"/>
-      <c r="D23" s="15" t="n"/>
-      <c r="E23" s="14" t="n"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="14" t="inlineStr">
-        <is>
-          <t>Read with pandas as: pd.read_excel(path, header=1), then drop the 'Unnamed' columns.</t>
-        </is>
-      </c>
-      <c r="B24" s="14" t="n"/>
-      <c r="C24" s="14" t="n"/>
-      <c r="D24" s="15" t="n"/>
-      <c r="E24" s="14" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Regenerate the data from raw inputs and rerun the benchmark
Merge the recomputed quencher and photocatalyst jobs into the extracted DFT tables and
rebuild every derived table from the raw inputs. Values in kcal/mol and V are written with
at most two decimals and Hartree energies with every digit; rounding happens only when a
table is written, and derived values are computed from full precision.

Rerun the benchmark and the further analyses on the regenerated dataset. The computational
cost changes slightly because the quencher merge replaced twelve jobs and their timings.

The READMEs no longer quote results; they point to the result files instead.
</commit_message>
<xml_diff>
--- a/data/computational_data_processed/photocatalyst_properties_calc.xlsx
+++ b/data/computational_data_processed/photocatalyst_properties_calc.xlsx
@@ -622,37 +622,37 @@
         </is>
       </c>
       <c r="E3" s="12" t="n">
-        <v>65.70102948398493</v>
+        <v>65.7</v>
       </c>
       <c r="G3" s="12" t="n">
-        <v>10.27558245293145</v>
+        <v>10.28</v>
       </c>
       <c r="H3" s="12" t="n">
-        <v>8.251113847131</v>
+        <v>8.25</v>
       </c>
       <c r="I3" s="12" t="n">
-        <v>2.719382899684559</v>
+        <v>2.72</v>
       </c>
       <c r="J3" s="12" t="n">
-        <v>2.579593446458603</v>
+        <v>2.58</v>
       </c>
       <c r="K3" s="12" t="n">
-        <v>6.066670200749988</v>
+        <v>6.07</v>
       </c>
       <c r="L3" s="12" t="n">
-        <v>6.115006106872588</v>
+        <v>6.12</v>
       </c>
       <c r="N3" s="12" t="n">
-        <v>78.88260727943963</v>
+        <v>78.88</v>
       </c>
       <c r="O3" s="12" t="n">
-        <v>-135.2331948117118</v>
+        <v>-135.23</v>
       </c>
       <c r="P3" s="12" t="n">
-        <v>1.44415137295485</v>
+        <v>1.44</v>
       </c>
       <c r="Q3" s="12" t="n">
-        <v>-0.9993934660491899</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="4">
@@ -668,37 +668,37 @@
         </is>
       </c>
       <c r="E4" s="12" t="n">
-        <v>64.17789905286688</v>
+        <v>64.18000000000001</v>
       </c>
       <c r="G4" s="12" t="n">
-        <v>11.35464264717792</v>
+        <v>11.35</v>
       </c>
       <c r="H4" s="12" t="n">
-        <v>9.349048755462885</v>
+        <v>9.35</v>
       </c>
       <c r="I4" s="12" t="n">
-        <v>2.931068175715682</v>
+        <v>2.93</v>
       </c>
       <c r="J4" s="12" t="n">
-        <v>2.801124465718414</v>
+        <v>2.8</v>
       </c>
       <c r="K4" s="12" t="n">
-        <v>6.016309364188979</v>
+        <v>6.02</v>
       </c>
       <c r="L4" s="12" t="n">
-        <v>8.595742985025044</v>
+        <v>8.6</v>
       </c>
       <c r="N4" s="12" t="n">
-        <v>68.86705232991353</v>
+        <v>68.87</v>
       </c>
       <c r="O4" s="12" t="n">
-        <v>-131.404820075322</v>
+        <v>-131.4</v>
       </c>
       <c r="P4" s="12" t="n">
-        <v>1.278140586935604</v>
+        <v>1.28</v>
       </c>
       <c r="Q4" s="12" t="n">
-        <v>-1.4337005190619</v>
+        <v>-1.43</v>
       </c>
     </row>
     <row r="5">
@@ -714,37 +714,37 @@
         </is>
       </c>
       <c r="E5" s="12" t="n">
-        <v>60.37977711302834</v>
+        <v>60.38</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>11.81912009778503</v>
+        <v>11.82</v>
       </c>
       <c r="H5" s="12" t="n">
-        <v>8.481128584206719</v>
+        <v>8.48</v>
       </c>
       <c r="I5" s="12" t="n">
-        <v>2.863742889509551</v>
+        <v>2.86</v>
       </c>
       <c r="J5" s="12" t="n">
-        <v>1.822697743843328</v>
+        <v>1.82</v>
       </c>
       <c r="K5" s="12" t="n">
-        <v>4.599361755362191</v>
+        <v>4.6</v>
       </c>
       <c r="L5" s="12" t="n">
-        <v>4.320535408871186</v>
+        <v>4.32</v>
       </c>
       <c r="N5" s="12" t="n">
-        <v>61.94475067884279</v>
+        <v>61.94</v>
       </c>
       <c r="O5" s="12" t="n">
-        <v>-108.3778519471726</v>
+        <v>-108.38</v>
       </c>
       <c r="P5" s="12" t="n">
-        <v>0.2796163196380288</v>
+        <v>0.28</v>
       </c>
       <c r="Q5" s="12" t="n">
-        <v>-1.733874043673614</v>
+        <v>-1.73</v>
       </c>
     </row>
     <row r="6">
@@ -760,37 +760,37 @@
         </is>
       </c>
       <c r="E6" s="12" t="n">
-        <v>65.61781249707244</v>
+        <v>65.62</v>
       </c>
       <c r="G6" s="12" t="n">
-        <v>13.32092869504703</v>
+        <v>13.32</v>
       </c>
       <c r="H6" s="12" t="n">
-        <v>8.885442302106865</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="I6" s="12" t="n">
-        <v>1.476863333423498</v>
+        <v>1.48</v>
       </c>
       <c r="J6" s="12" t="n">
-        <v>1.345780894116102</v>
+        <v>1.35</v>
       </c>
       <c r="K6" s="12" t="n">
-        <v>4.459122623498202</v>
+        <v>4.46</v>
       </c>
       <c r="L6" s="12" t="n">
-        <v>4.190890959573786</v>
+        <v>4.19</v>
       </c>
       <c r="N6" s="12" t="n">
-        <v>65.90427545472191</v>
+        <v>65.90000000000001</v>
       </c>
       <c r="O6" s="12" t="n">
-        <v>-116.1214419417835</v>
+        <v>-116.12</v>
       </c>
       <c r="P6" s="12" t="n">
-        <v>0.6154035792803239</v>
+        <v>0.62</v>
       </c>
       <c r="Q6" s="12" t="n">
-        <v>-1.562176165182693</v>
+        <v>-1.56</v>
       </c>
     </row>
     <row r="7">
@@ -806,37 +806,37 @@
         </is>
       </c>
       <c r="E7" s="12" t="n">
-        <v>45.75110330770049</v>
+        <v>45.75</v>
       </c>
       <c r="G7" s="12" t="n">
-        <v>7.329913250875807</v>
+        <v>7.33</v>
       </c>
       <c r="H7" s="12" t="n">
-        <v>7.640425739288484</v>
+        <v>7.64</v>
       </c>
       <c r="I7" s="12" t="n">
-        <v>0.9700102287098725</v>
+        <v>0.97</v>
       </c>
       <c r="J7" s="12" t="n">
-        <v>1.217932027280818</v>
+        <v>1.22</v>
       </c>
       <c r="K7" s="12" t="n">
-        <v>5.82943839833115</v>
+        <v>5.83</v>
       </c>
       <c r="L7" s="12" t="n">
-        <v>5.784461481258163</v>
+        <v>5.78</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>78.86315697989353</v>
+        <v>78.86</v>
       </c>
       <c r="O7" s="12" t="n">
-        <v>-111.274063522277</v>
+        <v>-111.27</v>
       </c>
       <c r="P7" s="12" t="n">
-        <v>0.4052054777449818</v>
+        <v>0.41</v>
       </c>
       <c r="Q7" s="12" t="n">
-        <v>-1.000236894328367</v>
+        <v>-1</v>
       </c>
     </row>
     <row r="8">
@@ -852,37 +852,37 @@
         </is>
       </c>
       <c r="E8" s="12" t="n">
-        <v>46.98057297731619</v>
+        <v>46.98</v>
       </c>
       <c r="G8" s="12" t="n">
-        <v>7.029133876579498</v>
+        <v>7.03</v>
       </c>
       <c r="H8" s="12" t="n">
-        <v>7.083066470863391</v>
+        <v>7.08</v>
       </c>
       <c r="I8" s="12" t="n">
-        <v>0.9323012928471144</v>
+        <v>0.93</v>
       </c>
       <c r="J8" s="12" t="n">
-        <v>1.031472113423926</v>
+        <v>1.03</v>
       </c>
       <c r="K8" s="12" t="n">
-        <v>5.30896556283638</v>
+        <v>5.31</v>
       </c>
       <c r="L8" s="12" t="n">
-        <v>5.340455803599435</v>
+        <v>5.34</v>
       </c>
       <c r="N8" s="12" t="n">
-        <v>101.2939351971944</v>
+        <v>101.29</v>
       </c>
       <c r="O8" s="12" t="n">
-        <v>-132.6745373221603</v>
+        <v>-132.67</v>
       </c>
       <c r="P8" s="12" t="n">
-        <v>1.333199658391234</v>
+        <v>1.33</v>
       </c>
       <c r="Q8" s="12" t="n">
-        <v>-0.02756536155438294</v>
+        <v>-0.03</v>
       </c>
     </row>
     <row r="9">
@@ -898,37 +898,37 @@
         </is>
       </c>
       <c r="E9" s="12" t="n">
-        <v>66.14982962376409</v>
+        <v>66.15000000000001</v>
       </c>
       <c r="G9" s="12" t="n">
-        <v>13.76995402293388</v>
+        <v>13.77</v>
       </c>
       <c r="H9" s="12" t="n">
-        <v>9.099952497328978</v>
+        <v>9.1</v>
       </c>
       <c r="I9" s="12" t="n">
-        <v>1.456602285984715</v>
+        <v>1.46</v>
       </c>
       <c r="J9" s="12" t="n">
-        <v>1.395618918193773</v>
+        <v>1.4</v>
       </c>
       <c r="K9" s="12" t="n">
-        <v>4.253755373423006</v>
+        <v>4.25</v>
       </c>
       <c r="L9" s="12" t="n">
-        <v>4.065051497415832</v>
+        <v>4.07</v>
       </c>
       <c r="N9" s="12" t="n">
-        <v>64.16731074439966</v>
+        <v>64.17</v>
       </c>
       <c r="O9" s="12" t="n">
-        <v>-114.7943917677952</v>
+        <v>-114.79</v>
       </c>
       <c r="P9" s="12" t="n">
-        <v>0.5578583655433516</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="Q9" s="12" t="n">
-        <v>-1.637496607068225</v>
+        <v>-1.64</v>
       </c>
     </row>
     <row r="10">
@@ -944,37 +944,37 @@
         </is>
       </c>
       <c r="E10" s="12" t="n">
-        <v>55.94263348569274</v>
+        <v>55.94</v>
       </c>
       <c r="G10" s="12" t="n">
-        <v>8.626784273100959</v>
+        <v>8.630000000000001</v>
       </c>
       <c r="H10" s="12" t="n">
-        <v>9.484973307772082</v>
+        <v>9.48</v>
       </c>
       <c r="I10" s="12" t="n">
-        <v>2.683798476231521</v>
+        <v>2.68</v>
       </c>
       <c r="J10" s="12" t="n">
-        <v>2.657746064229599</v>
+        <v>2.66</v>
       </c>
       <c r="K10" s="12" t="n">
-        <v>6.561976450410632</v>
+        <v>6.56</v>
       </c>
       <c r="L10" s="12" t="n">
-        <v>7.542257737116455</v>
+        <v>7.54</v>
       </c>
       <c r="N10" s="12" t="n">
-        <v>93.31472892397659</v>
+        <v>93.31</v>
       </c>
       <c r="O10" s="12" t="n">
-        <v>-139.6462722534329</v>
+        <v>-139.65</v>
       </c>
       <c r="P10" s="12" t="n">
-        <v>1.635516770887339</v>
+        <v>1.64</v>
       </c>
       <c r="Q10" s="12" t="n">
-        <v>-0.3735697097273931</v>
+        <v>-0.37</v>
       </c>
     </row>
     <row r="11">
@@ -990,37 +990,37 @@
         </is>
       </c>
       <c r="E11" s="12" t="n">
-        <v>67.13698165978478</v>
+        <v>67.14</v>
       </c>
       <c r="G11" s="12" t="n">
-        <v>12.87573434699418</v>
+        <v>12.88</v>
       </c>
       <c r="H11" s="12" t="n">
-        <v>11.71255566140693</v>
+        <v>11.71</v>
       </c>
       <c r="I11" s="12" t="n">
-        <v>2.545378533930856</v>
+        <v>2.55</v>
       </c>
       <c r="J11" s="12" t="n">
-        <v>2.435375699634205</v>
+        <v>2.44</v>
       </c>
       <c r="K11" s="12" t="n">
-        <v>6.015743179564084</v>
+        <v>6.02</v>
       </c>
       <c r="L11" s="12" t="n">
-        <v>6.049062549482249</v>
+        <v>6.05</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>74.28718158644462</v>
+        <v>74.29000000000001</v>
       </c>
       <c r="O11" s="12" t="n">
-        <v>-135.6423459650245</v>
+        <v>-135.64</v>
       </c>
       <c r="P11" s="12" t="n">
-        <v>1.461893498331578</v>
+        <v>1.46</v>
       </c>
       <c r="Q11" s="12" t="n">
-        <v>-1.198666077514218</v>
+        <v>-1.2</v>
       </c>
     </row>
     <row r="12">
@@ -1036,37 +1036,37 @@
         </is>
       </c>
       <c r="E12" s="12" t="n">
-        <v>65.8702851631418</v>
+        <v>65.87</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>13.53391634524303</v>
+        <v>13.53</v>
       </c>
       <c r="H12" s="12" t="n">
-        <v>13.49597664032086</v>
+        <v>13.5</v>
       </c>
       <c r="I12" s="12" t="n">
-        <v>2.508810561161085</v>
+        <v>2.51</v>
       </c>
       <c r="J12" s="12" t="n">
-        <v>2.442336292576434</v>
+        <v>2.44</v>
       </c>
       <c r="K12" s="12" t="n">
-        <v>6.00640945771851</v>
+        <v>6.01</v>
       </c>
       <c r="L12" s="12" t="n">
-        <v>6.012674562310913</v>
+        <v>6.01</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>74.64872727492202</v>
+        <v>74.65000000000001</v>
       </c>
       <c r="O12" s="12" t="n">
-        <v>-133.9430708969361</v>
+        <v>-133.94</v>
       </c>
       <c r="P12" s="12" t="n">
-        <v>1.388207401974595</v>
+        <v>1.39</v>
       </c>
       <c r="Q12" s="12" t="n">
-        <v>-1.182988279999912</v>
+        <v>-1.18</v>
       </c>
     </row>
     <row r="13">
@@ -1082,37 +1082,37 @@
         </is>
       </c>
       <c r="E13" s="12" t="n">
-        <v>65.66942408270566</v>
+        <v>65.67</v>
       </c>
       <c r="G13" s="12" t="n">
-        <v>10.34472844680575</v>
+        <v>10.34</v>
       </c>
       <c r="H13" s="12" t="n">
-        <v>8.752914474025813</v>
+        <v>8.75</v>
       </c>
       <c r="I13" s="12" t="n">
-        <v>2.600647921697557</v>
+        <v>2.6</v>
       </c>
       <c r="J13" s="12" t="n">
-        <v>2.4963453565413</v>
+        <v>2.5</v>
       </c>
       <c r="K13" s="12" t="n">
-        <v>5.974020827613913</v>
+        <v>5.97</v>
       </c>
       <c r="L13" s="12" t="n">
-        <v>6.038621989942818</v>
+        <v>6.04</v>
       </c>
       <c r="N13" s="12" t="n">
-        <v>79.72717607824583</v>
+        <v>79.73</v>
       </c>
       <c r="O13" s="12" t="n">
-        <v>-137.6903899744599</v>
+        <v>-137.69</v>
       </c>
       <c r="P13" s="12" t="n">
-        <v>1.55070335087203</v>
+        <v>1.55</v>
       </c>
       <c r="Q13" s="12" t="n">
-        <v>-0.9627702147241735</v>
+        <v>-0.96</v>
       </c>
     </row>
     <row r="14">
@@ -1128,37 +1128,37 @@
         </is>
       </c>
       <c r="E14" s="12" t="n">
-        <v>65.70741180742932</v>
+        <v>65.70999999999999</v>
       </c>
       <c r="G14" s="12" t="n">
-        <v>13.55304835413125</v>
+        <v>13.55</v>
       </c>
       <c r="H14" s="12" t="n">
-        <v>12.57740499189996</v>
+        <v>12.58</v>
       </c>
       <c r="I14" s="12" t="n">
-        <v>2.482008693893898</v>
+        <v>2.48</v>
       </c>
       <c r="J14" s="12" t="n">
-        <v>2.43176420351924</v>
+        <v>2.43</v>
       </c>
       <c r="K14" s="12" t="n">
-        <v>5.65132604483546</v>
+        <v>5.65</v>
       </c>
       <c r="L14" s="12" t="n">
-        <v>5.611819489054069</v>
+        <v>5.61</v>
       </c>
       <c r="N14" s="12" t="n">
-        <v>75.03522395951056</v>
+        <v>75.04000000000001</v>
       </c>
       <c r="O14" s="12" t="n">
-        <v>-132.4555462852245</v>
+        <v>-132.46</v>
       </c>
       <c r="P14" s="12" t="n">
-        <v>1.323703494437559</v>
+        <v>1.32</v>
       </c>
       <c r="Q14" s="12" t="n">
-        <v>-1.166228526104221</v>
+        <v>-1.17</v>
       </c>
     </row>
     <row r="15">
@@ -1174,37 +1174,37 @@
         </is>
       </c>
       <c r="E15" s="12" t="n">
-        <v>59.38875555604665</v>
+        <v>59.39</v>
       </c>
       <c r="G15" s="12" t="n">
-        <v>11.38909136611622</v>
+        <v>11.39</v>
       </c>
       <c r="H15" s="12" t="n">
-        <v>9.217988108379465</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="I15" s="12" t="n">
-        <v>2.205507214269044</v>
+        <v>2.21</v>
       </c>
       <c r="J15" s="12" t="n">
-        <v>2.051430093232368</v>
+        <v>2.05</v>
       </c>
       <c r="K15" s="12" t="n">
-        <v>5.708035342501153</v>
+        <v>5.71</v>
       </c>
       <c r="L15" s="12" t="n">
-        <v>5.772609777053156</v>
+        <v>5.77</v>
       </c>
       <c r="N15" s="12" t="n">
-        <v>88.04571359162615</v>
+        <v>88.05</v>
       </c>
       <c r="O15" s="12" t="n">
-        <v>-128.1152196675285</v>
+        <v>-128.12</v>
       </c>
       <c r="P15" s="12" t="n">
-        <v>1.13549280896442</v>
+        <v>1.14</v>
       </c>
       <c r="Q15" s="12" t="n">
-        <v>-0.6020513598011292</v>
+        <v>-0.6</v>
       </c>
     </row>
     <row r="16">
@@ -1220,37 +1220,37 @@
         </is>
       </c>
       <c r="E16" s="12" t="n">
-        <v>65.73606767103875</v>
+        <v>65.73999999999999</v>
       </c>
       <c r="G16" s="12" t="n">
-        <v>13.46619869627644</v>
+        <v>13.47</v>
       </c>
       <c r="H16" s="12" t="n">
-        <v>13.0762751285376</v>
+        <v>13.08</v>
       </c>
       <c r="I16" s="12" t="n">
-        <v>2.530507886461532</v>
+        <v>2.53</v>
       </c>
       <c r="J16" s="12" t="n">
-        <v>2.406867717645298</v>
+        <v>2.41</v>
       </c>
       <c r="K16" s="12" t="n">
-        <v>6.880910677440298</v>
+        <v>6.88</v>
       </c>
       <c r="L16" s="12" t="n">
-        <v>6.997038710981946</v>
+        <v>7</v>
       </c>
       <c r="N16" s="12" t="n">
-        <v>73.90577715059779</v>
+        <v>73.91</v>
       </c>
       <c r="O16" s="12" t="n">
-        <v>-131.7423321618763</v>
+        <v>-131.74</v>
       </c>
       <c r="P16" s="12" t="n">
-        <v>1.2927762092657</v>
+        <v>1.29</v>
       </c>
       <c r="Q16" s="12" t="n">
-        <v>-1.2152050149344</v>
+        <v>-1.22</v>
       </c>
     </row>
     <row r="17">
@@ -1266,37 +1266,37 @@
         </is>
       </c>
       <c r="E17" s="12" t="n">
-        <v>64.0383040145167</v>
+        <v>64.04000000000001</v>
       </c>
       <c r="G17" s="12" t="n">
-        <v>11.2845364211643</v>
+        <v>11.28</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>9.090609075592383</v>
+        <v>9.09</v>
       </c>
       <c r="I17" s="12" t="n">
-        <v>2.816155411363216</v>
+        <v>2.82</v>
       </c>
       <c r="J17" s="12" t="n">
-        <v>2.860118844488741</v>
+        <v>2.86</v>
       </c>
       <c r="K17" s="12" t="n">
-        <v>4.285634093794099</v>
+        <v>6.86</v>
       </c>
       <c r="L17" s="12" t="n">
-        <v>-5.074183378406207</v>
+        <v>6.97</v>
       </c>
       <c r="N17" s="12" t="n">
-        <v>68.28333024041815</v>
+        <v>68.28</v>
       </c>
       <c r="O17" s="12" t="n">
-        <v>-117.9798806199833</v>
+        <v>-129.28</v>
       </c>
       <c r="P17" s="12" t="n">
-        <v>0.6959915276867124</v>
+        <v>1.19</v>
       </c>
       <c r="Q17" s="12" t="n">
-        <v>-1.459012608281594</v>
+        <v>-1.46</v>
       </c>
     </row>
     <row r="18">
@@ -1312,37 +1312,37 @@
         </is>
       </c>
       <c r="E18" s="12" t="n">
-        <v>59.1370210539855</v>
+        <v>59.14</v>
       </c>
       <c r="G18" s="12" t="n">
-        <v>10.90235975619652</v>
+        <v>10.9</v>
       </c>
       <c r="H18" s="12" t="n">
-        <v>9.298218710358531</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="I18" s="12" t="n">
-        <v>1.785676380497938</v>
+        <v>1.79</v>
       </c>
       <c r="J18" s="12" t="n">
-        <v>2.234199341235402</v>
+        <v>2.23</v>
       </c>
       <c r="K18" s="12" t="n">
-        <v>6.28213780192523</v>
+        <v>6.28</v>
       </c>
       <c r="L18" s="12" t="n">
-        <v>6.153203585999094</v>
+        <v>6.15</v>
       </c>
       <c r="N18" s="12" t="n">
-        <v>88.67943246015832</v>
+        <v>88.68000000000001</v>
       </c>
       <c r="O18" s="12" t="n">
-        <v>-133.2013137747413</v>
+        <v>-133.2</v>
       </c>
       <c r="P18" s="12" t="n">
-        <v>1.356042399494441</v>
+        <v>1.36</v>
       </c>
       <c r="Q18" s="12" t="n">
-        <v>-0.5745712475539513</v>
+        <v>-0.57</v>
       </c>
     </row>
     <row r="19">
@@ -1358,29 +1358,37 @@
         </is>
       </c>
       <c r="E19" s="12" t="n">
-        <v>59.23661201034648</v>
+        <v>60.55</v>
       </c>
       <c r="G19" s="12" t="n">
-        <v>13.21362602139954</v>
-      </c>
-      <c r="H19" s="12" t="n"/>
+        <v>13.24</v>
+      </c>
+      <c r="H19" s="12" t="n">
+        <v>10.81</v>
+      </c>
       <c r="I19" s="12" t="n">
-        <v>1.957221583036022</v>
-      </c>
-      <c r="J19" s="12" t="n"/>
-      <c r="K19" s="12" t="n"/>
-      <c r="L19" s="12" t="n"/>
+        <v>1.99</v>
+      </c>
+      <c r="J19" s="12" t="n">
+        <v>2.11</v>
+      </c>
+      <c r="K19" s="12" t="n">
+        <v>6.3</v>
+      </c>
+      <c r="L19" s="12" t="n">
+        <v>6.41</v>
+      </c>
       <c r="N19" s="12" t="n">
-        <v>83.55219660419205</v>
+        <v>83.55</v>
       </c>
       <c r="O19" s="12" t="n">
-        <v>-125.4310577273175</v>
+        <v>-127.03</v>
       </c>
       <c r="P19" s="12" t="n">
-        <v>1.019098813031417</v>
+        <v>1.09</v>
       </c>
       <c r="Q19" s="12" t="n">
-        <v>-0.7969048781842916</v>
+        <v>-0.8</v>
       </c>
     </row>
     <row r="20">
@@ -1396,37 +1404,37 @@
         </is>
       </c>
       <c r="E20" s="12" t="n">
-        <v>64.8315352659377</v>
+        <v>64.83</v>
       </c>
       <c r="G20" s="12" t="n">
-        <v>12.70303161119155</v>
+        <v>12.7</v>
       </c>
       <c r="H20" s="12" t="n">
-        <v>33.66624621193642</v>
+        <v>11.75</v>
       </c>
       <c r="I20" s="12" t="n">
-        <v>2.57309291690476</v>
+        <v>2.57</v>
       </c>
       <c r="J20" s="12" t="n">
-        <v>2.445732512291535</v>
+        <v>2.45</v>
       </c>
       <c r="K20" s="12" t="n">
-        <v>6.007393363162096</v>
+        <v>6.01</v>
       </c>
       <c r="L20" s="12" t="n">
-        <v>6.075770581889359</v>
+        <v>6.08</v>
       </c>
       <c r="N20" s="12" t="n">
-        <v>73.615117528325</v>
+        <v>73.62</v>
       </c>
       <c r="O20" s="12" t="n">
-        <v>-129.3866789465363</v>
+        <v>-129.39</v>
       </c>
       <c r="P20" s="12" t="n">
-        <v>1.190627420603454</v>
+        <v>1.19</v>
       </c>
       <c r="Q20" s="12" t="n">
-        <v>-1.227808961956333</v>
+        <v>-1.23</v>
       </c>
     </row>
     <row r="21">
@@ -1442,37 +1450,37 @@
         </is>
       </c>
       <c r="E21" s="12" t="n">
-        <v>63.27288167154923</v>
+        <v>63.27</v>
       </c>
       <c r="G21" s="12" t="n">
-        <v>12.88250578863723</v>
+        <v>12.88</v>
       </c>
       <c r="H21" s="12" t="n">
-        <v>10.57362386348484</v>
+        <v>10.57</v>
       </c>
       <c r="I21" s="12" t="n">
-        <v>2.65388937934197</v>
+        <v>2.65</v>
       </c>
       <c r="J21" s="12" t="n">
-        <v>2.660838571659169</v>
+        <v>2.66</v>
       </c>
       <c r="K21" s="12" t="n">
-        <v>6.03815459399384</v>
+        <v>6.04</v>
       </c>
       <c r="L21" s="12" t="n">
-        <v>6.082955815541398</v>
+        <v>6.08</v>
       </c>
       <c r="N21" s="12" t="n">
-        <v>76.44849498775712</v>
+        <v>76.45</v>
       </c>
       <c r="O21" s="12" t="n">
-        <v>-131.5519090812027</v>
+        <v>-131.55</v>
       </c>
       <c r="P21" s="12" t="n">
-        <v>1.284518844855067</v>
+        <v>1.28</v>
       </c>
       <c r="Q21" s="12" t="n">
-        <v>-1.104944495565799</v>
+        <v>-1.1</v>
       </c>
     </row>
     <row r="22">
@@ -1488,37 +1496,37 @@
         </is>
       </c>
       <c r="E22" s="12" t="n">
-        <v>59.81068856039619</v>
+        <v>59.81</v>
       </c>
       <c r="G22" s="12" t="n">
-        <v>11.08713154202064</v>
+        <v>11.09</v>
       </c>
       <c r="H22" s="12" t="n">
-        <v>8.852471066733433</v>
+        <v>8.85</v>
       </c>
       <c r="I22" s="12" t="n">
-        <v>2.461022994512026</v>
+        <v>2.46</v>
       </c>
       <c r="J22" s="12" t="n">
-        <v>1.895941221429606</v>
+        <v>1.9</v>
       </c>
       <c r="K22" s="12" t="n">
-        <v>6.408061033793929</v>
+        <v>6.41</v>
       </c>
       <c r="L22" s="12" t="n">
-        <v>6.050213606260371</v>
+        <v>6.05</v>
       </c>
       <c r="N22" s="12" t="n">
-        <v>87.42182636278613</v>
+        <v>87.42</v>
       </c>
       <c r="O22" s="12" t="n">
-        <v>-129.4062550204988</v>
+        <v>-129.41</v>
       </c>
       <c r="P22" s="12" t="n">
-        <v>1.191476302870597</v>
+        <v>1.19</v>
       </c>
       <c r="Q22" s="12" t="n">
-        <v>-0.6291051401593108</v>
+        <v>-0.63</v>
       </c>
     </row>
     <row r="23">
@@ -1534,37 +1542,37 @@
         </is>
       </c>
       <c r="E23" s="12" t="n">
-        <v>66.11203682412281</v>
+        <v>66.11</v>
       </c>
       <c r="G23" s="12" t="n">
-        <v>8.121909435935089</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="H23" s="12" t="n">
-        <v>8.29544028994597</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="I23" s="12" t="n">
-        <v>2.803934133092058</v>
+        <v>2.8</v>
       </c>
       <c r="J23" s="12" t="n">
-        <v>3.109771258624045</v>
+        <v>3.11</v>
       </c>
       <c r="K23" s="12" t="n">
-        <v>6.04003272711709</v>
+        <v>6.04</v>
       </c>
       <c r="L23" s="12" t="n">
-        <v>6.080498563083318</v>
+        <v>6.08</v>
       </c>
       <c r="N23" s="12" t="n">
-        <v>78.62720513334003</v>
+        <v>78.63</v>
       </c>
       <c r="O23" s="12" t="n">
-        <v>-136.3437143390196</v>
+        <v>-136.34</v>
       </c>
       <c r="P23" s="12" t="n">
-        <v>1.49230711326567</v>
+        <v>1.49</v>
       </c>
       <c r="Q23" s="12" t="n">
-        <v>-1.010468534177181</v>
+        <v>-1.01</v>
       </c>
     </row>
     <row r="24">
@@ -1580,37 +1588,37 @@
         </is>
       </c>
       <c r="E24" s="12" t="n">
-        <v>65.03029109521688</v>
+        <v>65.03</v>
       </c>
       <c r="G24" s="12" t="n">
-        <v>9.084879332389162</v>
+        <v>9.08</v>
       </c>
       <c r="H24" s="12" t="n">
-        <v>0.8945106292958553</v>
+        <v>0.89</v>
       </c>
       <c r="I24" s="12" t="n">
-        <v>2.540560117061978</v>
+        <v>2.54</v>
       </c>
       <c r="J24" s="12" t="n">
-        <v>2.528051805112911</v>
+        <v>2.53</v>
       </c>
       <c r="K24" s="12" t="n">
-        <v>5.996302561646106</v>
+        <v>6</v>
       </c>
       <c r="L24" s="12" t="n">
-        <v>6.012177087340032</v>
+        <v>6.01</v>
       </c>
       <c r="N24" s="12" t="n">
-        <v>68.39471084960938</v>
+        <v>68.39</v>
       </c>
       <c r="O24" s="12" t="n">
-        <v>-131.2437533689646</v>
+        <v>-131.24</v>
       </c>
       <c r="P24" s="12" t="n">
-        <v>1.271156210440338</v>
+        <v>1.27</v>
       </c>
       <c r="Q24" s="12" t="n">
-        <v>-1.454182782636946</v>
+        <v>-1.45</v>
       </c>
     </row>
     <row r="25">
@@ -1626,37 +1634,37 @@
         </is>
       </c>
       <c r="E25" s="12" t="n">
-        <v>64.62076462366937</v>
+        <v>64.62</v>
       </c>
       <c r="G25" s="12" t="n">
-        <v>8.418931303248074</v>
+        <v>8.42</v>
       </c>
       <c r="H25" s="12" t="n">
-        <v>8.039895736479545</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="I25" s="12" t="n">
-        <v>2.593971714310483</v>
+        <v>2.59</v>
       </c>
       <c r="J25" s="12" t="n">
-        <v>2.430102285053141</v>
+        <v>2.43</v>
       </c>
       <c r="K25" s="12" t="n">
-        <v>6.182711907772715</v>
+        <v>6.18</v>
       </c>
       <c r="L25" s="12" t="n">
-        <v>6.118250203349784</v>
+        <v>6.12</v>
       </c>
       <c r="N25" s="12" t="n">
-        <v>75.91604772069415</v>
+        <v>75.92</v>
       </c>
       <c r="O25" s="12" t="n">
-        <v>-131.3725720970614</v>
+        <v>-131.37</v>
       </c>
       <c r="P25" s="12" t="n">
-        <v>1.276742209663997</v>
+        <v>1.28</v>
       </c>
       <c r="Q25" s="12" t="n">
-        <v>-1.12803314163765</v>
+        <v>-1.13</v>
       </c>
     </row>
     <row r="26">
@@ -1672,37 +1680,37 @@
         </is>
       </c>
       <c r="E26" s="12" t="n">
-        <v>64.09954293186671</v>
+        <v>64.09999999999999</v>
       </c>
       <c r="G26" s="12" t="n">
-        <v>11.5146944102667</v>
+        <v>11.51</v>
       </c>
       <c r="H26" s="12" t="n">
-        <v>9.772629043412993</v>
+        <v>9.77</v>
       </c>
       <c r="I26" s="12" t="n">
-        <v>2.779636097849052</v>
+        <v>2.78</v>
       </c>
       <c r="J26" s="12" t="n">
-        <v>2.830531793569066</v>
+        <v>2.83</v>
       </c>
       <c r="K26" s="12" t="n">
-        <v>5.110883243669188</v>
+        <v>5.11</v>
       </c>
       <c r="L26" s="12" t="n">
-        <v>5.057458912602819</v>
+        <v>5.06</v>
       </c>
       <c r="N26" s="12" t="n">
-        <v>69.69585627868229</v>
+        <v>69.7</v>
       </c>
       <c r="O26" s="12" t="n">
-        <v>-132.2987922271187</v>
+        <v>-132.3</v>
       </c>
       <c r="P26" s="12" t="n">
-        <v>1.316906128403741</v>
+        <v>1.32</v>
       </c>
       <c r="Q26" s="12" t="n">
-        <v>-1.397760882932991</v>
+        <v>-1.4</v>
       </c>
     </row>
     <row r="27">
@@ -1718,37 +1726,37 @@
         </is>
       </c>
       <c r="E27" s="12" t="n">
-        <v>73.2274801830293</v>
+        <v>73.23</v>
       </c>
       <c r="G27" s="12" t="n">
-        <v>14.36163396557207</v>
+        <v>14.36</v>
       </c>
       <c r="H27" s="12" t="n">
-        <v>13.68643387721228</v>
+        <v>13.69</v>
       </c>
       <c r="I27" s="12" t="n">
-        <v>6.635899196594867</v>
+        <v>6.64</v>
       </c>
       <c r="J27" s="12" t="n">
-        <v>4.992480401912901</v>
+        <v>4.99</v>
       </c>
       <c r="K27" s="12" t="n">
-        <v>8.807205305100316</v>
+        <v>8.81</v>
       </c>
       <c r="L27" s="12" t="n">
-        <v>5.854569338378427</v>
+        <v>5.85</v>
       </c>
       <c r="N27" s="12" t="n">
-        <v>53.51473286129815</v>
+        <v>53.51</v>
       </c>
       <c r="O27" s="12" t="n">
-        <v>-107.2914508438991</v>
+        <v>-107.29</v>
       </c>
       <c r="P27" s="12" t="n">
-        <v>0.2325064326741728</v>
+        <v>0.23</v>
       </c>
       <c r="Q27" s="12" t="n">
-        <v>-2.099427047339745</v>
+        <v>-2.1</v>
       </c>
     </row>
     <row r="28">
@@ -1764,37 +1772,37 @@
         </is>
       </c>
       <c r="E28" s="12" t="n">
-        <v>79.94932769353814</v>
+        <v>79.95</v>
       </c>
       <c r="G28" s="12" t="n">
-        <v>35.36355114061585</v>
+        <v>35.36</v>
       </c>
       <c r="H28" s="12" t="n">
-        <v>24.00107850124972</v>
+        <v>14.38</v>
       </c>
       <c r="I28" s="12" t="n">
-        <v>2.86117081125284</v>
+        <v>2.86</v>
       </c>
       <c r="J28" s="12" t="n">
-        <v>2.104280411731666</v>
+        <v>2.1</v>
       </c>
       <c r="K28" s="12" t="n">
-        <v>5.201027554317148</v>
+        <v>5.2</v>
       </c>
       <c r="L28" s="12" t="n">
-        <v>4.436353102971825</v>
+        <v>4.44</v>
       </c>
       <c r="N28" s="12" t="n">
-        <v>45.66178232999884</v>
+        <v>45.66</v>
       </c>
       <c r="O28" s="12" t="n">
-        <v>-112.7975231551972</v>
+        <v>-112.8</v>
       </c>
       <c r="P28" s="12" t="n">
-        <v>0.4712676447334099</v>
+        <v>0.47</v>
       </c>
       <c r="Q28" s="12" t="n">
-        <v>-2.43995653570969</v>
+        <v>-2.44</v>
       </c>
     </row>
     <row r="29">
@@ -1810,37 +1818,37 @@
         </is>
       </c>
       <c r="E29" s="12" t="n">
-        <v>79.87213161499287</v>
+        <v>79.87</v>
       </c>
       <c r="G29" s="12" t="n">
-        <v>34.95150900429803</v>
+        <v>34.95</v>
       </c>
       <c r="H29" s="12" t="n">
-        <v>14.49676600322688</v>
+        <v>14.5</v>
       </c>
       <c r="I29" s="12" t="n">
-        <v>2.97381494482185</v>
+        <v>2.97</v>
       </c>
       <c r="J29" s="12" t="n">
-        <v>2.023627123703744</v>
+        <v>2.02</v>
       </c>
       <c r="K29" s="12" t="n">
-        <v>5.17628633518545</v>
+        <v>5.18</v>
       </c>
       <c r="L29" s="12" t="n">
-        <v>4.417117776204636</v>
+        <v>4.42</v>
       </c>
       <c r="N29" s="12" t="n">
-        <v>47.3887496167302</v>
+        <v>47.39</v>
       </c>
       <c r="O29" s="12" t="n">
-        <v>-112.972392858981</v>
+        <v>-112.97</v>
       </c>
       <c r="P29" s="12" t="n">
-        <v>0.4788505641117471</v>
+        <v>0.48</v>
       </c>
       <c r="Q29" s="12" t="n">
-        <v>-2.365069614642461</v>
+        <v>-2.37</v>
       </c>
     </row>
   </sheetData>
@@ -1859,7 +1867,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -2283,7 +2291,7 @@
     <row r="18">
       <c r="A18" s="14" t="inlineStr">
         <is>
-          <t>Every value is computed from the ORCA outputs. Old PC19 (new 17) lacks four single</t>
+          <t>Every value is computed from the ORCA outputs. Total energies, Gibbs corrections and</t>
         </is>
       </c>
       <c r="B18" s="14" t="n"/>
@@ -2294,7 +2302,7 @@
     <row r="19">
       <c r="A19" s="14" t="inlineStr">
         <is>
-          <t>points, so four of its lambdas are blank. Total energies, Gibbs corrections and</t>
+          <t>frequency checks are in computational_data_raw/photocatalysts/photocatalyst_dft.csv.</t>
         </is>
       </c>
       <c r="B19" s="14" t="n"/>
@@ -2305,7 +2313,7 @@
     <row r="20">
       <c r="A20" s="14" t="inlineStr">
         <is>
-          <t>frequency checks are in computational_data_raw/photocatalysts/photocatalyst_dft.csv.</t>
+          <t>Read with pandas as: pd.read_excel(path, header=1), then drop the 'Unnamed' columns.</t>
         </is>
       </c>
       <c r="B20" s="14" t="n"/>
@@ -2313,17 +2321,6 @@
       <c r="D20" s="15" t="n"/>
       <c r="E20" s="14" t="n"/>
     </row>
-    <row r="21">
-      <c r="A21" s="14" t="inlineStr">
-        <is>
-          <t>Read with pandas as: pd.read_excel(path, header=1), then drop the 'Unnamed' columns.</t>
-        </is>
-      </c>
-      <c r="B21" s="14" t="n"/>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="15" t="n"/>
-      <c r="E21" s="14" t="n"/>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Merge the recomputed photocatalyst triplets and add the organophotocatalyst library
One triplet per photocatalyst: the lowest minimum, or within 1 kcal/mol the experimentally assigned character. The organophotocatalysts are a separate library that the dataset and the benchmark do not read.
</commit_message>
<xml_diff>
--- a/data/computational_data_processed/photocatalyst_properties_calc.xlsx
+++ b/data/computational_data_processed/photocatalyst_properties_calc.xlsx
@@ -668,13 +668,13 @@
         </is>
       </c>
       <c r="E4" s="12" t="n">
-        <v>64.18000000000001</v>
+        <v>59.35</v>
       </c>
       <c r="G4" s="12" t="n">
-        <v>11.35</v>
+        <v>8.83</v>
       </c>
       <c r="H4" s="12" t="n">
-        <v>9.35</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="I4" s="12" t="n">
         <v>2.93</v>
@@ -689,16 +689,16 @@
         <v>8.6</v>
       </c>
       <c r="N4" s="12" t="n">
-        <v>68.87</v>
+        <v>73.7</v>
       </c>
       <c r="O4" s="12" t="n">
-        <v>-131.4</v>
+        <v>-126.57</v>
       </c>
       <c r="P4" s="12" t="n">
-        <v>1.28</v>
+        <v>1.07</v>
       </c>
       <c r="Q4" s="12" t="n">
-        <v>-1.43</v>
+        <v>-1.22</v>
       </c>
     </row>
     <row r="5">
@@ -806,13 +806,13 @@
         </is>
       </c>
       <c r="E7" s="12" t="n">
-        <v>45.75</v>
+        <v>44.61</v>
       </c>
       <c r="G7" s="12" t="n">
-        <v>7.33</v>
+        <v>7.15</v>
       </c>
       <c r="H7" s="12" t="n">
-        <v>7.64</v>
+        <v>7.48</v>
       </c>
       <c r="I7" s="12" t="n">
         <v>0.97</v>
@@ -827,16 +827,16 @@
         <v>5.78</v>
       </c>
       <c r="N7" s="12" t="n">
-        <v>78.86</v>
+        <v>80.01000000000001</v>
       </c>
       <c r="O7" s="12" t="n">
-        <v>-111.27</v>
+        <v>-110.13</v>
       </c>
       <c r="P7" s="12" t="n">
-        <v>0.41</v>
+        <v>0.36</v>
       </c>
       <c r="Q7" s="12" t="n">
-        <v>-1</v>
+        <v>-0.95</v>
       </c>
     </row>
     <row r="8">
@@ -990,13 +990,13 @@
         </is>
       </c>
       <c r="E11" s="12" t="n">
-        <v>67.14</v>
+        <v>63.94</v>
       </c>
       <c r="G11" s="12" t="n">
-        <v>12.88</v>
+        <v>8.31</v>
       </c>
       <c r="H11" s="12" t="n">
-        <v>11.71</v>
+        <v>7.94</v>
       </c>
       <c r="I11" s="12" t="n">
         <v>2.55</v>
@@ -1011,16 +1011,16 @@
         <v>6.05</v>
       </c>
       <c r="N11" s="12" t="n">
-        <v>74.29000000000001</v>
+        <v>77.48999999999999</v>
       </c>
       <c r="O11" s="12" t="n">
-        <v>-135.64</v>
+        <v>-132.44</v>
       </c>
       <c r="P11" s="12" t="n">
-        <v>1.46</v>
+        <v>1.32</v>
       </c>
       <c r="Q11" s="12" t="n">
-        <v>-1.2</v>
+        <v>-1.06</v>
       </c>
     </row>
     <row r="12">
@@ -1036,13 +1036,13 @@
         </is>
       </c>
       <c r="E12" s="12" t="n">
-        <v>65.87</v>
+        <v>63.38</v>
       </c>
       <c r="G12" s="12" t="n">
-        <v>13.53</v>
+        <v>8.199999999999999</v>
       </c>
       <c r="H12" s="12" t="n">
-        <v>13.5</v>
+        <v>7.88</v>
       </c>
       <c r="I12" s="12" t="n">
         <v>2.51</v>
@@ -1057,16 +1057,16 @@
         <v>6.01</v>
       </c>
       <c r="N12" s="12" t="n">
-        <v>74.65000000000001</v>
+        <v>77.14</v>
       </c>
       <c r="O12" s="12" t="n">
-        <v>-133.94</v>
+        <v>-131.45</v>
       </c>
       <c r="P12" s="12" t="n">
-        <v>1.39</v>
+        <v>1.28</v>
       </c>
       <c r="Q12" s="12" t="n">
-        <v>-1.18</v>
+        <v>-1.07</v>
       </c>
     </row>
     <row r="13">
@@ -1266,13 +1266,13 @@
         </is>
       </c>
       <c r="E17" s="12" t="n">
-        <v>64.04000000000001</v>
+        <v>59.92</v>
       </c>
       <c r="G17" s="12" t="n">
-        <v>11.28</v>
+        <v>9.140000000000001</v>
       </c>
       <c r="H17" s="12" t="n">
-        <v>9.09</v>
+        <v>9.02</v>
       </c>
       <c r="I17" s="12" t="n">
         <v>2.82</v>
@@ -1287,16 +1287,16 @@
         <v>6.97</v>
       </c>
       <c r="N17" s="12" t="n">
-        <v>68.28</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="O17" s="12" t="n">
-        <v>-129.28</v>
+        <v>-125.16</v>
       </c>
       <c r="P17" s="12" t="n">
-        <v>1.19</v>
+        <v>1.01</v>
       </c>
       <c r="Q17" s="12" t="n">
-        <v>-1.46</v>
+        <v>-1.28</v>
       </c>
     </row>
     <row r="18">
@@ -1588,13 +1588,13 @@
         </is>
       </c>
       <c r="E24" s="12" t="n">
-        <v>65.03</v>
+        <v>59.01</v>
       </c>
       <c r="G24" s="12" t="n">
-        <v>9.08</v>
+        <v>8.289999999999999</v>
       </c>
       <c r="H24" s="12" t="n">
-        <v>0.89</v>
+        <v>7.93</v>
       </c>
       <c r="I24" s="12" t="n">
         <v>2.54</v>
@@ -1609,16 +1609,16 @@
         <v>6.01</v>
       </c>
       <c r="N24" s="12" t="n">
-        <v>68.39</v>
+        <v>74.41</v>
       </c>
       <c r="O24" s="12" t="n">
-        <v>-131.24</v>
+        <v>-125.22</v>
       </c>
       <c r="P24" s="12" t="n">
-        <v>1.27</v>
+        <v>1.01</v>
       </c>
       <c r="Q24" s="12" t="n">
-        <v>-1.45</v>
+        <v>-1.19</v>
       </c>
     </row>
     <row r="25">
@@ -1680,13 +1680,13 @@
         </is>
       </c>
       <c r="E26" s="12" t="n">
-        <v>64.09999999999999</v>
+        <v>57.55</v>
       </c>
       <c r="G26" s="12" t="n">
-        <v>11.51</v>
+        <v>7.93</v>
       </c>
       <c r="H26" s="12" t="n">
-        <v>9.77</v>
+        <v>7.58</v>
       </c>
       <c r="I26" s="12" t="n">
         <v>2.78</v>
@@ -1701,16 +1701,16 @@
         <v>5.06</v>
       </c>
       <c r="N26" s="12" t="n">
-        <v>69.7</v>
+        <v>76.25</v>
       </c>
       <c r="O26" s="12" t="n">
-        <v>-132.3</v>
+        <v>-125.75</v>
       </c>
       <c r="P26" s="12" t="n">
-        <v>1.32</v>
+        <v>1.03</v>
       </c>
       <c r="Q26" s="12" t="n">
-        <v>-1.4</v>
+        <v>-1.11</v>
       </c>
     </row>
     <row r="27">
@@ -1772,13 +1772,13 @@
         </is>
       </c>
       <c r="E28" s="12" t="n">
-        <v>79.95</v>
+        <v>76.81999999999999</v>
       </c>
       <c r="G28" s="12" t="n">
-        <v>35.36</v>
+        <v>19.11</v>
       </c>
       <c r="H28" s="12" t="n">
-        <v>14.38</v>
+        <v>13.66</v>
       </c>
       <c r="I28" s="12" t="n">
         <v>2.86</v>
@@ -1793,16 +1793,16 @@
         <v>4.44</v>
       </c>
       <c r="N28" s="12" t="n">
-        <v>45.66</v>
+        <v>48.79</v>
       </c>
       <c r="O28" s="12" t="n">
-        <v>-112.8</v>
+        <v>-109.67</v>
       </c>
       <c r="P28" s="12" t="n">
-        <v>0.47</v>
+        <v>0.34</v>
       </c>
       <c r="Q28" s="12" t="n">
-        <v>-2.44</v>
+        <v>-2.3</v>
       </c>
     </row>
     <row r="29">

</xml_diff>

<commit_message>
Add molecular radii from the S0 geometries to the data set
Radius of the volume-equivalent sphere (Bondi radii) for every photocatalyst and quencher, written by the DFT extraction stages and carried into exp_dataset_ent. All other columns are unchanged.
</commit_message>
<xml_diff>
--- a/data/computational_data_processed/photocatalyst_properties_calc.xlsx
+++ b/data/computational_data_processed/photocatalyst_properties_calc.xlsx
@@ -36,7 +36,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -63,6 +63,11 @@
         <fgColor rgb="00FCE4D6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -81,7 +86,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -98,6 +103,9 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -108,6 +116,9 @@
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="bottom"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -483,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q29"/>
+  <dimension ref="A1:S29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -503,6 +514,8 @@
     <col width="24" customWidth="1" min="15" max="15"/>
     <col width="22" customWidth="1" min="16" max="16"/>
     <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="2" customWidth="1" min="18" max="18"/>
+    <col width="15" customWidth="1" min="19" max="19"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
@@ -536,1319 +549,1410 @@
       <c r="O1" s="7" t="n"/>
       <c r="P1" s="7" t="n"/>
       <c r="Q1" s="7" t="n"/>
+      <c r="S1" s="8" t="inlineStr">
+        <is>
+          <t>Molecular size / A</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="9" t="inlineStr">
         <is>
           <t>new_id</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="9" t="inlineStr">
         <is>
           <t>old_id</t>
         </is>
       </c>
-      <c r="C2" s="8" t="inlineStr">
+      <c r="C2" s="9" t="inlineStr">
         <is>
           <t>compound</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr">
+      <c r="E2" s="10" t="inlineStr">
         <is>
           <t>E_T / kcal mol-1</t>
         </is>
       </c>
-      <c r="G2" s="10" t="inlineStr">
+      <c r="G2" s="11" t="inlineStr">
         <is>
           <t>lambda_S0_T1 / kcal mol-1</t>
         </is>
       </c>
-      <c r="H2" s="10" t="inlineStr">
+      <c r="H2" s="11" t="inlineStr">
         <is>
           <t>lambda_T1_S0 / kcal mol-1</t>
         </is>
       </c>
-      <c r="I2" s="10" t="inlineStr">
+      <c r="I2" s="11" t="inlineStr">
         <is>
           <t>lambda_S0_Dplus / kcal mol-1</t>
         </is>
       </c>
-      <c r="J2" s="10" t="inlineStr">
+      <c r="J2" s="11" t="inlineStr">
         <is>
           <t>lambda_Dplus_S0 / kcal mol-1</t>
         </is>
       </c>
-      <c r="K2" s="10" t="inlineStr">
+      <c r="K2" s="11" t="inlineStr">
         <is>
           <t>lambda_S0_Dminus / kcal mol-1</t>
         </is>
       </c>
-      <c r="L2" s="10" t="inlineStr">
+      <c r="L2" s="11" t="inlineStr">
         <is>
           <t>lambda_Dminus_S0 / kcal mol-1</t>
         </is>
       </c>
-      <c r="N2" s="11" t="inlineStr">
+      <c r="N2" s="12" t="inlineStr">
         <is>
           <t>dG_ox_ES / kcal mol-1</t>
         </is>
       </c>
-      <c r="O2" s="11" t="inlineStr">
+      <c r="O2" s="12" t="inlineStr">
         <is>
           <t>dG_red_ES / kcal mol-1</t>
         </is>
       </c>
-      <c r="P2" s="11" t="inlineStr">
+      <c r="P2" s="12" t="inlineStr">
         <is>
           <t>E_PCstar_PCminus / V</t>
         </is>
       </c>
-      <c r="Q2" s="11" t="inlineStr">
+      <c r="Q2" s="12" t="inlineStr">
         <is>
           <t>E_PCplus_PCstar / V</t>
         </is>
       </c>
+      <c r="S2" s="13" t="inlineStr">
+        <is>
+          <t>radius_S0 / A</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="n">
+      <c r="A3" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="12" t="n">
+      <c r="B3" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C3" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(CF3)ppy)2(dtbbpy)][PF6]</t>
         </is>
       </c>
-      <c r="E3" s="12" t="n">
+      <c r="E3" s="14" t="n">
         <v>65.7</v>
       </c>
-      <c r="G3" s="12" t="n">
+      <c r="G3" s="14" t="n">
         <v>10.28</v>
       </c>
-      <c r="H3" s="12" t="n">
+      <c r="H3" s="14" t="n">
         <v>8.25</v>
       </c>
-      <c r="I3" s="12" t="n">
+      <c r="I3" s="14" t="n">
         <v>2.72</v>
       </c>
-      <c r="J3" s="12" t="n">
+      <c r="J3" s="14" t="n">
         <v>2.58</v>
       </c>
-      <c r="K3" s="12" t="n">
+      <c r="K3" s="14" t="n">
         <v>6.07</v>
       </c>
-      <c r="L3" s="12" t="n">
+      <c r="L3" s="14" t="n">
         <v>6.12</v>
       </c>
-      <c r="N3" s="12" t="n">
+      <c r="N3" s="14" t="n">
         <v>78.88</v>
       </c>
-      <c r="O3" s="12" t="n">
+      <c r="O3" s="14" t="n">
         <v>-135.23</v>
       </c>
-      <c r="P3" s="12" t="n">
+      <c r="P3" s="14" t="n">
         <v>1.44</v>
       </c>
-      <c r="Q3" s="12" t="n">
+      <c r="Q3" s="14" t="n">
         <v>-1</v>
       </c>
+      <c r="S3" s="14" t="n">
+        <v>5.38</v>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="n">
+      <c r="A4" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="12" t="n">
+      <c r="B4" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="14" t="inlineStr">
         <is>
           <t>[Ir(ppy)2(dtbbpy)][PF6]</t>
         </is>
       </c>
-      <c r="E4" s="12" t="n">
+      <c r="E4" s="14" t="n">
         <v>59.35</v>
       </c>
-      <c r="G4" s="12" t="n">
+      <c r="G4" s="14" t="n">
         <v>8.83</v>
       </c>
-      <c r="H4" s="12" t="n">
+      <c r="H4" s="14" t="n">
         <v>8.539999999999999</v>
       </c>
-      <c r="I4" s="12" t="n">
+      <c r="I4" s="14" t="n">
         <v>2.93</v>
       </c>
-      <c r="J4" s="12" t="n">
+      <c r="J4" s="14" t="n">
         <v>2.8</v>
       </c>
-      <c r="K4" s="12" t="n">
+      <c r="K4" s="14" t="n">
         <v>6.02</v>
       </c>
-      <c r="L4" s="12" t="n">
+      <c r="L4" s="14" t="n">
         <v>8.6</v>
       </c>
-      <c r="N4" s="12" t="n">
+      <c r="N4" s="14" t="n">
         <v>73.7</v>
       </c>
-      <c r="O4" s="12" t="n">
+      <c r="O4" s="14" t="n">
         <v>-126.57</v>
       </c>
-      <c r="P4" s="12" t="n">
+      <c r="P4" s="14" t="n">
         <v>1.07</v>
       </c>
-      <c r="Q4" s="12" t="n">
+      <c r="Q4" s="14" t="n">
         <v>-1.22</v>
       </c>
+      <c r="S4" s="14" t="n">
+        <v>5.15</v>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="n">
+      <c r="A5" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="14" t="inlineStr">
         <is>
           <t>Ir(ppy)3</t>
         </is>
       </c>
-      <c r="E5" s="12" t="n">
+      <c r="E5" s="14" t="n">
         <v>60.38</v>
       </c>
-      <c r="G5" s="12" t="n">
+      <c r="G5" s="14" t="n">
         <v>11.82</v>
       </c>
-      <c r="H5" s="12" t="n">
+      <c r="H5" s="14" t="n">
         <v>8.48</v>
       </c>
-      <c r="I5" s="12" t="n">
+      <c r="I5" s="14" t="n">
         <v>2.86</v>
       </c>
-      <c r="J5" s="12" t="n">
+      <c r="J5" s="14" t="n">
         <v>1.82</v>
       </c>
-      <c r="K5" s="12" t="n">
+      <c r="K5" s="14" t="n">
         <v>4.6</v>
       </c>
-      <c r="L5" s="12" t="n">
+      <c r="L5" s="14" t="n">
         <v>4.32</v>
       </c>
-      <c r="N5" s="12" t="n">
+      <c r="N5" s="14" t="n">
         <v>61.94</v>
       </c>
-      <c r="O5" s="12" t="n">
+      <c r="O5" s="14" t="n">
         <v>-108.38</v>
       </c>
-      <c r="P5" s="12" t="n">
+      <c r="P5" s="14" t="n">
         <v>0.28</v>
       </c>
-      <c r="Q5" s="12" t="n">
+      <c r="Q5" s="14" t="n">
         <v>-1.73</v>
       </c>
+      <c r="S5" s="14" t="n">
+        <v>4.73</v>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="n">
+      <c r="A6" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>Ir(dFppy)3</t>
         </is>
       </c>
-      <c r="E6" s="12" t="n">
+      <c r="E6" s="14" t="n">
         <v>65.62</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G6" s="14" t="n">
         <v>13.32</v>
       </c>
-      <c r="H6" s="12" t="n">
+      <c r="H6" s="14" t="n">
         <v>8.890000000000001</v>
       </c>
-      <c r="I6" s="12" t="n">
+      <c r="I6" s="14" t="n">
         <v>1.48</v>
       </c>
-      <c r="J6" s="12" t="n">
+      <c r="J6" s="14" t="n">
         <v>1.35</v>
       </c>
-      <c r="K6" s="12" t="n">
+      <c r="K6" s="14" t="n">
         <v>4.46</v>
       </c>
-      <c r="L6" s="12" t="n">
+      <c r="L6" s="14" t="n">
         <v>4.19</v>
       </c>
-      <c r="N6" s="12" t="n">
+      <c r="N6" s="14" t="n">
         <v>65.90000000000001</v>
       </c>
-      <c r="O6" s="12" t="n">
+      <c r="O6" s="14" t="n">
         <v>-116.12</v>
       </c>
-      <c r="P6" s="12" t="n">
+      <c r="P6" s="14" t="n">
         <v>0.62</v>
       </c>
-      <c r="Q6" s="12" t="n">
+      <c r="Q6" s="14" t="n">
         <v>-1.56</v>
       </c>
+      <c r="S6" s="14" t="n">
+        <v>4.82</v>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="n">
+      <c r="A7" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="12" t="n">
+      <c r="B7" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="14" t="inlineStr">
         <is>
           <t>[Ru(dtbbpy)3][PF6]2</t>
         </is>
       </c>
-      <c r="E7" s="12" t="n">
+      <c r="E7" s="14" t="n">
         <v>44.61</v>
       </c>
-      <c r="G7" s="12" t="n">
+      <c r="G7" s="14" t="n">
         <v>7.15</v>
       </c>
-      <c r="H7" s="12" t="n">
+      <c r="H7" s="14" t="n">
         <v>7.48</v>
       </c>
-      <c r="I7" s="12" t="n">
+      <c r="I7" s="14" t="n">
         <v>0.97</v>
       </c>
-      <c r="J7" s="12" t="n">
+      <c r="J7" s="14" t="n">
         <v>1.22</v>
       </c>
-      <c r="K7" s="12" t="n">
+      <c r="K7" s="14" t="n">
         <v>5.83</v>
       </c>
-      <c r="L7" s="12" t="n">
+      <c r="L7" s="14" t="n">
         <v>5.78</v>
       </c>
-      <c r="N7" s="12" t="n">
+      <c r="N7" s="14" t="n">
         <v>80.01000000000001</v>
       </c>
-      <c r="O7" s="12" t="n">
+      <c r="O7" s="14" t="n">
         <v>-110.13</v>
       </c>
-      <c r="P7" s="12" t="n">
+      <c r="P7" s="14" t="n">
         <v>0.36</v>
       </c>
-      <c r="Q7" s="12" t="n">
+      <c r="Q7" s="14" t="n">
         <v>-0.95</v>
       </c>
+      <c r="S7" s="14" t="n">
+        <v>5.84</v>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="n">
+      <c r="A8" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>[Ru(bpz)3][PF6]2</t>
         </is>
       </c>
-      <c r="E8" s="12" t="n">
+      <c r="E8" s="14" t="n">
         <v>46.98</v>
       </c>
-      <c r="G8" s="12" t="n">
+      <c r="G8" s="14" t="n">
         <v>7.03</v>
       </c>
-      <c r="H8" s="12" t="n">
+      <c r="H8" s="14" t="n">
         <v>7.08</v>
       </c>
-      <c r="I8" s="12" t="n">
+      <c r="I8" s="14" t="n">
         <v>0.93</v>
       </c>
-      <c r="J8" s="12" t="n">
+      <c r="J8" s="14" t="n">
         <v>1.03</v>
       </c>
-      <c r="K8" s="12" t="n">
+      <c r="K8" s="14" t="n">
         <v>5.31</v>
       </c>
-      <c r="L8" s="12" t="n">
+      <c r="L8" s="14" t="n">
         <v>5.34</v>
       </c>
-      <c r="N8" s="12" t="n">
+      <c r="N8" s="14" t="n">
         <v>101.29</v>
       </c>
-      <c r="O8" s="12" t="n">
+      <c r="O8" s="14" t="n">
         <v>-132.67</v>
       </c>
-      <c r="P8" s="12" t="n">
+      <c r="P8" s="14" t="n">
         <v>1.33</v>
       </c>
-      <c r="Q8" s="12" t="n">
+      <c r="Q8" s="14" t="n">
         <v>-0.03</v>
       </c>
+      <c r="S8" s="14" t="n">
+        <v>4.61</v>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="n">
+      <c r="A9" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>Ir(dF(Me)ppy)3</t>
         </is>
       </c>
-      <c r="E9" s="12" t="n">
+      <c r="E9" s="14" t="n">
         <v>66.15000000000001</v>
       </c>
-      <c r="G9" s="12" t="n">
+      <c r="G9" s="14" t="n">
         <v>13.77</v>
       </c>
-      <c r="H9" s="12" t="n">
+      <c r="H9" s="14" t="n">
         <v>9.1</v>
       </c>
-      <c r="I9" s="12" t="n">
+      <c r="I9" s="14" t="n">
         <v>1.46</v>
       </c>
-      <c r="J9" s="12" t="n">
+      <c r="J9" s="14" t="n">
         <v>1.4</v>
       </c>
-      <c r="K9" s="12" t="n">
+      <c r="K9" s="14" t="n">
         <v>4.25</v>
       </c>
-      <c r="L9" s="12" t="n">
+      <c r="L9" s="14" t="n">
         <v>4.07</v>
       </c>
-      <c r="N9" s="12" t="n">
+      <c r="N9" s="14" t="n">
         <v>64.17</v>
       </c>
-      <c r="O9" s="12" t="n">
+      <c r="O9" s="14" t="n">
         <v>-114.79</v>
       </c>
-      <c r="P9" s="12" t="n">
+      <c r="P9" s="14" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="Q9" s="12" t="n">
+      <c r="Q9" s="14" t="n">
         <v>-1.64</v>
       </c>
+      <c r="S9" s="14" t="n">
+        <v>4.99</v>
+      </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="n">
+      <c r="A10" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(CF3)ppy)2(d(5,5)CF3bpy)]PF6</t>
         </is>
       </c>
-      <c r="E10" s="12" t="n">
+      <c r="E10" s="14" t="n">
         <v>55.94</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G10" s="14" t="n">
         <v>8.630000000000001</v>
       </c>
-      <c r="H10" s="12" t="n">
+      <c r="H10" s="14" t="n">
         <v>9.48</v>
       </c>
-      <c r="I10" s="12" t="n">
+      <c r="I10" s="14" t="n">
         <v>2.68</v>
       </c>
-      <c r="J10" s="12" t="n">
+      <c r="J10" s="14" t="n">
         <v>2.66</v>
       </c>
-      <c r="K10" s="12" t="n">
+      <c r="K10" s="14" t="n">
         <v>6.56</v>
       </c>
-      <c r="L10" s="12" t="n">
+      <c r="L10" s="14" t="n">
         <v>7.54</v>
       </c>
-      <c r="N10" s="12" t="n">
+      <c r="N10" s="14" t="n">
         <v>93.31</v>
       </c>
-      <c r="O10" s="12" t="n">
+      <c r="O10" s="14" t="n">
         <v>-139.65</v>
       </c>
-      <c r="P10" s="12" t="n">
+      <c r="P10" s="14" t="n">
         <v>1.64</v>
       </c>
-      <c r="Q10" s="12" t="n">
+      <c r="Q10" s="14" t="n">
         <v>-0.37</v>
       </c>
+      <c r="S10" s="14" t="n">
+        <v>5.18</v>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="n">
+      <c r="A11" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="12" t="n">
+      <c r="B11" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>[Ir(dFppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E11" s="12" t="n">
+      <c r="E11" s="14" t="n">
         <v>63.94</v>
       </c>
-      <c r="G11" s="12" t="n">
+      <c r="G11" s="14" t="n">
         <v>8.31</v>
       </c>
-      <c r="H11" s="12" t="n">
+      <c r="H11" s="14" t="n">
         <v>7.94</v>
       </c>
-      <c r="I11" s="12" t="n">
+      <c r="I11" s="14" t="n">
         <v>2.55</v>
       </c>
-      <c r="J11" s="12" t="n">
+      <c r="J11" s="14" t="n">
         <v>2.44</v>
       </c>
-      <c r="K11" s="12" t="n">
+      <c r="K11" s="14" t="n">
         <v>6.02</v>
       </c>
-      <c r="L11" s="12" t="n">
+      <c r="L11" s="14" t="n">
         <v>6.05</v>
       </c>
-      <c r="N11" s="12" t="n">
+      <c r="N11" s="14" t="n">
         <v>77.48999999999999</v>
       </c>
-      <c r="O11" s="12" t="n">
+      <c r="O11" s="14" t="n">
         <v>-132.44</v>
       </c>
-      <c r="P11" s="12" t="n">
+      <c r="P11" s="14" t="n">
         <v>1.32</v>
       </c>
-      <c r="Q11" s="12" t="n">
+      <c r="Q11" s="14" t="n">
         <v>-1.06</v>
       </c>
+      <c r="S11" s="14" t="n">
+        <v>5.21</v>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="n">
+      <c r="A12" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(Me)ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E12" s="12" t="n">
+      <c r="E12" s="14" t="n">
         <v>63.38</v>
       </c>
-      <c r="G12" s="12" t="n">
+      <c r="G12" s="14" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="H12" s="12" t="n">
+      <c r="H12" s="14" t="n">
         <v>7.88</v>
       </c>
-      <c r="I12" s="12" t="n">
+      <c r="I12" s="14" t="n">
         <v>2.51</v>
       </c>
-      <c r="J12" s="12" t="n">
+      <c r="J12" s="14" t="n">
         <v>2.44</v>
       </c>
-      <c r="K12" s="12" t="n">
+      <c r="K12" s="14" t="n">
         <v>6.01</v>
       </c>
-      <c r="L12" s="12" t="n">
+      <c r="L12" s="14" t="n">
         <v>6.01</v>
       </c>
-      <c r="N12" s="12" t="n">
+      <c r="N12" s="14" t="n">
         <v>77.14</v>
       </c>
-      <c r="O12" s="12" t="n">
+      <c r="O12" s="14" t="n">
         <v>-131.45</v>
       </c>
-      <c r="P12" s="12" t="n">
+      <c r="P12" s="14" t="n">
         <v>1.28</v>
       </c>
-      <c r="Q12" s="12" t="n">
+      <c r="Q12" s="14" t="n">
         <v>-1.07</v>
       </c>
+      <c r="S12" s="14" t="n">
+        <v>5.3</v>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="n">
+      <c r="A13" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(CF3)ppy)2(bpy)]PF6</t>
         </is>
       </c>
-      <c r="E13" s="12" t="n">
+      <c r="E13" s="14" t="n">
         <v>65.67</v>
       </c>
-      <c r="G13" s="12" t="n">
+      <c r="G13" s="14" t="n">
         <v>10.34</v>
       </c>
-      <c r="H13" s="12" t="n">
+      <c r="H13" s="14" t="n">
         <v>8.75</v>
       </c>
-      <c r="I13" s="12" t="n">
+      <c r="I13" s="14" t="n">
         <v>2.6</v>
       </c>
-      <c r="J13" s="12" t="n">
+      <c r="J13" s="14" t="n">
         <v>2.5</v>
       </c>
-      <c r="K13" s="12" t="n">
+      <c r="K13" s="14" t="n">
         <v>5.97</v>
       </c>
-      <c r="L13" s="12" t="n">
+      <c r="L13" s="14" t="n">
         <v>6.04</v>
       </c>
-      <c r="N13" s="12" t="n">
+      <c r="N13" s="14" t="n">
         <v>79.73</v>
       </c>
-      <c r="O13" s="12" t="n">
+      <c r="O13" s="14" t="n">
         <v>-137.69</v>
       </c>
-      <c r="P13" s="12" t="n">
+      <c r="P13" s="14" t="n">
         <v>1.55</v>
       </c>
-      <c r="Q13" s="12" t="n">
+      <c r="Q13" s="14" t="n">
         <v>-0.96</v>
       </c>
+      <c r="S13" s="14" t="n">
+        <v>4.99</v>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="n">
+      <c r="A14" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C14" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(Me)ppy)2(d(5,5)CH3bpy)]PF6</t>
         </is>
       </c>
-      <c r="E14" s="12" t="n">
+      <c r="E14" s="14" t="n">
         <v>65.70999999999999</v>
       </c>
-      <c r="G14" s="12" t="n">
+      <c r="G14" s="14" t="n">
         <v>13.55</v>
       </c>
-      <c r="H14" s="12" t="n">
+      <c r="H14" s="14" t="n">
         <v>12.58</v>
       </c>
-      <c r="I14" s="12" t="n">
+      <c r="I14" s="14" t="n">
         <v>2.48</v>
       </c>
-      <c r="J14" s="12" t="n">
+      <c r="J14" s="14" t="n">
         <v>2.43</v>
       </c>
-      <c r="K14" s="12" t="n">
+      <c r="K14" s="14" t="n">
         <v>5.65</v>
       </c>
-      <c r="L14" s="12" t="n">
+      <c r="L14" s="14" t="n">
         <v>5.61</v>
       </c>
-      <c r="N14" s="12" t="n">
+      <c r="N14" s="14" t="n">
         <v>75.04000000000001</v>
       </c>
-      <c r="O14" s="12" t="n">
+      <c r="O14" s="14" t="n">
         <v>-132.46</v>
       </c>
-      <c r="P14" s="12" t="n">
+      <c r="P14" s="14" t="n">
         <v>1.32</v>
       </c>
-      <c r="Q14" s="12" t="n">
+      <c r="Q14" s="14" t="n">
         <v>-1.17</v>
       </c>
+      <c r="S14" s="14" t="n">
+        <v>5.01</v>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="n">
+      <c r="A15" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="C15" s="14" t="inlineStr">
         <is>
           <t>[Ir(tCF3ppy)2(d(5,5)CH3bpy)]PF6</t>
         </is>
       </c>
-      <c r="E15" s="12" t="n">
+      <c r="E15" s="14" t="n">
         <v>59.39</v>
       </c>
-      <c r="G15" s="12" t="n">
+      <c r="G15" s="14" t="n">
         <v>11.39</v>
       </c>
-      <c r="H15" s="12" t="n">
+      <c r="H15" s="14" t="n">
         <v>9.220000000000001</v>
       </c>
-      <c r="I15" s="12" t="n">
+      <c r="I15" s="14" t="n">
         <v>2.21</v>
       </c>
-      <c r="J15" s="12" t="n">
+      <c r="J15" s="14" t="n">
         <v>2.05</v>
       </c>
-      <c r="K15" s="12" t="n">
+      <c r="K15" s="14" t="n">
         <v>5.71</v>
       </c>
-      <c r="L15" s="12" t="n">
+      <c r="L15" s="14" t="n">
         <v>5.77</v>
       </c>
-      <c r="N15" s="12" t="n">
+      <c r="N15" s="14" t="n">
         <v>88.05</v>
       </c>
-      <c r="O15" s="12" t="n">
+      <c r="O15" s="14" t="n">
         <v>-128.12</v>
       </c>
-      <c r="P15" s="12" t="n">
+      <c r="P15" s="14" t="n">
         <v>1.14</v>
       </c>
-      <c r="Q15" s="12" t="n">
+      <c r="Q15" s="14" t="n">
         <v>-0.6</v>
       </c>
+      <c r="S15" s="14" t="n">
+        <v>5.39</v>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="n">
+      <c r="A16" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="12" t="n">
+      <c r="B16" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C16" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(Me)ppy)2(d(OMe)bpy)]PF6</t>
         </is>
       </c>
-      <c r="E16" s="12" t="n">
+      <c r="E16" s="14" t="n">
         <v>65.73999999999999</v>
       </c>
-      <c r="G16" s="12" t="n">
+      <c r="G16" s="14" t="n">
         <v>13.47</v>
       </c>
-      <c r="H16" s="12" t="n">
+      <c r="H16" s="14" t="n">
         <v>13.08</v>
       </c>
-      <c r="I16" s="12" t="n">
+      <c r="I16" s="14" t="n">
         <v>2.53</v>
       </c>
-      <c r="J16" s="12" t="n">
+      <c r="J16" s="14" t="n">
         <v>2.41</v>
       </c>
-      <c r="K16" s="12" t="n">
+      <c r="K16" s="14" t="n">
         <v>6.88</v>
       </c>
-      <c r="L16" s="12" t="n">
+      <c r="L16" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="N16" s="12" t="n">
+      <c r="N16" s="14" t="n">
         <v>73.91</v>
       </c>
-      <c r="O16" s="12" t="n">
+      <c r="O16" s="14" t="n">
         <v>-131.74</v>
       </c>
-      <c r="P16" s="12" t="n">
+      <c r="P16" s="14" t="n">
         <v>1.29</v>
       </c>
-      <c r="Q16" s="12" t="n">
+      <c r="Q16" s="14" t="n">
         <v>-1.22</v>
       </c>
+      <c r="S16" s="14" t="n">
+        <v>5.06</v>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="n">
+      <c r="A17" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="12" t="n">
+      <c r="B17" s="14" t="n">
         <v>17</v>
       </c>
-      <c r="C17" s="12" t="inlineStr">
+      <c r="C17" s="14" t="inlineStr">
         <is>
           <t>[Ir(ppy)2(d(OMe)bpy)]PF6</t>
         </is>
       </c>
-      <c r="E17" s="12" t="n">
+      <c r="E17" s="14" t="n">
         <v>59.92</v>
       </c>
-      <c r="G17" s="12" t="n">
+      <c r="G17" s="14" t="n">
         <v>9.140000000000001</v>
       </c>
-      <c r="H17" s="12" t="n">
+      <c r="H17" s="14" t="n">
         <v>9.02</v>
       </c>
-      <c r="I17" s="12" t="n">
+      <c r="I17" s="14" t="n">
         <v>2.82</v>
       </c>
-      <c r="J17" s="12" t="n">
+      <c r="J17" s="14" t="n">
         <v>2.86</v>
       </c>
-      <c r="K17" s="12" t="n">
+      <c r="K17" s="14" t="n">
         <v>6.86</v>
       </c>
-      <c r="L17" s="12" t="n">
+      <c r="L17" s="14" t="n">
         <v>6.97</v>
       </c>
-      <c r="N17" s="12" t="n">
+      <c r="N17" s="14" t="n">
         <v>72.40000000000001</v>
       </c>
-      <c r="O17" s="12" t="n">
+      <c r="O17" s="14" t="n">
         <v>-125.16</v>
       </c>
-      <c r="P17" s="12" t="n">
+      <c r="P17" s="14" t="n">
         <v>1.01</v>
       </c>
-      <c r="Q17" s="12" t="n">
+      <c r="Q17" s="14" t="n">
         <v>-1.28</v>
       </c>
+      <c r="S17" s="14" t="n">
+        <v>4.9</v>
+      </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="n">
+      <c r="A18" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="12" t="n">
+      <c r="B18" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>[Ir(tCF3ppy)2(d(5,5)OMebpy)]PF6</t>
         </is>
       </c>
-      <c r="E18" s="12" t="n">
+      <c r="E18" s="14" t="n">
         <v>59.14</v>
       </c>
-      <c r="G18" s="12" t="n">
+      <c r="G18" s="14" t="n">
         <v>10.9</v>
       </c>
-      <c r="H18" s="12" t="n">
+      <c r="H18" s="14" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="I18" s="12" t="n">
+      <c r="I18" s="14" t="n">
         <v>1.79</v>
       </c>
-      <c r="J18" s="12" t="n">
+      <c r="J18" s="14" t="n">
         <v>2.23</v>
       </c>
-      <c r="K18" s="12" t="n">
+      <c r="K18" s="14" t="n">
         <v>6.28</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="L18" s="14" t="n">
         <v>6.15</v>
       </c>
-      <c r="N18" s="12" t="n">
+      <c r="N18" s="14" t="n">
         <v>88.68000000000001</v>
       </c>
-      <c r="O18" s="12" t="n">
+      <c r="O18" s="14" t="n">
         <v>-133.2</v>
       </c>
-      <c r="P18" s="12" t="n">
+      <c r="P18" s="14" t="n">
         <v>1.36</v>
       </c>
-      <c r="Q18" s="12" t="n">
+      <c r="Q18" s="14" t="n">
         <v>-0.57</v>
       </c>
+      <c r="S18" s="14" t="n">
+        <v>5.44</v>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="n">
+      <c r="A19" s="14" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="12" t="n">
+      <c r="B19" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="C19" s="12" t="inlineStr">
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>[Ir(dCF3ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E19" s="12" t="n">
+      <c r="E19" s="14" t="n">
         <v>60.55</v>
       </c>
-      <c r="G19" s="12" t="n">
+      <c r="G19" s="14" t="n">
         <v>13.24</v>
       </c>
-      <c r="H19" s="12" t="n">
+      <c r="H19" s="14" t="n">
         <v>10.81</v>
       </c>
-      <c r="I19" s="12" t="n">
+      <c r="I19" s="14" t="n">
         <v>1.99</v>
       </c>
-      <c r="J19" s="12" t="n">
+      <c r="J19" s="14" t="n">
         <v>2.11</v>
       </c>
-      <c r="K19" s="12" t="n">
+      <c r="K19" s="14" t="n">
         <v>6.3</v>
       </c>
-      <c r="L19" s="12" t="n">
+      <c r="L19" s="14" t="n">
         <v>6.41</v>
       </c>
-      <c r="N19" s="12" t="n">
+      <c r="N19" s="14" t="n">
         <v>83.55</v>
       </c>
-      <c r="O19" s="12" t="n">
+      <c r="O19" s="14" t="n">
         <v>-127.03</v>
       </c>
-      <c r="P19" s="12" t="n">
+      <c r="P19" s="14" t="n">
         <v>1.09</v>
       </c>
-      <c r="Q19" s="12" t="n">
+      <c r="Q19" s="14" t="n">
         <v>-0.8</v>
       </c>
+      <c r="S19" s="14" t="n">
+        <v>5.49</v>
+      </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="n">
+      <c r="A20" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="12" t="n">
+      <c r="B20" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C20" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(6-OMe)ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E20" s="12" t="n">
+      <c r="E20" s="14" t="n">
         <v>64.83</v>
       </c>
-      <c r="G20" s="12" t="n">
+      <c r="G20" s="14" t="n">
         <v>12.7</v>
       </c>
-      <c r="H20" s="12" t="n">
+      <c r="H20" s="14" t="n">
         <v>11.75</v>
       </c>
-      <c r="I20" s="12" t="n">
+      <c r="I20" s="14" t="n">
         <v>2.57</v>
       </c>
-      <c r="J20" s="12" t="n">
+      <c r="J20" s="14" t="n">
         <v>2.45</v>
       </c>
-      <c r="K20" s="12" t="n">
+      <c r="K20" s="14" t="n">
         <v>6.01</v>
       </c>
-      <c r="L20" s="12" t="n">
+      <c r="L20" s="14" t="n">
         <v>6.08</v>
       </c>
-      <c r="N20" s="12" t="n">
+      <c r="N20" s="14" t="n">
         <v>73.62</v>
       </c>
-      <c r="O20" s="12" t="n">
+      <c r="O20" s="14" t="n">
         <v>-129.39</v>
       </c>
-      <c r="P20" s="12" t="n">
+      <c r="P20" s="14" t="n">
         <v>1.19</v>
       </c>
-      <c r="Q20" s="12" t="n">
+      <c r="Q20" s="14" t="n">
         <v>-1.23</v>
       </c>
+      <c r="S20" s="14" t="n">
+        <v>5.35</v>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="n">
+      <c r="A21" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="12" t="n">
+      <c r="B21" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="C21" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(OMe)ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E21" s="12" t="n">
+      <c r="E21" s="14" t="n">
         <v>63.27</v>
       </c>
-      <c r="G21" s="12" t="n">
+      <c r="G21" s="14" t="n">
         <v>12.88</v>
       </c>
-      <c r="H21" s="12" t="n">
+      <c r="H21" s="14" t="n">
         <v>10.57</v>
       </c>
-      <c r="I21" s="12" t="n">
+      <c r="I21" s="14" t="n">
         <v>2.65</v>
       </c>
-      <c r="J21" s="12" t="n">
+      <c r="J21" s="14" t="n">
         <v>2.66</v>
       </c>
-      <c r="K21" s="12" t="n">
+      <c r="K21" s="14" t="n">
         <v>6.04</v>
       </c>
-      <c r="L21" s="12" t="n">
+      <c r="L21" s="14" t="n">
         <v>6.08</v>
       </c>
-      <c r="N21" s="12" t="n">
+      <c r="N21" s="14" t="n">
         <v>76.45</v>
       </c>
-      <c r="O21" s="12" t="n">
+      <c r="O21" s="14" t="n">
         <v>-131.55</v>
       </c>
-      <c r="P21" s="12" t="n">
+      <c r="P21" s="14" t="n">
         <v>1.28</v>
       </c>
-      <c r="Q21" s="12" t="n">
+      <c r="Q21" s="14" t="n">
         <v>-1.1</v>
       </c>
+      <c r="S21" s="14" t="n">
+        <v>5.35</v>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="n">
+      <c r="A22" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="12" t="n">
+      <c r="B22" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C22" s="14" t="inlineStr">
         <is>
           <t>[Ir(tCF3ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E22" s="12" t="n">
+      <c r="E22" s="14" t="n">
         <v>59.81</v>
       </c>
-      <c r="G22" s="12" t="n">
+      <c r="G22" s="14" t="n">
         <v>11.09</v>
       </c>
-      <c r="H22" s="12" t="n">
+      <c r="H22" s="14" t="n">
         <v>8.85</v>
       </c>
-      <c r="I22" s="12" t="n">
+      <c r="I22" s="14" t="n">
         <v>2.46</v>
       </c>
-      <c r="J22" s="12" t="n">
+      <c r="J22" s="14" t="n">
         <v>1.9</v>
       </c>
-      <c r="K22" s="12" t="n">
+      <c r="K22" s="14" t="n">
         <v>6.41</v>
       </c>
-      <c r="L22" s="12" t="n">
+      <c r="L22" s="14" t="n">
         <v>6.05</v>
       </c>
-      <c r="N22" s="12" t="n">
+      <c r="N22" s="14" t="n">
         <v>87.42</v>
       </c>
-      <c r="O22" s="12" t="n">
+      <c r="O22" s="14" t="n">
         <v>-129.41</v>
       </c>
-      <c r="P22" s="12" t="n">
+      <c r="P22" s="14" t="n">
         <v>1.19</v>
       </c>
-      <c r="Q22" s="12" t="n">
+      <c r="Q22" s="14" t="n">
         <v>-0.63</v>
       </c>
+      <c r="S22" s="14" t="n">
+        <v>5.65</v>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="n">
+      <c r="A23" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="B23" s="12" t="n">
+      <c r="B23" s="14" t="n">
         <v>23</v>
       </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="C23" s="14" t="inlineStr">
         <is>
           <t>[Ir(tetraFppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E23" s="12" t="n">
+      <c r="E23" s="14" t="n">
         <v>66.11</v>
       </c>
-      <c r="G23" s="12" t="n">
+      <c r="G23" s="14" t="n">
         <v>8.119999999999999</v>
       </c>
-      <c r="H23" s="12" t="n">
+      <c r="H23" s="14" t="n">
         <v>8.300000000000001</v>
       </c>
-      <c r="I23" s="12" t="n">
+      <c r="I23" s="14" t="n">
         <v>2.8</v>
       </c>
-      <c r="J23" s="12" t="n">
+      <c r="J23" s="14" t="n">
         <v>3.11</v>
       </c>
-      <c r="K23" s="12" t="n">
+      <c r="K23" s="14" t="n">
         <v>6.04</v>
       </c>
-      <c r="L23" s="12" t="n">
+      <c r="L23" s="14" t="n">
         <v>6.08</v>
       </c>
-      <c r="N23" s="12" t="n">
+      <c r="N23" s="14" t="n">
         <v>78.63</v>
       </c>
-      <c r="O23" s="12" t="n">
+      <c r="O23" s="14" t="n">
         <v>-136.34</v>
       </c>
-      <c r="P23" s="12" t="n">
+      <c r="P23" s="14" t="n">
         <v>1.49</v>
       </c>
-      <c r="Q23" s="12" t="n">
+      <c r="Q23" s="14" t="n">
         <v>-1.01</v>
       </c>
+      <c r="S23" s="14" t="n">
+        <v>5.26</v>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="n">
+      <c r="A24" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="B24" s="12" t="n">
+      <c r="B24" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C24" s="14" t="inlineStr">
         <is>
           <t>[Ir(d(OMe)ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E24" s="12" t="n">
+      <c r="E24" s="14" t="n">
         <v>59.01</v>
       </c>
-      <c r="G24" s="12" t="n">
+      <c r="G24" s="14" t="n">
         <v>8.289999999999999</v>
       </c>
-      <c r="H24" s="12" t="n">
+      <c r="H24" s="14" t="n">
         <v>7.93</v>
       </c>
-      <c r="I24" s="12" t="n">
+      <c r="I24" s="14" t="n">
         <v>2.54</v>
       </c>
-      <c r="J24" s="12" t="n">
+      <c r="J24" s="14" t="n">
         <v>2.53</v>
       </c>
-      <c r="K24" s="12" t="n">
+      <c r="K24" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="L24" s="12" t="n">
+      <c r="L24" s="14" t="n">
         <v>6.01</v>
       </c>
-      <c r="N24" s="12" t="n">
+      <c r="N24" s="14" t="n">
         <v>74.41</v>
       </c>
-      <c r="O24" s="12" t="n">
+      <c r="O24" s="14" t="n">
         <v>-125.22</v>
       </c>
-      <c r="P24" s="12" t="n">
+      <c r="P24" s="14" t="n">
         <v>1.01</v>
       </c>
-      <c r="Q24" s="12" t="n">
+      <c r="Q24" s="14" t="n">
         <v>-1.19</v>
       </c>
+      <c r="S24" s="14" t="n">
+        <v>5.43</v>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="n">
+      <c r="A25" s="14" t="n">
         <v>23</v>
       </c>
-      <c r="B25" s="12" t="n">
+      <c r="B25" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C25" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(4-Me)ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E25" s="12" t="n">
+      <c r="E25" s="14" t="n">
         <v>64.62</v>
       </c>
-      <c r="G25" s="12" t="n">
+      <c r="G25" s="14" t="n">
         <v>8.42</v>
       </c>
-      <c r="H25" s="12" t="n">
+      <c r="H25" s="14" t="n">
         <v>8.039999999999999</v>
       </c>
-      <c r="I25" s="12" t="n">
+      <c r="I25" s="14" t="n">
         <v>2.59</v>
       </c>
-      <c r="J25" s="12" t="n">
+      <c r="J25" s="14" t="n">
         <v>2.43</v>
       </c>
-      <c r="K25" s="12" t="n">
+      <c r="K25" s="14" t="n">
         <v>6.18</v>
       </c>
-      <c r="L25" s="12" t="n">
+      <c r="L25" s="14" t="n">
         <v>6.12</v>
       </c>
-      <c r="N25" s="12" t="n">
+      <c r="N25" s="14" t="n">
         <v>75.92</v>
       </c>
-      <c r="O25" s="12" t="n">
+      <c r="O25" s="14" t="n">
         <v>-131.37</v>
       </c>
-      <c r="P25" s="12" t="n">
+      <c r="P25" s="14" t="n">
         <v>1.28</v>
       </c>
-      <c r="Q25" s="12" t="n">
+      <c r="Q25" s="14" t="n">
         <v>-1.13</v>
       </c>
+      <c r="S25" s="14" t="n">
+        <v>5.3</v>
+      </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="n">
+      <c r="A26" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="B26" s="12" t="n">
+      <c r="B26" s="14" t="n">
         <v>27</v>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="C26" s="14" t="inlineStr">
         <is>
           <t>[Ir(ppy)2(phen)]PF6</t>
         </is>
       </c>
-      <c r="E26" s="12" t="n">
+      <c r="E26" s="14" t="n">
         <v>57.55</v>
       </c>
-      <c r="G26" s="12" t="n">
+      <c r="G26" s="14" t="n">
         <v>7.93</v>
       </c>
-      <c r="H26" s="12" t="n">
+      <c r="H26" s="14" t="n">
         <v>7.58</v>
       </c>
-      <c r="I26" s="12" t="n">
+      <c r="I26" s="14" t="n">
         <v>2.78</v>
       </c>
-      <c r="J26" s="12" t="n">
+      <c r="J26" s="14" t="n">
         <v>2.83</v>
       </c>
-      <c r="K26" s="12" t="n">
+      <c r="K26" s="14" t="n">
         <v>5.11</v>
       </c>
-      <c r="L26" s="12" t="n">
+      <c r="L26" s="14" t="n">
         <v>5.06</v>
       </c>
-      <c r="N26" s="12" t="n">
+      <c r="N26" s="14" t="n">
         <v>76.25</v>
       </c>
-      <c r="O26" s="12" t="n">
+      <c r="O26" s="14" t="n">
         <v>-125.75</v>
       </c>
-      <c r="P26" s="12" t="n">
+      <c r="P26" s="14" t="n">
         <v>1.03</v>
       </c>
-      <c r="Q26" s="12" t="n">
+      <c r="Q26" s="14" t="n">
         <v>-1.11</v>
       </c>
+      <c r="S26" s="14" t="n">
+        <v>4.78</v>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="n">
+      <c r="A27" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="B27" s="12" t="n">
+      <c r="B27" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="C27" s="12" t="inlineStr">
+      <c r="C27" s="14" t="inlineStr">
         <is>
           <t>[Ir(CF3-pmb)3]</t>
         </is>
       </c>
-      <c r="E27" s="12" t="n">
+      <c r="E27" s="14" t="n">
         <v>73.23</v>
       </c>
-      <c r="G27" s="12" t="n">
+      <c r="G27" s="14" t="n">
         <v>14.36</v>
       </c>
-      <c r="H27" s="12" t="n">
+      <c r="H27" s="14" t="n">
         <v>13.69</v>
       </c>
-      <c r="I27" s="12" t="n">
+      <c r="I27" s="14" t="n">
         <v>6.64</v>
       </c>
-      <c r="J27" s="12" t="n">
+      <c r="J27" s="14" t="n">
         <v>4.99</v>
       </c>
-      <c r="K27" s="12" t="n">
+      <c r="K27" s="14" t="n">
         <v>8.81</v>
       </c>
-      <c r="L27" s="12" t="n">
+      <c r="L27" s="14" t="n">
         <v>5.85</v>
       </c>
-      <c r="N27" s="12" t="n">
+      <c r="N27" s="14" t="n">
         <v>53.51</v>
       </c>
-      <c r="O27" s="12" t="n">
+      <c r="O27" s="14" t="n">
         <v>-107.29</v>
       </c>
-      <c r="P27" s="12" t="n">
+      <c r="P27" s="14" t="n">
         <v>0.23</v>
       </c>
-      <c r="Q27" s="12" t="n">
+      <c r="Q27" s="14" t="n">
         <v>-2.1</v>
       </c>
+      <c r="S27" s="14" t="n">
+        <v>5.43</v>
+      </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="n">
+      <c r="A28" s="14" t="n">
         <v>26</v>
       </c>
-      <c r="B28" s="12" t="n">
+      <c r="B28" s="14" t="n">
         <v>28</v>
       </c>
-      <c r="C28" s="12" t="inlineStr">
+      <c r="C28" s="14" t="inlineStr">
         <is>
           <t>[Ir(CH3-pmb)3]</t>
         </is>
       </c>
-      <c r="E28" s="12" t="n">
+      <c r="E28" s="14" t="n">
         <v>76.81999999999999</v>
       </c>
-      <c r="G28" s="12" t="n">
+      <c r="G28" s="14" t="n">
         <v>19.11</v>
       </c>
-      <c r="H28" s="12" t="n">
+      <c r="H28" s="14" t="n">
         <v>13.66</v>
       </c>
-      <c r="I28" s="12" t="n">
+      <c r="I28" s="14" t="n">
         <v>2.86</v>
       </c>
-      <c r="J28" s="12" t="n">
+      <c r="J28" s="14" t="n">
         <v>2.1</v>
       </c>
-      <c r="K28" s="12" t="n">
+      <c r="K28" s="14" t="n">
         <v>5.2</v>
       </c>
-      <c r="L28" s="12" t="n">
+      <c r="L28" s="14" t="n">
         <v>4.44</v>
       </c>
-      <c r="N28" s="12" t="n">
+      <c r="N28" s="14" t="n">
         <v>48.79</v>
       </c>
-      <c r="O28" s="12" t="n">
+      <c r="O28" s="14" t="n">
         <v>-109.67</v>
       </c>
-      <c r="P28" s="12" t="n">
+      <c r="P28" s="14" t="n">
         <v>0.34</v>
       </c>
-      <c r="Q28" s="12" t="n">
+      <c r="Q28" s="14" t="n">
         <v>-2.3</v>
       </c>
+      <c r="S28" s="14" t="n">
+        <v>5.31</v>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="n">
+      <c r="A29" s="14" t="n">
         <v>27</v>
       </c>
-      <c r="B29" s="12" t="n">
+      <c r="B29" s="14" t="n">
         <v>29</v>
       </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="C29" s="14" t="inlineStr">
         <is>
           <t>[Ir(pmb)3]</t>
         </is>
       </c>
-      <c r="E29" s="12" t="n">
+      <c r="E29" s="14" t="n">
         <v>79.87</v>
       </c>
-      <c r="G29" s="12" t="n">
+      <c r="G29" s="14" t="n">
         <v>34.95</v>
       </c>
-      <c r="H29" s="12" t="n">
+      <c r="H29" s="14" t="n">
         <v>14.5</v>
       </c>
-      <c r="I29" s="12" t="n">
+      <c r="I29" s="14" t="n">
         <v>2.97</v>
       </c>
-      <c r="J29" s="12" t="n">
+      <c r="J29" s="14" t="n">
         <v>2.02</v>
       </c>
-      <c r="K29" s="12" t="n">
+      <c r="K29" s="14" t="n">
         <v>5.18</v>
       </c>
-      <c r="L29" s="12" t="n">
+      <c r="L29" s="14" t="n">
         <v>4.42</v>
       </c>
-      <c r="N29" s="12" t="n">
+      <c r="N29" s="14" t="n">
         <v>47.39</v>
       </c>
-      <c r="O29" s="12" t="n">
+      <c r="O29" s="14" t="n">
         <v>-112.97</v>
       </c>
-      <c r="P29" s="12" t="n">
+      <c r="P29" s="14" t="n">
         <v>0.48</v>
       </c>
-      <c r="Q29" s="12" t="n">
+      <c r="Q29" s="14" t="n">
         <v>-2.37</v>
+      </c>
+      <c r="S29" s="14" t="n">
+        <v>5.17</v>
       </c>
     </row>
   </sheetData>
@@ -1867,7 +1971,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -1878,448 +1982,475 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="13" t="inlineStr">
+      <c r="A1" s="15" t="inlineStr">
         <is>
           <t>Block</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="B1" s="15" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
+      <c r="C1" s="15" t="inlineStr">
         <is>
           <t>Unit</t>
         </is>
       </c>
-      <c r="D1" s="13" t="inlineStr">
+      <c r="D1" s="15" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
       </c>
-      <c r="E1" s="13" t="inlineStr">
+      <c r="E1" s="15" t="inlineStr">
         <is>
           <t>Taken from</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="14" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Identity</t>
         </is>
       </c>
-      <c r="B2" s="14" t="inlineStr">
+      <c r="B2" s="16" t="inlineStr">
         <is>
           <t>new_id</t>
         </is>
       </c>
-      <c r="C2" s="14" t="inlineStr"/>
-      <c r="D2" s="15" t="inlineStr">
+      <c r="C2" s="16" t="inlineStr"/>
+      <c r="D2" s="17" t="inlineStr">
         <is>
           <t>PC number used downstream and in the paper, 1-27.</t>
         </is>
       </c>
-      <c r="E2" s="14" t="inlineStr">
+      <c r="E2" s="16" t="inlineStr">
         <is>
           <t>compound_identification.xlsx: Photocatalysts/new_id</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="inlineStr">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Identity</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>old_id</t>
         </is>
       </c>
-      <c r="C3" s="14" t="inlineStr"/>
-      <c r="D3" s="15" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr"/>
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>PC number during the screen, used by the raw files.</t>
         </is>
       </c>
-      <c r="E3" s="14" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: pc_id</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="14" t="inlineStr">
+      <c r="A4" s="16" t="inlineStr">
         <is>
           <t>Identity</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
         <is>
           <t>compound</t>
         </is>
       </c>
-      <c r="C4" s="14" t="inlineStr"/>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="C4" s="16" t="inlineStr"/>
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>Compound.</t>
         </is>
       </c>
-      <c r="E4" s="14" t="inlineStr">
+      <c r="E4" s="16" t="inlineStr">
         <is>
           <t>compound_identification.xlsx: Photocatalysts/name</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="14" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Triplet energy / kcal mol-1</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
         <is>
           <t>E_T / kcal mol-1</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="C5" s="16" t="inlineStr">
         <is>
           <t>kcal mol-1</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>Adiabatic, Gibbs-corrected: ((E_T1 + G_T1) - (E_S0 + G_S0)) x 627.509.</t>
         </is>
       </c>
-      <c r="E5" s="14" t="inlineStr">
+      <c r="E5" s="16" t="inlineStr">
         <is>
           <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: E_T / kcal mol-1</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="14" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Reorganization energies / kcal mol-1</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>lambda_S0_T1 / kcal mol-1</t>
         </is>
       </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="C6" s="16" t="inlineStr">
         <is>
           <t>kcal mol-1</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="D6" s="17" t="inlineStr">
         <is>
           <t>S0 surface: E_S0 at the T1 geometry minus E_S0 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
-      <c r="E6" s="14" t="inlineStr">
+      <c r="E6" s="16" t="inlineStr">
         <is>
           <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_S0_T1 / kcal mol-1</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="14" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Reorganization energies / kcal mol-1</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
         <is>
           <t>lambda_T1_S0 / kcal mol-1</t>
         </is>
       </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="C7" s="16" t="inlineStr">
         <is>
           <t>kcal mol-1</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>T1 surface: E_T1 at the S0 geometry minus E_T1 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
-      <c r="E7" s="14" t="inlineStr">
+      <c r="E7" s="16" t="inlineStr">
         <is>
           <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_T1_S0 / kcal mol-1</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="14" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Reorganization energies / kcal mol-1</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
         <is>
           <t>lambda_S0_Dplus / kcal mol-1</t>
         </is>
       </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="C8" s="16" t="inlineStr">
         <is>
           <t>kcal mol-1</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="D8" s="17" t="inlineStr">
         <is>
           <t>S0 surface: E_S0 at the Dplus geometry minus E_S0 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
-      <c r="E8" s="14" t="inlineStr">
+      <c r="E8" s="16" t="inlineStr">
         <is>
           <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_S0_Dplus / kcal mol-1</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="14" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>Reorganization energies / kcal mol-1</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
         <is>
           <t>lambda_Dplus_S0 / kcal mol-1</t>
         </is>
       </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="C9" s="16" t="inlineStr">
         <is>
           <t>kcal mol-1</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>Dplus surface: E_Dplus at the S0 geometry minus E_Dplus at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
-      <c r="E9" s="14" t="inlineStr">
+      <c r="E9" s="16" t="inlineStr">
         <is>
           <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_Dplus_S0 / kcal mol-1</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Reorganization energies / kcal mol-1</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
         <is>
           <t>lambda_S0_Dminus / kcal mol-1</t>
         </is>
       </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="C10" s="16" t="inlineStr">
         <is>
           <t>kcal mol-1</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>S0 surface: E_S0 at the Dminus geometry minus E_S0 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
-      <c r="E10" s="14" t="inlineStr">
+      <c r="E10" s="16" t="inlineStr">
         <is>
           <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_S0_Dminus / kcal mol-1</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>Reorganization energies / kcal mol-1</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
         <is>
           <t>lambda_Dminus_S0 / kcal mol-1</t>
         </is>
       </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="C11" s="16" t="inlineStr">
         <is>
           <t>kcal mol-1</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>Dminus surface: E_Dminus at the S0 geometry minus E_Dminus at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
-      <c r="E11" s="14" t="inlineStr">
+      <c r="E11" s="16" t="inlineStr">
         <is>
           <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_Dminus_S0 / kcal mol-1</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>Excited-state redox / kcal mol-1 and V vs SCE</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
         <is>
           <t>dG_ox_ES / kcal mol-1</t>
         </is>
       </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="C12" s="16" t="inlineStr">
         <is>
           <t>kcal mol-1</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>PC* -&gt; PC+: ((E_ox + G_ox) - (E_T1 + G_T1)) x 627.509.</t>
         </is>
       </c>
-      <c r="E12" s="14" t="inlineStr">
+      <c r="E12" s="16" t="inlineStr">
         <is>
           <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: dG_ox_ES / kcal mol-1</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>Excited-state redox / kcal mol-1 and V vs SCE</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
         <is>
           <t>dG_red_ES / kcal mol-1</t>
         </is>
       </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="C13" s="16" t="inlineStr">
         <is>
           <t>kcal mol-1</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>PC* -&gt; PC-: ((E_red + G_red) - (E_T1 + G_T1)) x 627.509.</t>
         </is>
       </c>
-      <c r="E13" s="14" t="inlineStr">
+      <c r="E13" s="16" t="inlineStr">
         <is>
           <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: dG_red_ES / kcal mol-1</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>Excited-state redox / kcal mol-1 and V vs SCE</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
         <is>
           <t>E_PCstar_PCminus / V</t>
         </is>
       </c>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="C14" s="16" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>PC*/PC-, how strong an oxidant the triplet is: -dG_red_ES / 23.061 - 4.42.</t>
         </is>
       </c>
-      <c r="E14" s="14" t="inlineStr">
+      <c r="E14" s="16" t="inlineStr">
         <is>
           <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: E_PCstar_PCminus / V</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>Excited-state redox / kcal mol-1 and V vs SCE</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
         <is>
           <t>E_PCplus_PCstar / V</t>
         </is>
       </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="C15" s="16" t="inlineStr">
         <is>
           <t>V</t>
         </is>
       </c>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>PC+/PC*, how strong a reductant the triplet is: dG_ox_ES / 23.061 - 4.42.</t>
         </is>
       </c>
-      <c r="E15" s="14" t="inlineStr">
+      <c r="E15" s="16" t="inlineStr">
         <is>
           <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: E_PCplus_PCstar / V</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="n"/>
-      <c r="B16" s="14" t="n"/>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="15" t="n"/>
-      <c r="E16" s="14" t="n"/>
+      <c r="A16" s="16" t="inlineStr">
+        <is>
+          <t>Molecular size / A</t>
+        </is>
+      </c>
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>radius_S0 / A</t>
+        </is>
+      </c>
+      <c r="C16" s="16" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
+        <is>
+          <t>Radius of the sphere with the van der Waals volume of the optimised S0 geometry: union of atomic spheres with Bondi radii (Ir and Ru 2.00 A), counted on a 0.1 A grid. r_PC + r_Q is the contact distance of a pair in the benchmark.</t>
+        </is>
+      </c>
+      <c r="E16" s="16" t="inlineStr">
+        <is>
+          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: radius_S0 / A</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="16" t="n"/>
+      <c r="B17" s="16" t="n"/>
+      <c r="C17" s="16" t="n"/>
+      <c r="D17" s="17" t="n"/>
+      <c r="E17" s="16" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>One row per photocatalyst in the screen, sorted by new_id; the raw files use old_id.</t>
         </is>
       </c>
-      <c r="B17" s="14" t="n"/>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="15" t="n"/>
-      <c r="E17" s="14" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="B18" s="16" t="n"/>
+      <c r="C18" s="16" t="n"/>
+      <c r="D18" s="17" t="n"/>
+      <c r="E18" s="16" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>Every value is computed from the ORCA outputs. Total energies, Gibbs corrections and</t>
         </is>
       </c>
-      <c r="B18" s="14" t="n"/>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="15" t="n"/>
-      <c r="E18" s="14" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="B19" s="16" t="n"/>
+      <c r="C19" s="16" t="n"/>
+      <c r="D19" s="17" t="n"/>
+      <c r="E19" s="16" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>frequency checks are in computational_data_raw/photocatalysts/photocatalyst_dft.csv.</t>
         </is>
       </c>
-      <c r="B19" s="14" t="n"/>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="15" t="n"/>
-      <c r="E19" s="14" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="14" t="inlineStr">
+      <c r="B20" s="16" t="n"/>
+      <c r="C20" s="16" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="16" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Read with pandas as: pd.read_excel(path, header=1), then drop the 'Unnamed' columns.</t>
         </is>
       </c>
-      <c r="B20" s="14" t="n"/>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="15" t="n"/>
-      <c r="E20" s="14" t="n"/>
+      <c r="B21" s="16" t="n"/>
+      <c r="C21" s="16" t="n"/>
+      <c r="D21" s="17" t="n"/>
+      <c r="E21" s="16" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Merge the phenyl triplet of PC27 and rerun the benchmark
PC27 ([Ir(pmb)3]) takes its phenyl-centred T1 minimum, the lowest in Gibbs free energy, so the Ir(pmb)3 series PC25-27 now has one triplet character throughout. E_T, both reorganization energies and the excited-state potentials of PC27 change; the pair set is unchanged. Benchmark and further analysis rerun: no classification of the two-gate, adiabatic or DvTE criteria changes; the plain-barrier reference re-tunes its threshold, and the rate predictions of the two scored PC27 pairs rise.
</commit_message>
<xml_diff>
--- a/data/computational_data_processed/photocatalyst_properties_calc.xlsx
+++ b/data/computational_data_processed/photocatalyst_properties_calc.xlsx
@@ -1919,13 +1919,13 @@
         </is>
       </c>
       <c r="E29" s="14" t="n">
-        <v>79.87</v>
+        <v>77.7</v>
       </c>
       <c r="G29" s="14" t="n">
-        <v>34.95</v>
+        <v>17.43</v>
       </c>
       <c r="H29" s="14" t="n">
-        <v>14.5</v>
+        <v>12.77</v>
       </c>
       <c r="I29" s="14" t="n">
         <v>2.97</v>
@@ -1940,16 +1940,16 @@
         <v>4.42</v>
       </c>
       <c r="N29" s="14" t="n">
-        <v>47.39</v>
+        <v>49.56</v>
       </c>
       <c r="O29" s="14" t="n">
-        <v>-112.97</v>
+        <v>-110.8</v>
       </c>
       <c r="P29" s="14" t="n">
-        <v>0.48</v>
+        <v>0.38</v>
       </c>
       <c r="Q29" s="14" t="n">
-        <v>-2.37</v>
+        <v>-2.27</v>
       </c>
       <c r="S29" s="14" t="n">
         <v>5.17</v>

</xml_diff>

<commit_message>
Recompute PC25 as the fac isomer and rerun the benchmark
The PC25 deposit now holds the fac-[Ir(CF3-pmb)3] calculations (triplet 73.75 kcal/mol,
phenyl character). Its excited-state potentials rule out electron transfer for 13 more
quenching pairs, so the scored set grows to 868 pairs (392 quenching).
</commit_message>
<xml_diff>
--- a/data/computational_data_processed/photocatalyst_properties_calc.xlsx
+++ b/data/computational_data_processed/photocatalyst_properties_calc.xlsx
@@ -1821,37 +1821,37 @@
         </is>
       </c>
       <c r="E27" s="14" t="n">
-        <v>73.23</v>
+        <v>73.75</v>
       </c>
       <c r="G27" s="14" t="n">
-        <v>14.36</v>
+        <v>14.33</v>
       </c>
       <c r="H27" s="14" t="n">
-        <v>13.69</v>
+        <v>13.2</v>
       </c>
       <c r="I27" s="14" t="n">
-        <v>6.64</v>
+        <v>4.12</v>
       </c>
       <c r="J27" s="14" t="n">
-        <v>4.99</v>
+        <v>2.29</v>
       </c>
       <c r="K27" s="14" t="n">
-        <v>8.81</v>
+        <v>8.08</v>
       </c>
       <c r="L27" s="14" t="n">
-        <v>5.85</v>
+        <v>5.94</v>
       </c>
       <c r="N27" s="14" t="n">
-        <v>53.51</v>
+        <v>58.31</v>
       </c>
       <c r="O27" s="14" t="n">
-        <v>-107.29</v>
+        <v>-107.78</v>
       </c>
       <c r="P27" s="14" t="n">
-        <v>0.23</v>
+        <v>0.25</v>
       </c>
       <c r="Q27" s="14" t="n">
-        <v>-2.1</v>
+        <v>-1.89</v>
       </c>
       <c r="S27" s="14" t="n">
         <v>5.43</v>

</xml_diff>

<commit_message>
Key the photocatalyst data by the new ids throughout
Only compound_identification.xlsx carries the old ids now. The raw experimental
files keep their names; the Stern-Volmer and TCSPC scripts map old to new ids
on reading. The photocatalyst DFT, extent and mode scripts read
computational_data_raw/photocatalysts_new_ids, which now holds the tracked
photocatalyst_dft.csv.

Drop old_id and pc_old_id from the workbooks and datasets, key
molecular_extent.csv and reorganization_modes.csv by new id, and join mlj.py
and exclusion.py on pc_new_id. Correct the PC16 molar mass to 1269.79.
</commit_message>
<xml_diff>
--- a/data/computational_data_processed/photocatalyst_properties_calc.xlsx
+++ b/data/computational_data_processed/photocatalyst_properties_calc.xlsx
@@ -494,28 +494,27 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S29"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
-    <col width="8" customWidth="1" min="2" max="2"/>
-    <col width="36" customWidth="1" min="3" max="3"/>
-    <col width="2" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="2" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
+    <col width="2" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="2" customWidth="1" min="5" max="5"/>
+    <col width="27" customWidth="1" min="6" max="6"/>
     <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
     <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="31" customWidth="1" min="10" max="10"/>
     <col width="31" customWidth="1" min="11" max="11"/>
-    <col width="31" customWidth="1" min="12" max="12"/>
-    <col width="2" customWidth="1" min="13" max="13"/>
-    <col width="23" customWidth="1" min="14" max="14"/>
-    <col width="24" customWidth="1" min="15" max="15"/>
-    <col width="22" customWidth="1" min="16" max="16"/>
-    <col width="21" customWidth="1" min="17" max="17"/>
-    <col width="2" customWidth="1" min="18" max="18"/>
-    <col width="15" customWidth="1" min="19" max="19"/>
+    <col width="2" customWidth="1" min="12" max="12"/>
+    <col width="23" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="2" customWidth="1" min="17" max="17"/>
+    <col width="15" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
@@ -525,31 +524,30 @@
         </is>
       </c>
       <c r="B1" s="2" t="n"/>
-      <c r="C1" s="2" t="n"/>
-      <c r="E1" s="3" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Triplet energy / kcal mol-1</t>
         </is>
       </c>
-      <c r="G1" s="4" t="inlineStr">
+      <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Reorganization energies / kcal mol-1</t>
         </is>
       </c>
+      <c r="G1" s="5" t="n"/>
       <c r="H1" s="5" t="n"/>
       <c r="I1" s="5" t="n"/>
       <c r="J1" s="5" t="n"/>
       <c r="K1" s="5" t="n"/>
-      <c r="L1" s="5" t="n"/>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>Excited-state redox / kcal mol-1 and V vs SCE</t>
         </is>
       </c>
+      <c r="N1" s="7" t="n"/>
       <c r="O1" s="7" t="n"/>
       <c r="P1" s="7" t="n"/>
-      <c r="Q1" s="7" t="n"/>
-      <c r="S1" s="8" t="inlineStr">
+      <c r="R1" s="8" t="inlineStr">
         <is>
           <t>Molecular size / A</t>
         </is>
@@ -563,70 +561,65 @@
       </c>
       <c r="B2" s="9" t="inlineStr">
         <is>
-          <t>old_id</t>
-        </is>
-      </c>
-      <c r="C2" s="9" t="inlineStr">
-        <is>
           <t>compound</t>
         </is>
       </c>
-      <c r="E2" s="10" t="inlineStr">
+      <c r="D2" s="10" t="inlineStr">
         <is>
           <t>E_T / kcal mol-1</t>
         </is>
       </c>
+      <c r="F2" s="11" t="inlineStr">
+        <is>
+          <t>lambda_S0_T1 / kcal mol-1</t>
+        </is>
+      </c>
       <c r="G2" s="11" t="inlineStr">
         <is>
-          <t>lambda_S0_T1 / kcal mol-1</t>
+          <t>lambda_T1_S0 / kcal mol-1</t>
         </is>
       </c>
       <c r="H2" s="11" t="inlineStr">
         <is>
-          <t>lambda_T1_S0 / kcal mol-1</t>
+          <t>lambda_S0_Dplus / kcal mol-1</t>
         </is>
       </c>
       <c r="I2" s="11" t="inlineStr">
         <is>
-          <t>lambda_S0_Dplus / kcal mol-1</t>
+          <t>lambda_Dplus_S0 / kcal mol-1</t>
         </is>
       </c>
       <c r="J2" s="11" t="inlineStr">
         <is>
-          <t>lambda_Dplus_S0 / kcal mol-1</t>
+          <t>lambda_S0_Dminus / kcal mol-1</t>
         </is>
       </c>
       <c r="K2" s="11" t="inlineStr">
         <is>
-          <t>lambda_S0_Dminus / kcal mol-1</t>
-        </is>
-      </c>
-      <c r="L2" s="11" t="inlineStr">
-        <is>
           <t>lambda_Dminus_S0 / kcal mol-1</t>
         </is>
       </c>
+      <c r="M2" s="12" t="inlineStr">
+        <is>
+          <t>dG_ox_ES / kcal mol-1</t>
+        </is>
+      </c>
       <c r="N2" s="12" t="inlineStr">
         <is>
-          <t>dG_ox_ES / kcal mol-1</t>
+          <t>dG_red_ES / kcal mol-1</t>
         </is>
       </c>
       <c r="O2" s="12" t="inlineStr">
         <is>
-          <t>dG_red_ES / kcal mol-1</t>
+          <t>E_PCstar_PCminus / V</t>
         </is>
       </c>
       <c r="P2" s="12" t="inlineStr">
         <is>
-          <t>E_PCstar_PCminus / V</t>
-        </is>
-      </c>
-      <c r="Q2" s="12" t="inlineStr">
-        <is>
           <t>E_PCplus_PCstar / V</t>
         </is>
       </c>
-      <c r="S2" s="13" t="inlineStr">
+      <c r="R2" s="13" t="inlineStr">
         <is>
           <t>radius_S0 / A</t>
         </is>
@@ -636,48 +629,45 @@
       <c r="A3" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="C3" s="14" t="inlineStr">
+      <c r="B3" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(CF3)ppy)2(dtbbpy)][PF6]</t>
         </is>
       </c>
-      <c r="E3" s="14" t="n">
+      <c r="D3" s="14" t="n">
         <v>65.7</v>
       </c>
+      <c r="F3" s="14" t="n">
+        <v>10.28</v>
+      </c>
       <c r="G3" s="14" t="n">
-        <v>10.28</v>
+        <v>8.25</v>
       </c>
       <c r="H3" s="14" t="n">
-        <v>8.25</v>
+        <v>2.72</v>
       </c>
       <c r="I3" s="14" t="n">
-        <v>2.72</v>
+        <v>2.58</v>
       </c>
       <c r="J3" s="14" t="n">
-        <v>2.58</v>
+        <v>6.07</v>
       </c>
       <c r="K3" s="14" t="n">
-        <v>6.07</v>
-      </c>
-      <c r="L3" s="14" t="n">
         <v>6.12</v>
       </c>
+      <c r="M3" s="14" t="n">
+        <v>78.88</v>
+      </c>
       <c r="N3" s="14" t="n">
-        <v>78.88</v>
+        <v>-135.23</v>
       </c>
       <c r="O3" s="14" t="n">
-        <v>-135.23</v>
+        <v>1.44</v>
       </c>
       <c r="P3" s="14" t="n">
-        <v>1.44</v>
-      </c>
-      <c r="Q3" s="14" t="n">
         <v>-1</v>
       </c>
-      <c r="S3" s="14" t="n">
+      <c r="R3" s="14" t="n">
         <v>5.38</v>
       </c>
     </row>
@@ -685,48 +675,45 @@
       <c r="A4" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="B4" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" s="14" t="inlineStr">
+      <c r="B4" s="14" t="inlineStr">
         <is>
           <t>[Ir(ppy)2(dtbbpy)][PF6]</t>
         </is>
       </c>
-      <c r="E4" s="14" t="n">
+      <c r="D4" s="14" t="n">
         <v>59.35</v>
       </c>
+      <c r="F4" s="14" t="n">
+        <v>8.83</v>
+      </c>
       <c r="G4" s="14" t="n">
-        <v>8.83</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="H4" s="14" t="n">
-        <v>8.539999999999999</v>
+        <v>2.93</v>
       </c>
       <c r="I4" s="14" t="n">
-        <v>2.93</v>
+        <v>2.8</v>
       </c>
       <c r="J4" s="14" t="n">
-        <v>2.8</v>
+        <v>6.02</v>
       </c>
       <c r="K4" s="14" t="n">
-        <v>6.02</v>
-      </c>
-      <c r="L4" s="14" t="n">
         <v>8.6</v>
       </c>
+      <c r="M4" s="14" t="n">
+        <v>73.7</v>
+      </c>
       <c r="N4" s="14" t="n">
-        <v>73.7</v>
+        <v>-126.57</v>
       </c>
       <c r="O4" s="14" t="n">
-        <v>-126.57</v>
+        <v>1.07</v>
       </c>
       <c r="P4" s="14" t="n">
-        <v>1.07</v>
-      </c>
-      <c r="Q4" s="14" t="n">
         <v>-1.22</v>
       </c>
-      <c r="S4" s="14" t="n">
+      <c r="R4" s="14" t="n">
         <v>5.15</v>
       </c>
     </row>
@@ -734,48 +721,45 @@
       <c r="A5" s="14" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="14" t="n">
-        <v>3</v>
-      </c>
-      <c r="C5" s="14" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>Ir(ppy)3</t>
         </is>
       </c>
-      <c r="E5" s="14" t="n">
+      <c r="D5" s="14" t="n">
         <v>60.38</v>
       </c>
+      <c r="F5" s="14" t="n">
+        <v>11.82</v>
+      </c>
       <c r="G5" s="14" t="n">
-        <v>11.82</v>
+        <v>8.48</v>
       </c>
       <c r="H5" s="14" t="n">
-        <v>8.48</v>
+        <v>2.86</v>
       </c>
       <c r="I5" s="14" t="n">
-        <v>2.86</v>
+        <v>1.82</v>
       </c>
       <c r="J5" s="14" t="n">
-        <v>1.82</v>
+        <v>4.6</v>
       </c>
       <c r="K5" s="14" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="L5" s="14" t="n">
         <v>4.32</v>
       </c>
+      <c r="M5" s="14" t="n">
+        <v>61.94</v>
+      </c>
       <c r="N5" s="14" t="n">
-        <v>61.94</v>
+        <v>-108.38</v>
       </c>
       <c r="O5" s="14" t="n">
-        <v>-108.38</v>
+        <v>0.28</v>
       </c>
       <c r="P5" s="14" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="Q5" s="14" t="n">
         <v>-1.73</v>
       </c>
-      <c r="S5" s="14" t="n">
+      <c r="R5" s="14" t="n">
         <v>4.73</v>
       </c>
     </row>
@@ -783,48 +767,45 @@
       <c r="A6" s="14" t="n">
         <v>4</v>
       </c>
-      <c r="B6" s="14" t="n">
-        <v>4</v>
-      </c>
-      <c r="C6" s="14" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>Ir(dFppy)3</t>
         </is>
       </c>
-      <c r="E6" s="14" t="n">
+      <c r="D6" s="14" t="n">
         <v>65.62</v>
       </c>
+      <c r="F6" s="14" t="n">
+        <v>13.32</v>
+      </c>
       <c r="G6" s="14" t="n">
-        <v>13.32</v>
+        <v>8.890000000000001</v>
       </c>
       <c r="H6" s="14" t="n">
-        <v>8.890000000000001</v>
+        <v>1.48</v>
       </c>
       <c r="I6" s="14" t="n">
-        <v>1.48</v>
+        <v>1.35</v>
       </c>
       <c r="J6" s="14" t="n">
-        <v>1.35</v>
+        <v>4.46</v>
       </c>
       <c r="K6" s="14" t="n">
-        <v>4.46</v>
-      </c>
-      <c r="L6" s="14" t="n">
         <v>4.19</v>
       </c>
+      <c r="M6" s="14" t="n">
+        <v>65.90000000000001</v>
+      </c>
       <c r="N6" s="14" t="n">
-        <v>65.90000000000001</v>
+        <v>-116.12</v>
       </c>
       <c r="O6" s="14" t="n">
-        <v>-116.12</v>
+        <v>0.62</v>
       </c>
       <c r="P6" s="14" t="n">
-        <v>0.62</v>
-      </c>
-      <c r="Q6" s="14" t="n">
         <v>-1.56</v>
       </c>
-      <c r="S6" s="14" t="n">
+      <c r="R6" s="14" t="n">
         <v>4.82</v>
       </c>
     </row>
@@ -832,48 +813,45 @@
       <c r="A7" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="14" t="n">
-        <v>5</v>
-      </c>
-      <c r="C7" s="14" t="inlineStr">
+      <c r="B7" s="14" t="inlineStr">
         <is>
           <t>[Ru(dtbbpy)3][PF6]2</t>
         </is>
       </c>
-      <c r="E7" s="14" t="n">
+      <c r="D7" s="14" t="n">
         <v>44.61</v>
       </c>
+      <c r="F7" s="14" t="n">
+        <v>7.15</v>
+      </c>
       <c r="G7" s="14" t="n">
-        <v>7.15</v>
+        <v>7.48</v>
       </c>
       <c r="H7" s="14" t="n">
-        <v>7.48</v>
+        <v>0.97</v>
       </c>
       <c r="I7" s="14" t="n">
-        <v>0.97</v>
+        <v>1.22</v>
       </c>
       <c r="J7" s="14" t="n">
-        <v>1.22</v>
+        <v>5.83</v>
       </c>
       <c r="K7" s="14" t="n">
-        <v>5.83</v>
-      </c>
-      <c r="L7" s="14" t="n">
         <v>5.78</v>
       </c>
+      <c r="M7" s="14" t="n">
+        <v>80.01000000000001</v>
+      </c>
       <c r="N7" s="14" t="n">
-        <v>80.01000000000001</v>
+        <v>-110.13</v>
       </c>
       <c r="O7" s="14" t="n">
-        <v>-110.13</v>
+        <v>0.36</v>
       </c>
       <c r="P7" s="14" t="n">
-        <v>0.36</v>
-      </c>
-      <c r="Q7" s="14" t="n">
         <v>-0.95</v>
       </c>
-      <c r="S7" s="14" t="n">
+      <c r="R7" s="14" t="n">
         <v>5.84</v>
       </c>
     </row>
@@ -881,48 +859,45 @@
       <c r="A8" s="14" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="C8" s="14" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>[Ru(bpz)3][PF6]2</t>
         </is>
       </c>
-      <c r="E8" s="14" t="n">
+      <c r="D8" s="14" t="n">
         <v>46.98</v>
       </c>
+      <c r="F8" s="14" t="n">
+        <v>7.03</v>
+      </c>
       <c r="G8" s="14" t="n">
-        <v>7.03</v>
+        <v>7.08</v>
       </c>
       <c r="H8" s="14" t="n">
-        <v>7.08</v>
+        <v>0.93</v>
       </c>
       <c r="I8" s="14" t="n">
-        <v>0.93</v>
+        <v>1.03</v>
       </c>
       <c r="J8" s="14" t="n">
-        <v>1.03</v>
+        <v>5.31</v>
       </c>
       <c r="K8" s="14" t="n">
-        <v>5.31</v>
-      </c>
-      <c r="L8" s="14" t="n">
         <v>5.34</v>
       </c>
+      <c r="M8" s="14" t="n">
+        <v>101.29</v>
+      </c>
       <c r="N8" s="14" t="n">
-        <v>101.29</v>
+        <v>-132.67</v>
       </c>
       <c r="O8" s="14" t="n">
-        <v>-132.67</v>
+        <v>1.33</v>
       </c>
       <c r="P8" s="14" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="Q8" s="14" t="n">
         <v>-0.03</v>
       </c>
-      <c r="S8" s="14" t="n">
+      <c r="R8" s="14" t="n">
         <v>4.61</v>
       </c>
     </row>
@@ -930,48 +905,45 @@
       <c r="A9" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="14" t="n">
-        <v>9</v>
-      </c>
-      <c r="C9" s="14" t="inlineStr">
+      <c r="B9" s="14" t="inlineStr">
         <is>
           <t>Ir(dF(Me)ppy)3</t>
         </is>
       </c>
-      <c r="E9" s="14" t="n">
+      <c r="D9" s="14" t="n">
         <v>66.15000000000001</v>
       </c>
+      <c r="F9" s="14" t="n">
+        <v>13.77</v>
+      </c>
       <c r="G9" s="14" t="n">
-        <v>13.77</v>
+        <v>9.1</v>
       </c>
       <c r="H9" s="14" t="n">
-        <v>9.1</v>
+        <v>1.46</v>
       </c>
       <c r="I9" s="14" t="n">
-        <v>1.46</v>
+        <v>1.4</v>
       </c>
       <c r="J9" s="14" t="n">
-        <v>1.4</v>
+        <v>4.25</v>
       </c>
       <c r="K9" s="14" t="n">
-        <v>4.25</v>
-      </c>
-      <c r="L9" s="14" t="n">
         <v>4.07</v>
       </c>
+      <c r="M9" s="14" t="n">
+        <v>64.17</v>
+      </c>
       <c r="N9" s="14" t="n">
-        <v>64.17</v>
+        <v>-114.79</v>
       </c>
       <c r="O9" s="14" t="n">
-        <v>-114.79</v>
+        <v>0.5600000000000001</v>
       </c>
       <c r="P9" s="14" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="Q9" s="14" t="n">
         <v>-1.64</v>
       </c>
-      <c r="S9" s="14" t="n">
+      <c r="R9" s="14" t="n">
         <v>4.99</v>
       </c>
     </row>
@@ -979,48 +951,45 @@
       <c r="A10" s="14" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="14" t="n">
-        <v>10</v>
-      </c>
-      <c r="C10" s="14" t="inlineStr">
+      <c r="B10" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(CF3)ppy)2(d(5,5)CF3bpy)]PF6</t>
         </is>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="D10" s="14" t="n">
         <v>55.94</v>
       </c>
+      <c r="F10" s="14" t="n">
+        <v>8.630000000000001</v>
+      </c>
       <c r="G10" s="14" t="n">
-        <v>8.630000000000001</v>
+        <v>9.48</v>
       </c>
       <c r="H10" s="14" t="n">
-        <v>9.48</v>
+        <v>2.68</v>
       </c>
       <c r="I10" s="14" t="n">
-        <v>2.68</v>
+        <v>2.66</v>
       </c>
       <c r="J10" s="14" t="n">
-        <v>2.66</v>
+        <v>6.56</v>
       </c>
       <c r="K10" s="14" t="n">
-        <v>6.56</v>
-      </c>
-      <c r="L10" s="14" t="n">
         <v>7.54</v>
       </c>
+      <c r="M10" s="14" t="n">
+        <v>93.31</v>
+      </c>
       <c r="N10" s="14" t="n">
-        <v>93.31</v>
+        <v>-139.65</v>
       </c>
       <c r="O10" s="14" t="n">
-        <v>-139.65</v>
+        <v>1.64</v>
       </c>
       <c r="P10" s="14" t="n">
-        <v>1.64</v>
-      </c>
-      <c r="Q10" s="14" t="n">
         <v>-0.37</v>
       </c>
-      <c r="S10" s="14" t="n">
+      <c r="R10" s="14" t="n">
         <v>5.18</v>
       </c>
     </row>
@@ -1028,48 +997,45 @@
       <c r="A11" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="14" t="n">
-        <v>11</v>
-      </c>
-      <c r="C11" s="14" t="inlineStr">
+      <c r="B11" s="14" t="inlineStr">
         <is>
           <t>[Ir(dFppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E11" s="14" t="n">
+      <c r="D11" s="14" t="n">
         <v>63.94</v>
       </c>
+      <c r="F11" s="14" t="n">
+        <v>8.31</v>
+      </c>
       <c r="G11" s="14" t="n">
-        <v>8.31</v>
+        <v>7.94</v>
       </c>
       <c r="H11" s="14" t="n">
-        <v>7.94</v>
+        <v>2.55</v>
       </c>
       <c r="I11" s="14" t="n">
-        <v>2.55</v>
+        <v>2.44</v>
       </c>
       <c r="J11" s="14" t="n">
-        <v>2.44</v>
+        <v>6.02</v>
       </c>
       <c r="K11" s="14" t="n">
-        <v>6.02</v>
-      </c>
-      <c r="L11" s="14" t="n">
         <v>6.05</v>
       </c>
+      <c r="M11" s="14" t="n">
+        <v>77.48999999999999</v>
+      </c>
       <c r="N11" s="14" t="n">
-        <v>77.48999999999999</v>
+        <v>-132.44</v>
       </c>
       <c r="O11" s="14" t="n">
-        <v>-132.44</v>
+        <v>1.32</v>
       </c>
       <c r="P11" s="14" t="n">
-        <v>1.32</v>
-      </c>
-      <c r="Q11" s="14" t="n">
         <v>-1.06</v>
       </c>
-      <c r="S11" s="14" t="n">
+      <c r="R11" s="14" t="n">
         <v>5.21</v>
       </c>
     </row>
@@ -1077,48 +1043,45 @@
       <c r="A12" s="14" t="n">
         <v>10</v>
       </c>
-      <c r="B12" s="14" t="n">
-        <v>12</v>
-      </c>
-      <c r="C12" s="14" t="inlineStr">
+      <c r="B12" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(Me)ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E12" s="14" t="n">
+      <c r="D12" s="14" t="n">
         <v>63.38</v>
       </c>
+      <c r="F12" s="14" t="n">
+        <v>8.199999999999999</v>
+      </c>
       <c r="G12" s="14" t="n">
-        <v>8.199999999999999</v>
+        <v>7.88</v>
       </c>
       <c r="H12" s="14" t="n">
-        <v>7.88</v>
+        <v>2.51</v>
       </c>
       <c r="I12" s="14" t="n">
-        <v>2.51</v>
+        <v>2.44</v>
       </c>
       <c r="J12" s="14" t="n">
-        <v>2.44</v>
+        <v>6.01</v>
       </c>
       <c r="K12" s="14" t="n">
         <v>6.01</v>
       </c>
-      <c r="L12" s="14" t="n">
-        <v>6.01</v>
+      <c r="M12" s="14" t="n">
+        <v>77.14</v>
       </c>
       <c r="N12" s="14" t="n">
-        <v>77.14</v>
+        <v>-131.45</v>
       </c>
       <c r="O12" s="14" t="n">
-        <v>-131.45</v>
+        <v>1.28</v>
       </c>
       <c r="P12" s="14" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="Q12" s="14" t="n">
         <v>-1.07</v>
       </c>
-      <c r="S12" s="14" t="n">
+      <c r="R12" s="14" t="n">
         <v>5.3</v>
       </c>
     </row>
@@ -1126,48 +1089,45 @@
       <c r="A13" s="14" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="14" t="n">
-        <v>13</v>
-      </c>
-      <c r="C13" s="14" t="inlineStr">
+      <c r="B13" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(CF3)ppy)2(bpy)]PF6</t>
         </is>
       </c>
-      <c r="E13" s="14" t="n">
+      <c r="D13" s="14" t="n">
         <v>65.67</v>
       </c>
+      <c r="F13" s="14" t="n">
+        <v>10.34</v>
+      </c>
       <c r="G13" s="14" t="n">
-        <v>10.34</v>
+        <v>8.75</v>
       </c>
       <c r="H13" s="14" t="n">
-        <v>8.75</v>
+        <v>2.6</v>
       </c>
       <c r="I13" s="14" t="n">
-        <v>2.6</v>
+        <v>2.5</v>
       </c>
       <c r="J13" s="14" t="n">
-        <v>2.5</v>
+        <v>5.97</v>
       </c>
       <c r="K13" s="14" t="n">
-        <v>5.97</v>
-      </c>
-      <c r="L13" s="14" t="n">
         <v>6.04</v>
       </c>
+      <c r="M13" s="14" t="n">
+        <v>79.73</v>
+      </c>
       <c r="N13" s="14" t="n">
-        <v>79.73</v>
+        <v>-137.69</v>
       </c>
       <c r="O13" s="14" t="n">
-        <v>-137.69</v>
+        <v>1.55</v>
       </c>
       <c r="P13" s="14" t="n">
-        <v>1.55</v>
-      </c>
-      <c r="Q13" s="14" t="n">
         <v>-0.96</v>
       </c>
-      <c r="S13" s="14" t="n">
+      <c r="R13" s="14" t="n">
         <v>4.99</v>
       </c>
     </row>
@@ -1175,48 +1135,45 @@
       <c r="A14" s="14" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="14" t="n">
-        <v>14</v>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
+      <c r="B14" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(Me)ppy)2(d(5,5)CH3bpy)]PF6</t>
         </is>
       </c>
-      <c r="E14" s="14" t="n">
+      <c r="D14" s="14" t="n">
         <v>65.70999999999999</v>
       </c>
+      <c r="F14" s="14" t="n">
+        <v>13.55</v>
+      </c>
       <c r="G14" s="14" t="n">
-        <v>13.55</v>
+        <v>12.58</v>
       </c>
       <c r="H14" s="14" t="n">
-        <v>12.58</v>
+        <v>2.48</v>
       </c>
       <c r="I14" s="14" t="n">
-        <v>2.48</v>
+        <v>2.43</v>
       </c>
       <c r="J14" s="14" t="n">
-        <v>2.43</v>
+        <v>5.65</v>
       </c>
       <c r="K14" s="14" t="n">
-        <v>5.65</v>
-      </c>
-      <c r="L14" s="14" t="n">
         <v>5.61</v>
       </c>
+      <c r="M14" s="14" t="n">
+        <v>75.04000000000001</v>
+      </c>
       <c r="N14" s="14" t="n">
-        <v>75.04000000000001</v>
+        <v>-132.46</v>
       </c>
       <c r="O14" s="14" t="n">
-        <v>-132.46</v>
+        <v>1.32</v>
       </c>
       <c r="P14" s="14" t="n">
-        <v>1.32</v>
-      </c>
-      <c r="Q14" s="14" t="n">
         <v>-1.17</v>
       </c>
-      <c r="S14" s="14" t="n">
+      <c r="R14" s="14" t="n">
         <v>5.01</v>
       </c>
     </row>
@@ -1224,48 +1181,45 @@
       <c r="A15" s="14" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="14" t="n">
-        <v>15</v>
-      </c>
-      <c r="C15" s="14" t="inlineStr">
+      <c r="B15" s="14" t="inlineStr">
         <is>
           <t>[Ir(tCF3ppy)2(d(5,5)CH3bpy)]PF6</t>
         </is>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="D15" s="14" t="n">
         <v>59.39</v>
       </c>
+      <c r="F15" s="14" t="n">
+        <v>11.39</v>
+      </c>
       <c r="G15" s="14" t="n">
-        <v>11.39</v>
+        <v>9.220000000000001</v>
       </c>
       <c r="H15" s="14" t="n">
-        <v>9.220000000000001</v>
+        <v>2.21</v>
       </c>
       <c r="I15" s="14" t="n">
-        <v>2.21</v>
+        <v>2.05</v>
       </c>
       <c r="J15" s="14" t="n">
-        <v>2.05</v>
+        <v>5.71</v>
       </c>
       <c r="K15" s="14" t="n">
-        <v>5.71</v>
-      </c>
-      <c r="L15" s="14" t="n">
         <v>5.77</v>
       </c>
+      <c r="M15" s="14" t="n">
+        <v>88.05</v>
+      </c>
       <c r="N15" s="14" t="n">
-        <v>88.05</v>
+        <v>-128.12</v>
       </c>
       <c r="O15" s="14" t="n">
-        <v>-128.12</v>
+        <v>1.14</v>
       </c>
       <c r="P15" s="14" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="Q15" s="14" t="n">
         <v>-0.6</v>
       </c>
-      <c r="S15" s="14" t="n">
+      <c r="R15" s="14" t="n">
         <v>5.39</v>
       </c>
     </row>
@@ -1273,48 +1227,45 @@
       <c r="A16" s="14" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="14" t="n">
-        <v>16</v>
-      </c>
-      <c r="C16" s="14" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(Me)ppy)2(d(OMe)bpy)]PF6</t>
         </is>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="D16" s="14" t="n">
         <v>65.73999999999999</v>
       </c>
+      <c r="F16" s="14" t="n">
+        <v>13.47</v>
+      </c>
       <c r="G16" s="14" t="n">
-        <v>13.47</v>
+        <v>13.08</v>
       </c>
       <c r="H16" s="14" t="n">
-        <v>13.08</v>
+        <v>2.53</v>
       </c>
       <c r="I16" s="14" t="n">
-        <v>2.53</v>
+        <v>2.41</v>
       </c>
       <c r="J16" s="14" t="n">
-        <v>2.41</v>
+        <v>6.88</v>
       </c>
       <c r="K16" s="14" t="n">
-        <v>6.88</v>
-      </c>
-      <c r="L16" s="14" t="n">
         <v>7</v>
       </c>
+      <c r="M16" s="14" t="n">
+        <v>73.91</v>
+      </c>
       <c r="N16" s="14" t="n">
-        <v>73.91</v>
+        <v>-131.74</v>
       </c>
       <c r="O16" s="14" t="n">
-        <v>-131.74</v>
+        <v>1.29</v>
       </c>
       <c r="P16" s="14" t="n">
-        <v>1.29</v>
-      </c>
-      <c r="Q16" s="14" t="n">
         <v>-1.22</v>
       </c>
-      <c r="S16" s="14" t="n">
+      <c r="R16" s="14" t="n">
         <v>5.06</v>
       </c>
     </row>
@@ -1322,48 +1273,45 @@
       <c r="A17" s="14" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="14" t="n">
-        <v>17</v>
-      </c>
-      <c r="C17" s="14" t="inlineStr">
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>[Ir(ppy)2(d(OMe)bpy)]PF6</t>
         </is>
       </c>
-      <c r="E17" s="14" t="n">
+      <c r="D17" s="14" t="n">
         <v>59.92</v>
       </c>
+      <c r="F17" s="14" t="n">
+        <v>9.140000000000001</v>
+      </c>
       <c r="G17" s="14" t="n">
-        <v>9.140000000000001</v>
+        <v>9.02</v>
       </c>
       <c r="H17" s="14" t="n">
-        <v>9.02</v>
+        <v>2.82</v>
       </c>
       <c r="I17" s="14" t="n">
-        <v>2.82</v>
+        <v>2.86</v>
       </c>
       <c r="J17" s="14" t="n">
-        <v>2.86</v>
+        <v>6.86</v>
       </c>
       <c r="K17" s="14" t="n">
-        <v>6.86</v>
-      </c>
-      <c r="L17" s="14" t="n">
         <v>6.97</v>
       </c>
+      <c r="M17" s="14" t="n">
+        <v>72.40000000000001</v>
+      </c>
       <c r="N17" s="14" t="n">
-        <v>72.40000000000001</v>
+        <v>-125.16</v>
       </c>
       <c r="O17" s="14" t="n">
-        <v>-125.16</v>
+        <v>1.01</v>
       </c>
       <c r="P17" s="14" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="Q17" s="14" t="n">
         <v>-1.28</v>
       </c>
-      <c r="S17" s="14" t="n">
+      <c r="R17" s="14" t="n">
         <v>4.9</v>
       </c>
     </row>
@@ -1371,48 +1319,45 @@
       <c r="A18" s="14" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="14" t="n">
-        <v>18</v>
-      </c>
-      <c r="C18" s="14" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>[Ir(tCF3ppy)2(d(5,5)OMebpy)]PF6</t>
         </is>
       </c>
-      <c r="E18" s="14" t="n">
+      <c r="D18" s="14" t="n">
         <v>59.14</v>
       </c>
+      <c r="F18" s="14" t="n">
+        <v>10.9</v>
+      </c>
       <c r="G18" s="14" t="n">
-        <v>10.9</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="H18" s="14" t="n">
-        <v>9.300000000000001</v>
+        <v>1.79</v>
       </c>
       <c r="I18" s="14" t="n">
-        <v>1.79</v>
+        <v>2.23</v>
       </c>
       <c r="J18" s="14" t="n">
-        <v>2.23</v>
+        <v>6.28</v>
       </c>
       <c r="K18" s="14" t="n">
-        <v>6.28</v>
-      </c>
-      <c r="L18" s="14" t="n">
         <v>6.15</v>
       </c>
+      <c r="M18" s="14" t="n">
+        <v>88.68000000000001</v>
+      </c>
       <c r="N18" s="14" t="n">
-        <v>88.68000000000001</v>
+        <v>-133.2</v>
       </c>
       <c r="O18" s="14" t="n">
-        <v>-133.2</v>
+        <v>1.36</v>
       </c>
       <c r="P18" s="14" t="n">
-        <v>1.36</v>
-      </c>
-      <c r="Q18" s="14" t="n">
         <v>-0.57</v>
       </c>
-      <c r="S18" s="14" t="n">
+      <c r="R18" s="14" t="n">
         <v>5.44</v>
       </c>
     </row>
@@ -1420,48 +1365,45 @@
       <c r="A19" s="14" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="14" t="n">
-        <v>19</v>
-      </c>
-      <c r="C19" s="14" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>[Ir(dCF3ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E19" s="14" t="n">
+      <c r="D19" s="14" t="n">
         <v>60.55</v>
       </c>
+      <c r="F19" s="14" t="n">
+        <v>13.24</v>
+      </c>
       <c r="G19" s="14" t="n">
-        <v>13.24</v>
+        <v>10.81</v>
       </c>
       <c r="H19" s="14" t="n">
-        <v>10.81</v>
+        <v>1.99</v>
       </c>
       <c r="I19" s="14" t="n">
-        <v>1.99</v>
+        <v>2.11</v>
       </c>
       <c r="J19" s="14" t="n">
-        <v>2.11</v>
+        <v>6.3</v>
       </c>
       <c r="K19" s="14" t="n">
-        <v>6.3</v>
-      </c>
-      <c r="L19" s="14" t="n">
         <v>6.41</v>
       </c>
+      <c r="M19" s="14" t="n">
+        <v>83.55</v>
+      </c>
       <c r="N19" s="14" t="n">
-        <v>83.55</v>
+        <v>-127.03</v>
       </c>
       <c r="O19" s="14" t="n">
-        <v>-127.03</v>
+        <v>1.09</v>
       </c>
       <c r="P19" s="14" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="Q19" s="14" t="n">
         <v>-0.8</v>
       </c>
-      <c r="S19" s="14" t="n">
+      <c r="R19" s="14" t="n">
         <v>5.49</v>
       </c>
     </row>
@@ -1469,48 +1411,45 @@
       <c r="A20" s="14" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="14" t="n">
-        <v>20</v>
-      </c>
-      <c r="C20" s="14" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(6-OMe)ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E20" s="14" t="n">
+      <c r="D20" s="14" t="n">
         <v>64.83</v>
       </c>
+      <c r="F20" s="14" t="n">
+        <v>12.7</v>
+      </c>
       <c r="G20" s="14" t="n">
-        <v>12.7</v>
+        <v>11.75</v>
       </c>
       <c r="H20" s="14" t="n">
-        <v>11.75</v>
+        <v>2.57</v>
       </c>
       <c r="I20" s="14" t="n">
-        <v>2.57</v>
+        <v>2.45</v>
       </c>
       <c r="J20" s="14" t="n">
-        <v>2.45</v>
+        <v>6.01</v>
       </c>
       <c r="K20" s="14" t="n">
-        <v>6.01</v>
-      </c>
-      <c r="L20" s="14" t="n">
         <v>6.08</v>
       </c>
+      <c r="M20" s="14" t="n">
+        <v>73.62</v>
+      </c>
       <c r="N20" s="14" t="n">
-        <v>73.62</v>
+        <v>-129.39</v>
       </c>
       <c r="O20" s="14" t="n">
-        <v>-129.39</v>
+        <v>1.19</v>
       </c>
       <c r="P20" s="14" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="Q20" s="14" t="n">
         <v>-1.23</v>
       </c>
-      <c r="S20" s="14" t="n">
+      <c r="R20" s="14" t="n">
         <v>5.35</v>
       </c>
     </row>
@@ -1518,48 +1457,45 @@
       <c r="A21" s="14" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="14" t="n">
-        <v>21</v>
-      </c>
-      <c r="C21" s="14" t="inlineStr">
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(OMe)ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E21" s="14" t="n">
+      <c r="D21" s="14" t="n">
         <v>63.27</v>
       </c>
+      <c r="F21" s="14" t="n">
+        <v>12.88</v>
+      </c>
       <c r="G21" s="14" t="n">
-        <v>12.88</v>
+        <v>10.57</v>
       </c>
       <c r="H21" s="14" t="n">
-        <v>10.57</v>
+        <v>2.65</v>
       </c>
       <c r="I21" s="14" t="n">
-        <v>2.65</v>
+        <v>2.66</v>
       </c>
       <c r="J21" s="14" t="n">
-        <v>2.66</v>
+        <v>6.04</v>
       </c>
       <c r="K21" s="14" t="n">
-        <v>6.04</v>
-      </c>
-      <c r="L21" s="14" t="n">
         <v>6.08</v>
       </c>
+      <c r="M21" s="14" t="n">
+        <v>76.45</v>
+      </c>
       <c r="N21" s="14" t="n">
-        <v>76.45</v>
+        <v>-131.55</v>
       </c>
       <c r="O21" s="14" t="n">
-        <v>-131.55</v>
+        <v>1.28</v>
       </c>
       <c r="P21" s="14" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="Q21" s="14" t="n">
         <v>-1.1</v>
       </c>
-      <c r="S21" s="14" t="n">
+      <c r="R21" s="14" t="n">
         <v>5.35</v>
       </c>
     </row>
@@ -1567,48 +1503,45 @@
       <c r="A22" s="14" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="14" t="n">
-        <v>22</v>
-      </c>
-      <c r="C22" s="14" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>[Ir(tCF3ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E22" s="14" t="n">
+      <c r="D22" s="14" t="n">
         <v>59.81</v>
       </c>
+      <c r="F22" s="14" t="n">
+        <v>11.09</v>
+      </c>
       <c r="G22" s="14" t="n">
-        <v>11.09</v>
+        <v>8.85</v>
       </c>
       <c r="H22" s="14" t="n">
-        <v>8.85</v>
+        <v>2.46</v>
       </c>
       <c r="I22" s="14" t="n">
-        <v>2.46</v>
+        <v>1.9</v>
       </c>
       <c r="J22" s="14" t="n">
-        <v>1.9</v>
+        <v>6.41</v>
       </c>
       <c r="K22" s="14" t="n">
-        <v>6.41</v>
-      </c>
-      <c r="L22" s="14" t="n">
         <v>6.05</v>
       </c>
+      <c r="M22" s="14" t="n">
+        <v>87.42</v>
+      </c>
       <c r="N22" s="14" t="n">
-        <v>87.42</v>
+        <v>-129.41</v>
       </c>
       <c r="O22" s="14" t="n">
-        <v>-129.41</v>
+        <v>1.19</v>
       </c>
       <c r="P22" s="14" t="n">
-        <v>1.19</v>
-      </c>
-      <c r="Q22" s="14" t="n">
         <v>-0.63</v>
       </c>
-      <c r="S22" s="14" t="n">
+      <c r="R22" s="14" t="n">
         <v>5.65</v>
       </c>
     </row>
@@ -1616,48 +1549,45 @@
       <c r="A23" s="14" t="n">
         <v>21</v>
       </c>
-      <c r="B23" s="14" t="n">
-        <v>23</v>
-      </c>
-      <c r="C23" s="14" t="inlineStr">
+      <c r="B23" s="14" t="inlineStr">
         <is>
           <t>[Ir(tetraFppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E23" s="14" t="n">
+      <c r="D23" s="14" t="n">
         <v>66.11</v>
       </c>
+      <c r="F23" s="14" t="n">
+        <v>8.119999999999999</v>
+      </c>
       <c r="G23" s="14" t="n">
-        <v>8.119999999999999</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="H23" s="14" t="n">
-        <v>8.300000000000001</v>
+        <v>2.8</v>
       </c>
       <c r="I23" s="14" t="n">
-        <v>2.8</v>
+        <v>3.11</v>
       </c>
       <c r="J23" s="14" t="n">
-        <v>3.11</v>
+        <v>6.04</v>
       </c>
       <c r="K23" s="14" t="n">
-        <v>6.04</v>
-      </c>
-      <c r="L23" s="14" t="n">
         <v>6.08</v>
       </c>
+      <c r="M23" s="14" t="n">
+        <v>78.63</v>
+      </c>
       <c r="N23" s="14" t="n">
-        <v>78.63</v>
+        <v>-136.34</v>
       </c>
       <c r="O23" s="14" t="n">
-        <v>-136.34</v>
+        <v>1.49</v>
       </c>
       <c r="P23" s="14" t="n">
-        <v>1.49</v>
-      </c>
-      <c r="Q23" s="14" t="n">
         <v>-1.01</v>
       </c>
-      <c r="S23" s="14" t="n">
+      <c r="R23" s="14" t="n">
         <v>5.26</v>
       </c>
     </row>
@@ -1665,48 +1595,45 @@
       <c r="A24" s="14" t="n">
         <v>22</v>
       </c>
-      <c r="B24" s="14" t="n">
-        <v>24</v>
-      </c>
-      <c r="C24" s="14" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>[Ir(d(OMe)ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E24" s="14" t="n">
+      <c r="D24" s="14" t="n">
         <v>59.01</v>
       </c>
+      <c r="F24" s="14" t="n">
+        <v>8.289999999999999</v>
+      </c>
       <c r="G24" s="14" t="n">
-        <v>8.289999999999999</v>
+        <v>7.93</v>
       </c>
       <c r="H24" s="14" t="n">
-        <v>7.93</v>
+        <v>2.54</v>
       </c>
       <c r="I24" s="14" t="n">
-        <v>2.54</v>
+        <v>2.53</v>
       </c>
       <c r="J24" s="14" t="n">
-        <v>2.53</v>
+        <v>6</v>
       </c>
       <c r="K24" s="14" t="n">
-        <v>6</v>
-      </c>
-      <c r="L24" s="14" t="n">
         <v>6.01</v>
       </c>
+      <c r="M24" s="14" t="n">
+        <v>74.41</v>
+      </c>
       <c r="N24" s="14" t="n">
-        <v>74.41</v>
+        <v>-125.22</v>
       </c>
       <c r="O24" s="14" t="n">
-        <v>-125.22</v>
+        <v>1.01</v>
       </c>
       <c r="P24" s="14" t="n">
-        <v>1.01</v>
-      </c>
-      <c r="Q24" s="14" t="n">
         <v>-1.19</v>
       </c>
-      <c r="S24" s="14" t="n">
+      <c r="R24" s="14" t="n">
         <v>5.43</v>
       </c>
     </row>
@@ -1714,48 +1641,45 @@
       <c r="A25" s="14" t="n">
         <v>23</v>
       </c>
-      <c r="B25" s="14" t="n">
-        <v>25</v>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
         <is>
           <t>[Ir(dF(4-Me)ppy)2(dtbbpy)]PF6</t>
         </is>
       </c>
-      <c r="E25" s="14" t="n">
+      <c r="D25" s="14" t="n">
         <v>64.62</v>
       </c>
+      <c r="F25" s="14" t="n">
+        <v>8.42</v>
+      </c>
       <c r="G25" s="14" t="n">
-        <v>8.42</v>
+        <v>8.039999999999999</v>
       </c>
       <c r="H25" s="14" t="n">
-        <v>8.039999999999999</v>
+        <v>2.59</v>
       </c>
       <c r="I25" s="14" t="n">
-        <v>2.59</v>
+        <v>2.43</v>
       </c>
       <c r="J25" s="14" t="n">
-        <v>2.43</v>
+        <v>6.18</v>
       </c>
       <c r="K25" s="14" t="n">
-        <v>6.18</v>
-      </c>
-      <c r="L25" s="14" t="n">
         <v>6.12</v>
       </c>
+      <c r="M25" s="14" t="n">
+        <v>75.92</v>
+      </c>
       <c r="N25" s="14" t="n">
-        <v>75.92</v>
+        <v>-131.37</v>
       </c>
       <c r="O25" s="14" t="n">
-        <v>-131.37</v>
+        <v>1.28</v>
       </c>
       <c r="P25" s="14" t="n">
-        <v>1.28</v>
-      </c>
-      <c r="Q25" s="14" t="n">
         <v>-1.13</v>
       </c>
-      <c r="S25" s="14" t="n">
+      <c r="R25" s="14" t="n">
         <v>5.3</v>
       </c>
     </row>
@@ -1763,48 +1687,45 @@
       <c r="A26" s="14" t="n">
         <v>24</v>
       </c>
-      <c r="B26" s="14" t="n">
-        <v>27</v>
-      </c>
-      <c r="C26" s="14" t="inlineStr">
+      <c r="B26" s="14" t="inlineStr">
         <is>
           <t>[Ir(ppy)2(phen)]PF6</t>
         </is>
       </c>
-      <c r="E26" s="14" t="n">
+      <c r="D26" s="14" t="n">
         <v>57.55</v>
       </c>
+      <c r="F26" s="14" t="n">
+        <v>7.93</v>
+      </c>
       <c r="G26" s="14" t="n">
-        <v>7.93</v>
+        <v>7.58</v>
       </c>
       <c r="H26" s="14" t="n">
-        <v>7.58</v>
+        <v>2.78</v>
       </c>
       <c r="I26" s="14" t="n">
-        <v>2.78</v>
+        <v>2.83</v>
       </c>
       <c r="J26" s="14" t="n">
-        <v>2.83</v>
+        <v>5.11</v>
       </c>
       <c r="K26" s="14" t="n">
-        <v>5.11</v>
-      </c>
-      <c r="L26" s="14" t="n">
         <v>5.06</v>
       </c>
+      <c r="M26" s="14" t="n">
+        <v>76.25</v>
+      </c>
       <c r="N26" s="14" t="n">
-        <v>76.25</v>
+        <v>-125.75</v>
       </c>
       <c r="O26" s="14" t="n">
-        <v>-125.75</v>
+        <v>1.03</v>
       </c>
       <c r="P26" s="14" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="Q26" s="14" t="n">
         <v>-1.11</v>
       </c>
-      <c r="S26" s="14" t="n">
+      <c r="R26" s="14" t="n">
         <v>4.78</v>
       </c>
     </row>
@@ -1812,48 +1733,45 @@
       <c r="A27" s="14" t="n">
         <v>25</v>
       </c>
-      <c r="B27" s="14" t="n">
-        <v>8</v>
-      </c>
-      <c r="C27" s="14" t="inlineStr">
+      <c r="B27" s="14" t="inlineStr">
         <is>
           <t>[Ir(CF3-pmb)3]</t>
         </is>
       </c>
-      <c r="E27" s="14" t="n">
+      <c r="D27" s="14" t="n">
         <v>73.75</v>
       </c>
+      <c r="F27" s="14" t="n">
+        <v>14.33</v>
+      </c>
       <c r="G27" s="14" t="n">
-        <v>14.33</v>
+        <v>13.2</v>
       </c>
       <c r="H27" s="14" t="n">
-        <v>13.2</v>
+        <v>4.12</v>
       </c>
       <c r="I27" s="14" t="n">
-        <v>4.12</v>
+        <v>2.29</v>
       </c>
       <c r="J27" s="14" t="n">
-        <v>2.29</v>
+        <v>8.08</v>
       </c>
       <c r="K27" s="14" t="n">
-        <v>8.08</v>
-      </c>
-      <c r="L27" s="14" t="n">
         <v>5.94</v>
       </c>
+      <c r="M27" s="14" t="n">
+        <v>58.31</v>
+      </c>
       <c r="N27" s="14" t="n">
-        <v>58.31</v>
+        <v>-107.78</v>
       </c>
       <c r="O27" s="14" t="n">
-        <v>-107.78</v>
+        <v>0.25</v>
       </c>
       <c r="P27" s="14" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="Q27" s="14" t="n">
         <v>-1.89</v>
       </c>
-      <c r="S27" s="14" t="n">
+      <c r="R27" s="14" t="n">
         <v>5.43</v>
       </c>
     </row>
@@ -1861,48 +1779,45 @@
       <c r="A28" s="14" t="n">
         <v>26</v>
       </c>
-      <c r="B28" s="14" t="n">
-        <v>28</v>
-      </c>
-      <c r="C28" s="14" t="inlineStr">
+      <c r="B28" s="14" t="inlineStr">
         <is>
           <t>[Ir(CH3-pmb)3]</t>
         </is>
       </c>
-      <c r="E28" s="14" t="n">
+      <c r="D28" s="14" t="n">
         <v>76.81999999999999</v>
       </c>
+      <c r="F28" s="14" t="n">
+        <v>19.11</v>
+      </c>
       <c r="G28" s="14" t="n">
-        <v>19.11</v>
+        <v>13.66</v>
       </c>
       <c r="H28" s="14" t="n">
-        <v>13.66</v>
+        <v>2.86</v>
       </c>
       <c r="I28" s="14" t="n">
-        <v>2.86</v>
+        <v>2.1</v>
       </c>
       <c r="J28" s="14" t="n">
-        <v>2.1</v>
+        <v>5.2</v>
       </c>
       <c r="K28" s="14" t="n">
-        <v>5.2</v>
-      </c>
-      <c r="L28" s="14" t="n">
         <v>4.44</v>
       </c>
+      <c r="M28" s="14" t="n">
+        <v>48.79</v>
+      </c>
       <c r="N28" s="14" t="n">
-        <v>48.79</v>
+        <v>-109.67</v>
       </c>
       <c r="O28" s="14" t="n">
-        <v>-109.67</v>
+        <v>0.34</v>
       </c>
       <c r="P28" s="14" t="n">
-        <v>0.34</v>
-      </c>
-      <c r="Q28" s="14" t="n">
         <v>-2.3</v>
       </c>
-      <c r="S28" s="14" t="n">
+      <c r="R28" s="14" t="n">
         <v>5.31</v>
       </c>
     </row>
@@ -1910,56 +1825,53 @@
       <c r="A29" s="14" t="n">
         <v>27</v>
       </c>
-      <c r="B29" s="14" t="n">
-        <v>29</v>
-      </c>
-      <c r="C29" s="14" t="inlineStr">
+      <c r="B29" s="14" t="inlineStr">
         <is>
           <t>[Ir(pmb)3]</t>
         </is>
       </c>
-      <c r="E29" s="14" t="n">
+      <c r="D29" s="14" t="n">
         <v>77.7</v>
       </c>
+      <c r="F29" s="14" t="n">
+        <v>17.43</v>
+      </c>
       <c r="G29" s="14" t="n">
-        <v>17.43</v>
+        <v>12.77</v>
       </c>
       <c r="H29" s="14" t="n">
-        <v>12.77</v>
+        <v>2.97</v>
       </c>
       <c r="I29" s="14" t="n">
-        <v>2.97</v>
+        <v>2.02</v>
       </c>
       <c r="J29" s="14" t="n">
-        <v>2.02</v>
+        <v>5.18</v>
       </c>
       <c r="K29" s="14" t="n">
-        <v>5.18</v>
-      </c>
-      <c r="L29" s="14" t="n">
         <v>4.42</v>
       </c>
+      <c r="M29" s="14" t="n">
+        <v>49.56</v>
+      </c>
       <c r="N29" s="14" t="n">
-        <v>49.56</v>
+        <v>-110.8</v>
       </c>
       <c r="O29" s="14" t="n">
-        <v>-110.8</v>
+        <v>0.38</v>
       </c>
       <c r="P29" s="14" t="n">
-        <v>0.38</v>
-      </c>
-      <c r="Q29" s="14" t="n">
         <v>-2.27</v>
       </c>
-      <c r="S29" s="14" t="n">
+      <c r="R29" s="14" t="n">
         <v>5.17</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="G1:L1"/>
-    <mergeCell ref="N1:Q1"/>
+    <mergeCell ref="F1:K1"/>
+    <mergeCell ref="M1:P1"/>
+    <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2022,12 +1934,12 @@
       <c r="C2" s="16" t="inlineStr"/>
       <c r="D2" s="17" t="inlineStr">
         <is>
-          <t>PC number used downstream and in the paper, 1-27.</t>
+          <t>PC number, 1-27.</t>
         </is>
       </c>
       <c r="E2" s="16" t="inlineStr">
         <is>
-          <t>compound_identification.xlsx: Photocatalysts/new_id</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: pc_new_id</t>
         </is>
       </c>
     </row>
@@ -2039,53 +1951,57 @@
       </c>
       <c r="B3" s="16" t="inlineStr">
         <is>
-          <t>old_id</t>
+          <t>compound</t>
         </is>
       </c>
       <c r="C3" s="16" t="inlineStr"/>
       <c r="D3" s="17" t="inlineStr">
         <is>
-          <t>PC number during the screen, used by the raw files.</t>
+          <t>Compound.</t>
         </is>
       </c>
       <c r="E3" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: pc_id</t>
+          <t>compound_identification.xlsx: Photocatalysts/name</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="16" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Triplet energy / kcal mol-1</t>
         </is>
       </c>
       <c r="B4" s="16" t="inlineStr">
         <is>
-          <t>compound</t>
-        </is>
-      </c>
-      <c r="C4" s="16" t="inlineStr"/>
+          <t>E_T / kcal mol-1</t>
+        </is>
+      </c>
+      <c r="C4" s="16" t="inlineStr">
+        <is>
+          <t>kcal mol-1</t>
+        </is>
+      </c>
       <c r="D4" s="17" t="inlineStr">
         <is>
-          <t>Compound.</t>
+          <t>Adiabatic, Gibbs-corrected: ((E_T1 + G_T1) - (E_S0 + G_S0)) x 627.509.</t>
         </is>
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
-          <t>compound_identification.xlsx: Photocatalysts/name</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: E_T / kcal mol-1</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="16" t="inlineStr">
         <is>
-          <t>Triplet energy / kcal mol-1</t>
+          <t>Reorganization energies / kcal mol-1</t>
         </is>
       </c>
       <c r="B5" s="16" t="inlineStr">
         <is>
-          <t>E_T / kcal mol-1</t>
+          <t>lambda_S0_T1 / kcal mol-1</t>
         </is>
       </c>
       <c r="C5" s="16" t="inlineStr">
@@ -2095,12 +2011,12 @@
       </c>
       <c r="D5" s="17" t="inlineStr">
         <is>
-          <t>Adiabatic, Gibbs-corrected: ((E_T1 + G_T1) - (E_S0 + G_S0)) x 627.509.</t>
+          <t>S0 surface: E_S0 at the T1 geometry minus E_S0 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: E_T / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: lambda_S0_T1 / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2112,7 +2028,7 @@
       </c>
       <c r="B6" s="16" t="inlineStr">
         <is>
-          <t>lambda_S0_T1 / kcal mol-1</t>
+          <t>lambda_T1_S0 / kcal mol-1</t>
         </is>
       </c>
       <c r="C6" s="16" t="inlineStr">
@@ -2122,12 +2038,12 @@
       </c>
       <c r="D6" s="17" t="inlineStr">
         <is>
-          <t>S0 surface: E_S0 at the T1 geometry minus E_S0 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
+          <t>T1 surface: E_T1 at the S0 geometry minus E_T1 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_S0_T1 / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: lambda_T1_S0 / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2055,7 @@
       </c>
       <c r="B7" s="16" t="inlineStr">
         <is>
-          <t>lambda_T1_S0 / kcal mol-1</t>
+          <t>lambda_S0_Dplus / kcal mol-1</t>
         </is>
       </c>
       <c r="C7" s="16" t="inlineStr">
@@ -2149,12 +2065,12 @@
       </c>
       <c r="D7" s="17" t="inlineStr">
         <is>
-          <t>T1 surface: E_T1 at the S0 geometry minus E_T1 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
+          <t>S0 surface: E_S0 at the Dplus geometry minus E_S0 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_T1_S0 / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: lambda_S0_Dplus / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2166,7 +2082,7 @@
       </c>
       <c r="B8" s="16" t="inlineStr">
         <is>
-          <t>lambda_S0_Dplus / kcal mol-1</t>
+          <t>lambda_Dplus_S0 / kcal mol-1</t>
         </is>
       </c>
       <c r="C8" s="16" t="inlineStr">
@@ -2176,12 +2092,12 @@
       </c>
       <c r="D8" s="17" t="inlineStr">
         <is>
-          <t>S0 surface: E_S0 at the Dplus geometry minus E_S0 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
+          <t>Dplus surface: E_Dplus at the S0 geometry minus E_Dplus at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_S0_Dplus / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: lambda_Dplus_S0 / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2193,7 +2109,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>lambda_Dplus_S0 / kcal mol-1</t>
+          <t>lambda_S0_Dminus / kcal mol-1</t>
         </is>
       </c>
       <c r="C9" s="16" t="inlineStr">
@@ -2203,12 +2119,12 @@
       </c>
       <c r="D9" s="17" t="inlineStr">
         <is>
-          <t>Dplus surface: E_Dplus at the S0 geometry minus E_Dplus at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
+          <t>S0 surface: E_S0 at the Dminus geometry minus E_S0 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_Dplus_S0 / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: lambda_S0_Dminus / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2220,7 +2136,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>lambda_S0_Dminus / kcal mol-1</t>
+          <t>lambda_Dminus_S0 / kcal mol-1</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
@@ -2230,24 +2146,24 @@
       </c>
       <c r="D10" s="17" t="inlineStr">
         <is>
-          <t>S0 surface: E_S0 at the Dminus geometry minus E_S0 at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
+          <t>Dminus surface: E_Dminus at the S0 geometry minus E_Dminus at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_S0_Dminus / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: lambda_Dminus_S0 / kcal mol-1</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="16" t="inlineStr">
         <is>
-          <t>Reorganization energies / kcal mol-1</t>
+          <t>Excited-state redox / kcal mol-1 and V vs SCE</t>
         </is>
       </c>
       <c r="B11" s="16" t="inlineStr">
         <is>
-          <t>lambda_Dminus_S0 / kcal mol-1</t>
+          <t>dG_ox_ES / kcal mol-1</t>
         </is>
       </c>
       <c r="C11" s="16" t="inlineStr">
@@ -2257,12 +2173,12 @@
       </c>
       <c r="D11" s="17" t="inlineStr">
         <is>
-          <t>Dminus surface: E_Dminus at the S0 geometry minus E_Dminus at its own, electronic energies x 627.509. Dplus and Dminus are the one-electron oxidized and reduced states.</t>
+          <t>PC* -&gt; PC+: ((E_ox + G_ox) - (E_T1 + G_T1)) x 627.509.</t>
         </is>
       </c>
       <c r="E11" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: lambda_Dminus_S0 / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: dG_ox_ES / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2274,7 +2190,7 @@
       </c>
       <c r="B12" s="16" t="inlineStr">
         <is>
-          <t>dG_ox_ES / kcal mol-1</t>
+          <t>dG_red_ES / kcal mol-1</t>
         </is>
       </c>
       <c r="C12" s="16" t="inlineStr">
@@ -2284,12 +2200,12 @@
       </c>
       <c r="D12" s="17" t="inlineStr">
         <is>
-          <t>PC* -&gt; PC+: ((E_ox + G_ox) - (E_T1 + G_T1)) x 627.509.</t>
+          <t>PC* -&gt; PC-: ((E_red + G_red) - (E_T1 + G_T1)) x 627.509.</t>
         </is>
       </c>
       <c r="E12" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: dG_ox_ES / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: dG_red_ES / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2301,22 +2217,22 @@
       </c>
       <c r="B13" s="16" t="inlineStr">
         <is>
-          <t>dG_red_ES / kcal mol-1</t>
+          <t>E_PCstar_PCminus / V</t>
         </is>
       </c>
       <c r="C13" s="16" t="inlineStr">
         <is>
-          <t>kcal mol-1</t>
+          <t>V</t>
         </is>
       </c>
       <c r="D13" s="17" t="inlineStr">
         <is>
-          <t>PC* -&gt; PC-: ((E_red + G_red) - (E_T1 + G_T1)) x 627.509.</t>
+          <t>PC*/PC-, how strong an oxidant the triplet is: -dG_red_ES / 23.061 - 4.42.</t>
         </is>
       </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: dG_red_ES / kcal mol-1</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: E_PCstar_PCminus / V</t>
         </is>
       </c>
     </row>
@@ -2328,7 +2244,7 @@
       </c>
       <c r="B14" s="16" t="inlineStr">
         <is>
-          <t>E_PCstar_PCminus / V</t>
+          <t>E_PCplus_PCstar / V</t>
         </is>
       </c>
       <c r="C14" s="16" t="inlineStr">
@@ -2338,71 +2254,55 @@
       </c>
       <c r="D14" s="17" t="inlineStr">
         <is>
-          <t>PC*/PC-, how strong an oxidant the triplet is: -dG_red_ES / 23.061 - 4.42.</t>
+          <t>PC+/PC*, how strong a reductant the triplet is: dG_ox_ES / 23.061 - 4.42.</t>
         </is>
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: E_PCstar_PCminus / V</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: E_PCplus_PCstar / V</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="16" t="inlineStr">
         <is>
-          <t>Excited-state redox / kcal mol-1 and V vs SCE</t>
+          <t>Molecular size / A</t>
         </is>
       </c>
       <c r="B15" s="16" t="inlineStr">
         <is>
-          <t>E_PCplus_PCstar / V</t>
+          <t>radius_S0 / A</t>
         </is>
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>V</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D15" s="17" t="inlineStr">
         <is>
-          <t>PC+/PC*, how strong a reductant the triplet is: dG_ox_ES / 23.061 - 4.42.</t>
+          <t>Radius of the sphere with the van der Waals volume of the optimised S0 geometry: union of atomic spheres with Bondi radii (Ir and Ru 2.00 A), counted on a 0.1 A grid. r_PC + r_Q is the contact distance of a pair in the benchmark.</t>
         </is>
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: E_PCplus_PCstar / V</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: radius_S0 / A</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
-        <is>
-          <t>Molecular size / A</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>radius_S0 / A</t>
-        </is>
-      </c>
-      <c r="C16" s="16" t="inlineStr">
-        <is>
-          <t>A</t>
-        </is>
-      </c>
-      <c r="D16" s="17" t="inlineStr">
-        <is>
-          <t>Radius of the sphere with the van der Waals volume of the optimised S0 geometry: union of atomic spheres with Bondi radii (Ir and Ru 2.00 A), counted on a 0.1 A grid. r_PC + r_Q is the contact distance of a pair in the benchmark.</t>
-        </is>
-      </c>
-      <c r="E16" s="16" t="inlineStr">
-        <is>
-          <t>computational_data_raw/photocatalysts/photocatalyst_dft.csv: radius_S0 / A</t>
-        </is>
-      </c>
+      <c r="A16" s="16" t="n"/>
+      <c r="B16" s="16" t="n"/>
+      <c r="C16" s="16" t="n"/>
+      <c r="D16" s="17" t="n"/>
+      <c r="E16" s="16" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="n"/>
+      <c r="A17" s="16" t="inlineStr">
+        <is>
+          <t>One row per photocatalyst in the screen, sorted by new_id.</t>
+        </is>
+      </c>
       <c r="B17" s="16" t="n"/>
       <c r="C17" s="16" t="n"/>
       <c r="D17" s="17" t="n"/>
@@ -2411,7 +2311,7 @@
     <row r="18">
       <c r="A18" s="16" t="inlineStr">
         <is>
-          <t>One row per photocatalyst in the screen, sorted by new_id; the raw files use old_id.</t>
+          <t>Every value is computed from the ORCA outputs. Total energies, Gibbs corrections and</t>
         </is>
       </c>
       <c r="B18" s="16" t="n"/>
@@ -2422,7 +2322,7 @@
     <row r="19">
       <c r="A19" s="16" t="inlineStr">
         <is>
-          <t>Every value is computed from the ORCA outputs. Total energies, Gibbs corrections and</t>
+          <t>frequency checks are in</t>
         </is>
       </c>
       <c r="B19" s="16" t="n"/>
@@ -2433,7 +2333,7 @@
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>frequency checks are in computational_data_raw/photocatalysts/photocatalyst_dft.csv.</t>
+          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv.</t>
         </is>
       </c>
       <c r="B20" s="16" t="n"/>

</xml_diff>

<commit_message>
Move the extracted and hand-entered tables into the processed folders
The tables the extraction scripts write, and the hand-entered redox tables, move from the
raw folders to data/experimental_data_processed/ and data/computational_data_processed/.
Writers, readers, reproduce.py inputs, the workbook column keys and the READMEs follow.
</commit_message>
<xml_diff>
--- a/data/computational_data_processed/photocatalyst_properties_calc.xlsx
+++ b/data/computational_data_processed/photocatalyst_properties_calc.xlsx
@@ -1939,7 +1939,7 @@
       </c>
       <c r="E2" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: pc_new_id</t>
+          <t>computational_data_processed/photocatalyst_dft.csv: pc_new_id</t>
         </is>
       </c>
     </row>
@@ -1989,7 +1989,7 @@
       </c>
       <c r="E4" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: E_T / kcal mol-1</t>
+          <t>computational_data_processed/photocatalyst_dft.csv: E_T / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: lambda_S0_T1 / kcal mol-1</t>
+          <t>computational_data_processed/photocatalyst_dft.csv: lambda_S0_T1 / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2043,7 +2043,7 @@
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: lambda_T1_S0 / kcal mol-1</t>
+          <t>computational_data_processed/photocatalyst_dft.csv: lambda_T1_S0 / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2070,7 +2070,7 @@
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: lambda_S0_Dplus / kcal mol-1</t>
+          <t>computational_data_processed/photocatalyst_dft.csv: lambda_S0_Dplus / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2097,7 +2097,7 @@
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: lambda_Dplus_S0 / kcal mol-1</t>
+          <t>computational_data_processed/photocatalyst_dft.csv: lambda_Dplus_S0 / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2124,7 +2124,7 @@
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: lambda_S0_Dminus / kcal mol-1</t>
+          <t>computational_data_processed/photocatalyst_dft.csv: lambda_S0_Dminus / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: lambda_Dminus_S0 / kcal mol-1</t>
+          <t>computational_data_processed/photocatalyst_dft.csv: lambda_Dminus_S0 / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2178,7 +2178,7 @@
       </c>
       <c r="E11" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: dG_ox_ES / kcal mol-1</t>
+          <t>computational_data_processed/photocatalyst_dft.csv: dG_ox_ES / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2205,7 +2205,7 @@
       </c>
       <c r="E12" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: dG_red_ES / kcal mol-1</t>
+          <t>computational_data_processed/photocatalyst_dft.csv: dG_red_ES / kcal mol-1</t>
         </is>
       </c>
     </row>
@@ -2232,7 +2232,7 @@
       </c>
       <c r="E13" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: E_PCstar_PCminus / V</t>
+          <t>computational_data_processed/photocatalyst_dft.csv: E_PCstar_PCminus / V</t>
         </is>
       </c>
     </row>
@@ -2259,7 +2259,7 @@
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: E_PCplus_PCstar / V</t>
+          <t>computational_data_processed/photocatalyst_dft.csv: E_PCplus_PCstar / V</t>
         </is>
       </c>
     </row>
@@ -2286,7 +2286,7 @@
       </c>
       <c r="E15" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv: radius_S0 / A</t>
+          <t>computational_data_processed/photocatalyst_dft.csv: radius_S0 / A</t>
         </is>
       </c>
     </row>
@@ -2333,7 +2333,7 @@
     <row r="20">
       <c r="A20" s="16" t="inlineStr">
         <is>
-          <t>computational_data_raw/photocatalysts_new_ids/photocatalyst_dft.csv.</t>
+          <t>computational_data_processed/photocatalyst_dft.csv.</t>
         </is>
       </c>
       <c r="B20" s="16" t="n"/>

</xml_diff>